<commit_message>
Adiciona Elas Jogam Summit e WIFS
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R159269007bd44164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R28e462a28ad94f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Re5ae98ba442a4de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R82bdb4eb256244dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Re416c13d26714670"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R852b9c000cbb40d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rad5aa9665b274197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R2cac4f2ca385476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R204033f7c31245ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rf5500965605c478d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R88def3617b9549c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R91e5071af8fa4b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R64aa04f78f9b4d28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R4dbc69f6f24e4f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R42c17e83c6c046f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R3cec115a5b294c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R81348a501df245d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R42aa7e0119964e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rb0967acbdad647ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rc6b3b4308e8646b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rfd31b2ecd18f49c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rc5c5d797671f4d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R0af5086ef5e54738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R3b172669f308408e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rc873556d045447b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rf8d40107423f489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Ra365d65daa5443b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R333aa679afda46cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Ra3f4a8eb23e842d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R1f4d34f2eaa94de6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Ra3bc34d5b23845ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rae0f8e19c28a4755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R5e6f430b20bd48ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R74bbbe1da83a4818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rb5d89597555f4487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rc4376f455bc441b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2138,7 +2138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5281fbeb6b9b4c6a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9391fa8ce74c4fe8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2168,7 +2168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fabd1f3a17e4b17"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R475d9e2337d04213"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2198,7 +2198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R816500b6f9204388"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc15ab185c75d40fa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2228,7 +2228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R441bbdfd238148f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dced995b4ad4c8a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2263,7 +2263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb51bc3232f8b458d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4227748c3d4e4dde"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2961,7 +2961,7 @@
       </x:c>
       <x:c r="B17" s="2" t="n">
         <x:f>COUNTIF('02_Eventos'!B2:B495,"Confirmado")</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="2" t="s">
@@ -3874,7 +3874,7 @@
     <x:mergeCell ref="D5:F7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3356364de0442da"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f6e3317a1b34646"/>
 </x:worksheet>
 </file>
 
@@ -6101,7 +6101,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7caa752a60da4f97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96fdda61605e4301"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8341,7 +8341,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae38f2fcf2184d8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree30292abefb4dc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8939,7 +8939,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf73a5c0ecff4393"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe75dceacb2543d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13089,9 +13089,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fa43d691c3a444c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b0a9b2769ed4d51"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R051118f7427047dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc23731bdb6e84368"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13282,7 +13282,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7065938dbf3e4966"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9ed01857dce4f0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14847,40 +14847,100 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="5"/>
-      <x:c r="B17" s="5"/>
-      <x:c r="C17" s="6"/>
-      <x:c r="D17" s="5"/>
-      <x:c r="E17" s="5"/>
-      <x:c r="F17" s="5"/>
-      <x:c r="G17" s="5"/>
-      <x:c r="H17" s="7"/>
+      <x:c r="A17" s="5" t="str">
+        <x:v>EVT-0021</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="str">
+        <x:v>Confirmado</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="D17" s="5" t="str">
+        <x:v>SP</x:v>
+      </x:c>
+      <x:c r="E17" s="5" t="str">
+        <x:v>São Paulo</x:v>
+      </x:c>
+      <x:c r="F17" s="5" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G17" s="5" t="str">
+        <x:v>Instituto Futuro em Jogo</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I17" s="5"/>
-      <x:c r="J17" s="5"/>
-      <x:c r="K17" s="8"/>
-      <x:c r="L17" s="8"/>
-      <x:c r="M17" s="5"/>
-      <x:c r="N17" s="5"/>
-      <x:c r="O17" s="5"/>
-      <x:c r="P17" s="5"/>
+      <x:c r="J17" s="5" t="str">
+        <x:v>Museu do Futebol</x:v>
+      </x:c>
+      <x:c r="K17" s="8" t="n">
+        <x:v>-23.5477</x:v>
+      </x:c>
+      <x:c r="L17" s="8" t="n">
+        <x:v>-46.6657</x:v>
+      </x:c>
+      <x:c r="M17" s="5" t="str">
+        <x:v>https://www.sympla.com.br/evento/elas-jogam-summit-sao-paulo-e-o-legado-da-copa-de-2027-23-08-domingo/3508796</x:v>
+      </x:c>
+      <x:c r="N17" s="5" t="str">
+        <x:v>Elas Jogam Summit — São Paulo e o Legado da Copa 2027. Evento presencial em 23/08/2026, das 8h30 às 19h, no Museu do Futebol.</x:v>
+      </x:c>
+      <x:c r="O17" s="5" t="str">
+        <x:v>Ago</x:v>
+      </x:c>
+      <x:c r="P17" s="5" t="n">
+        <x:v>2026</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="5"/>
-      <x:c r="B18" s="5"/>
-      <x:c r="C18" s="6"/>
-      <x:c r="D18" s="5"/>
-      <x:c r="E18" s="5"/>
-      <x:c r="F18" s="5"/>
-      <x:c r="G18" s="5"/>
-      <x:c r="H18" s="7"/>
+      <x:c r="A18" s="5" t="str">
+        <x:v>EVT-0022</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>Confirmado</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="str">
+        <x:v>RJ</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="str">
+        <x:v>Rio de Janeiro</x:v>
+      </x:c>
+      <x:c r="F18" s="5" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="str">
+        <x:v>CONFUT / WIFS</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I18" s="5"/>
-      <x:c r="J18" s="5"/>
-      <x:c r="K18" s="8"/>
-      <x:c r="L18" s="8"/>
-      <x:c r="M18" s="5"/>
-      <x:c r="N18" s="5"/>
-      <x:c r="O18" s="5"/>
-      <x:c r="P18" s="5"/>
+      <x:c r="J18" s="5" t="str">
+        <x:v>Museu do Amanhã</x:v>
+      </x:c>
+      <x:c r="K18" s="8" t="n">
+        <x:v>-22.8942</x:v>
+      </x:c>
+      <x:c r="L18" s="8" t="n">
+        <x:v>-43.1794</x:v>
+      </x:c>
+      <x:c r="M18" s="5" t="str">
+        <x:v>https://womanifs.com/</x:v>
+      </x:c>
+      <x:c r="N18" s="5" t="str">
+        <x:v>Women's International Football Summit (WIFS), encontro internacional dedicado ao futebol feminino, em 14 e 15/09/2026 no Museu do Amanhã.</x:v>
+      </x:c>
+      <x:c r="O18" s="5" t="str">
+        <x:v>Set</x:v>
+      </x:c>
+      <x:c r="P18" s="5" t="n">
+        <x:v>2026</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5"/>
@@ -23577,7 +23637,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d9c72f7c6e84200"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6054aa2f02f647e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23617,7 +23677,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str" cm="1">
-        <x:f t="array" ref="A2:A12" ca="1">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
+        <x:f t="array" ref="A2:A14" ca="1">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
         <x:v>EVT-0006</x:v>
       </x:c>
       <x:c r="B2" s="6">
@@ -23902,7 +23962,9 @@
       <x:c r="H12" s="5"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="5"/>
+      <x:c r="A13" s="5" t="str">
+        <x:v>EVT-0021</x:v>
+      </x:c>
       <x:c r="B13" s="6"/>
       <x:c r="C13" s="5"/>
       <x:c r="D13" s="5"/>
@@ -23912,7 +23974,9 @@
       <x:c r="H13" s="5"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="5"/>
+      <x:c r="A14" s="5" t="str">
+        <x:v>EVT-0022</x:v>
+      </x:c>
       <x:c r="B14" s="6"/>
       <x:c r="C14" s="5"/>
       <x:c r="D14" s="5"/>
@@ -24271,7 +24335,7 @@
       </x:c>
       <x:c r="C2" s="13" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A2)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D2" s="13" t="n">
         <x:f>SUMIF('02_Eventos'!E:E,A2,'02_Eventos'!H:H)</x:f>
@@ -24296,7 +24360,7 @@
       </x:c>
       <x:c r="J2" s="13" t="n">
         <x:f t="shared" ref="J2:J9" si="0">MIN(100,(C2*5)+(MIN(D2/1000,20))+(E2*4)+(F2*3)+(G2*0.1)+(H2*0.1)+(I2*0.1))</x:f>
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K2" s="5" t="str">
         <x:f t="shared" ref="K2:K9" si="1">IF(J2&gt;=85,"Excelente",IF(J2&gt;=70,"Alta",IF(J2&gt;=50,"Moderada",IF(J2&gt;=30,"Baixa","Muito baixa"))))</x:f>
@@ -24312,7 +24376,7 @@
       </x:c>
       <x:c r="C3" s="13" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A3)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D3" s="13" t="n">
         <x:f>SUMIF('02_Eventos'!E:E,A3,'02_Eventos'!H:H)</x:f>
@@ -25536,7 +25600,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07b7e171c63e46be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb472b3239e3a4126"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25894,7 +25958,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7821b3ac882745fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc55b17861d21400b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31564,7 +31628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6bff7ef71034b9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf880a8e4ecc9432f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31625,7 +31689,7 @@
       </x:c>
       <x:c r="G2" s="5" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A2)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H2" s="5" t="n">
         <x:f>SUMIF('02_Eventos'!E:E,A2,'02_Eventos'!H:H)</x:f>
@@ -31655,7 +31719,7 @@
       </x:c>
       <x:c r="G3" s="5" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A3)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H3" s="5" t="n">
         <x:f>SUMIF('02_Eventos'!E:E,A3,'02_Eventos'!H:H)</x:f>
@@ -32419,7 +32483,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7a38b7f6c134b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06f19dab258e4251"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33252,7 +33316,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0fb42fab373469e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2a058e369240f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33325,7 +33389,7 @@
       </x:c>
       <x:c r="I2" s="5" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A2)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J2" s="5"/>
     </x:row>
@@ -33358,7 +33422,7 @@
       </x:c>
       <x:c r="I3" s="5" t="n">
         <x:f>COUNTIF('02_Eventos'!E:E,A3)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J3" s="5"/>
     </x:row>
@@ -33575,7 +33639,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6c599b876f7461f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda96f52ec1c240fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Amplia cobertura das Seleções Femininas de Base
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rdfbeea171d0b47f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R84d1607cbd7040e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R7435b56e3f7447c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R6f08503667354cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rb568b056e4a54791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R4e2bb888a4294719"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rbf1f0896d2984431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Ra953369f0a0c421c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R9bfd6fa24e2f4338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rd7d249ac76204930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R51f4c8f9212e4dc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rff6871ecfcef4006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rf5a945bf03a34b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R071000f1b00f4526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R89762c74128b48fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R0bc81299fbcb4a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rcf40ca356a8d4f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R7c720eef2f3048a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Re4a8e6b82bf34087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R6678d1c686ea492b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rfadcbdfe2ee94ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R386015c0557c470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R5217fb5b2484406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R8743fa7bfeb548cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Raf2f6cd441b14f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R4293f74300f34cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R416616569c354c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R7ee01149339b4c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rfa1d57aac00c4812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rd6b60d2127c24c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R44b57440da144cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R00bf4bdc92ff43ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Ra84e7c4eace94d93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R52ece500c8874125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R538d36ba235e4dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rffc43e39042748fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1913,7 +1913,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac4540fd459d402a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c0fa3564c544efd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1943,7 +1943,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa51f57aef664f99"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R429cc9a6e756448a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1973,7 +1973,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R653aad4f572a4172"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R034d1253fd174832"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2003,7 +2003,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8cc8e09a81c94676"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R617e8ee1cbc84c60"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2038,7 +2038,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R47678e4b3b5b4ce9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1263772c20b24999"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2487,13 +2487,13 @@
     <x:row r="5">
       <x:c r="A5" s="22" t="str">
         <x:v>TOTAL DE EVENTOS
-77</x:v>
+84</x:v>
       </x:c>
       <x:c r="B5" s="21"/>
       <x:c r="C5" s="21"/>
       <x:c r="D5" s="22" t="str">
         <x:v>EVENTOS FUTUROS
-19</x:v>
+25</x:v>
       </x:c>
       <x:c r="E5" s="21"/>
       <x:c r="F5" s="21"/>
@@ -2563,7 +2563,7 @@
     <x:row r="9">
       <x:c r="A9" s="22" t="str">
         <x:v>CIDADES MONITORADAS
-13</x:v>
+15</x:v>
       </x:c>
       <x:c r="B9" s="21"/>
       <x:c r="C9" s="21"/>
@@ -2705,7 +2705,7 @@
       </x:c>
       <x:c r="B16" s="2" t="n">
         <x:f>COUNTIF('02_Eventos'!B2:B495,"Planejado")</x:f>
-        <x:v>19</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="2" t="s">
@@ -3654,7 +3654,7 @@
     <x:mergeCell ref="D5:F7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08991600f45746cc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cbed872552e44e2"/>
 </x:worksheet>
 </file>
 
@@ -5881,7 +5881,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra894be8e951b4e19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94e169cd96bd41c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8121,7 +8121,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6450ac56a1b641b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e9695fbbe194203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8719,7 +8719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccc1475c255341eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd2acd60e73a45b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12869,9 +12869,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R631e7c5eb05a4af6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R315aa27ecb37432e"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra22a7e10b66b4074"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re442a30852c548f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13062,7 +13062,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R286fe002c60a40fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra11175bafc4f489c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16656,44 +16656,40 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="str">
-        <x:v>EVT-0022</x:v>
+        <x:v>EVT-0083</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C63" s="27" t="n">
-        <x:v>46279.5</x:v>
+        <x:v>46273.5</x:v>
       </x:c>
       <x:c r="D63" s="5" t="str">
-        <x:v>RJ</x:v>
+        <x:v>PRY</x:v>
       </x:c>
       <x:c r="E63" s="5" t="str">
-        <x:v>Rio de Janeiro</x:v>
+        <x:v>Assunção</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
-        <x:v>Summit</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G63" s="5" t="str">
-        <x:v>CONFUT / WIFS</x:v>
+        <x:v>CONMEBOL / CBF / Seleção Brasileira Feminina Sub-15</x:v>
       </x:c>
       <x:c r="H63" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I63" s="5" t="str"/>
       <x:c r="J63" s="5" t="str">
-        <x:v>Museu do Amanhã</x:v>
-      </x:c>
-      <x:c r="K63" s="8" t="n">
-        <x:v>-22.8942</x:v>
-      </x:c>
-      <x:c r="L63" s="8" t="n">
-        <x:v>-43.1794</x:v>
-      </x:c>
+        <x:v>Local a definir</x:v>
+      </x:c>
+      <x:c r="K63" s="8"/>
+      <x:c r="L63" s="8"/>
       <x:c r="M63" s="5" t="str">
-        <x:v>https://womanifs.com/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="N63" s="5" t="str">
-        <x:v>Women's International Football Summit (WIFS), encontro internacional dedicado ao futebol feminino, em 14 e 15/09/2026 no Museu do Amanhã.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-15 busca o bicampeonato da CONMEBOL Liga Evolução, disputada de 08 a 20/09/2026 no Paraguai. A fonte confirma Assunção como cidade de referência, mas não informa o local físico dos jogos.</x:v>
       </x:c>
       <x:c r="O63" s="5" t="str">
         <x:v>Set</x:v>
@@ -16704,13 +16700,13 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="5" t="str">
-        <x:v>EVT-0062</x:v>
+        <x:v>EVT-0022</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C64" s="27" t="n">
-        <x:v>46284.5</x:v>
+        <x:v>46279.5</x:v>
       </x:c>
       <x:c r="D64" s="5" t="str">
         <x:v>RJ</x:v>
@@ -16719,25 +16715,29 @@
         <x:v>Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
-        <x:v>Tour histórico-cultural</x:v>
+        <x:v>Summit</x:v>
       </x:c>
       <x:c r="G64" s="5" t="str">
-        <x:v>Tour Delas</x:v>
+        <x:v>CONFUT / WIFS</x:v>
       </x:c>
       <x:c r="H64" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I64" s="5" t="str"/>
       <x:c r="J64" s="5" t="str">
-        <x:v>Praça Tiradentes — ponto de encontro em frente ao VLT</x:v>
-      </x:c>
-      <x:c r="K64" s="8"/>
-      <x:c r="L64" s="8"/>
+        <x:v>Museu do Amanhã</x:v>
+      </x:c>
+      <x:c r="K64" s="8" t="n">
+        <x:v>-22.8942</x:v>
+      </x:c>
+      <x:c r="L64" s="8" t="n">
+        <x:v>-43.1794</x:v>
+      </x:c>
       <x:c r="M64" s="5" t="str">
-        <x:v>https://www.sympla.com.br/evento/historia-do-futebol-feminino-no-rio/3546698</x:v>
+        <x:v>https://womanifs.com/</x:v>
       </x:c>
       <x:c r="N64" s="5" t="str">
-        <x:v>Walking tour previsto para 19/09/2026, das 10h às 13h, pelo centro do Rio. O roteiro resgata a história do futebol feminino no Brasil, incluindo a proibição da modalidade, as pioneiras, a força dos coletivos de torcedoras e a Copa do Mundo Feminina 2027 como marco de um século de resistência. A realização depende de um mínimo de cinco participantes.</x:v>
+        <x:v>Women's International Football Summit (WIFS), encontro internacional dedicado ao futebol feminino, em 14 e 15/09/2026 no Museu do Amanhã.</x:v>
       </x:c>
       <x:c r="O64" s="5" t="str">
         <x:v>Set</x:v>
@@ -16748,43 +16748,43 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="5" t="str">
-        <x:v>EVT-0074</x:v>
+        <x:v>EVT-0062</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C65" s="27" t="n">
-        <x:v>46298.5</x:v>
+        <x:v>46284.5</x:v>
       </x:c>
       <x:c r="D65" s="5" t="str">
-        <x:v>SP</x:v>
+        <x:v>RJ</x:v>
       </x:c>
       <x:c r="E65" s="5" t="str">
-        <x:v>São Paulo</x:v>
+        <x:v>Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F65" s="5" t="str">
-        <x:v>Palestra</x:v>
+        <x:v>Tour histórico-cultural</x:v>
       </x:c>
       <x:c r="G65" s="5" t="str">
-        <x:v>COB Expo</x:v>
+        <x:v>Tour Delas</x:v>
       </x:c>
       <x:c r="H65" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I65" s="5" t="str"/>
       <x:c r="J65" s="5" t="str">
-        <x:v>Pro Magno Centro de Eventos</x:v>
+        <x:v>Praça Tiradentes — ponto de encontro em frente ao VLT</x:v>
       </x:c>
       <x:c r="K65" s="8"/>
       <x:c r="L65" s="8"/>
       <x:c r="M65" s="5" t="str">
-        <x:v>https://cobexpo.soudaliga.com.br/reserva?date=2026-10-03&amp;id=22500&amp;nextInternalLocale=pt-BR</x:v>
+        <x:v>https://www.sympla.com.br/evento/historia-do-futebol-feminino-no-rio/3546698</x:v>
       </x:c>
       <x:c r="N65" s="5" t="str">
-        <x:v>Sessão “Copa do Mundo Feminina FIFA 2027 no Brasil: mídia, visibilidade e construção de legado”, em 03/10/2026, das 9h30 às 11h30, durante a COB Expo 2026.</x:v>
+        <x:v>Walking tour previsto para 19/09/2026, das 10h às 13h, pelo centro do Rio. O roteiro resgata a história do futebol feminino no Brasil, incluindo a proibição da modalidade, as pioneiras, a força dos coletivos de torcedoras e a Copa do Mundo Feminina 2027 como marco de um século de resistência. A realização depende de um mínimo de cinco participantes.</x:v>
       </x:c>
       <x:c r="O65" s="5" t="str">
-        <x:v>Out</x:v>
+        <x:v>Set</x:v>
       </x:c>
       <x:c r="P65" s="5" t="n">
         <x:v>2026</x:v>
@@ -16792,43 +16792,43 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="5" t="str">
-        <x:v>EVT-0006</x:v>
+        <x:v>EVT-0084</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C66" s="27" t="n">
-        <x:v>46300.5</x:v>
+        <x:v>46287.5</x:v>
       </x:c>
       <x:c r="D66" s="5" t="str">
-        <x:v>BR</x:v>
+        <x:v>RJ</x:v>
       </x:c>
       <x:c r="E66" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Teresópolis</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str">
-        <x:v>Amistosos da Seleção</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G66" s="5" t="str">
-        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina Sub-17</x:v>
       </x:c>
       <x:c r="H66" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I66" s="5" t="str"/>
       <x:c r="J66" s="5" t="str">
-        <x:v>A definir</x:v>
+        <x:v>Granja Comary</x:v>
       </x:c>
       <x:c r="K66" s="8"/>
       <x:c r="L66" s="8"/>
       <x:c r="M66" s="5" t="str">
-        <x:v>Informado pelo usuário</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N66" s="5" t="str">
-        <x:v>Janela reservada de 05 a 13/10/2026 para realização de até 2 jogos amistosos.</x:v>
+        <x:v>Período de treinamento da Seleção Brasileira Feminina Sub-17 entre 22/09 e 16/10/2026, na Granja Comary, como preparação final para a Copa do Mundo da categoria no Marrocos.</x:v>
       </x:c>
       <x:c r="O66" s="5" t="str">
-        <x:v>Out</x:v>
+        <x:v>Set</x:v>
       </x:c>
       <x:c r="P66" s="5" t="n">
         <x:v>2026</x:v>
@@ -16836,13 +16836,13 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="5" t="str">
-        <x:v>EVT-0055</x:v>
+        <x:v>EVT-0074</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C67" s="27" t="n">
-        <x:v>46341.5</x:v>
+        <x:v>46298.5</x:v>
       </x:c>
       <x:c r="D67" s="5" t="str">
         <x:v>SP</x:v>
@@ -16851,30 +16851,28 @@
         <x:v>São Paulo</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
-        <x:v>Premiação</x:v>
+        <x:v>Palestra</x:v>
       </x:c>
       <x:c r="G67" s="5" t="str">
-        <x:v>TV Brasil / EBC / Petrobras</x:v>
+        <x:v>COB Expo</x:v>
       </x:c>
       <x:c r="H67" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I67" s="5" t="str">
-        <x:v>Petrobras</x:v>
-      </x:c>
+      <x:c r="I67" s="5" t="str"/>
       <x:c r="J67" s="5" t="str">
-        <x:v>Local a definir</x:v>
+        <x:v>Pro Magno Centro de Eventos</x:v>
       </x:c>
       <x:c r="K67" s="8"/>
       <x:c r="L67" s="8"/>
       <x:c r="M67" s="5" t="str">
-        <x:v>https://www.ebc.com.br/premiotvbrasilpetrobrasparaelas/</x:v>
+        <x:v>https://cobexpo.soudaliga.com.br/reserva?date=2026-10-03&amp;id=22500&amp;nextInternalLocale=pt-BR</x:v>
       </x:c>
       <x:c r="N67" s="5" t="str">
-        <x:v>Primeira edição do Prêmio TV Brasil Petrobras Para Elas, marcada para 15/11/2026, em São Paulo, com transmissão ao vivo pela TV Brasil e YouTube. A premiação reconhece atletas, treinadoras, clubes, departamentos e iniciativas relevantes para o fortalecimento do futebol feminino brasileiro. A fonte oficial confirma cidade e data, mas não informa o local físico.</x:v>
+        <x:v>Sessão “Copa do Mundo Feminina FIFA 2027 no Brasil: mídia, visibilidade e construção de legado”, em 03/10/2026, das 9h30 às 11h30, durante a COB Expo 2026.</x:v>
       </x:c>
       <x:c r="O67" s="5" t="str">
-        <x:v>Nov</x:v>
+        <x:v>Out</x:v>
       </x:c>
       <x:c r="P67" s="5" t="n">
         <x:v>2026</x:v>
@@ -16882,13 +16880,13 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="5" t="str">
-        <x:v>EVT-0007</x:v>
+        <x:v>EVT-0006</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C68" s="27" t="n">
-        <x:v>46350.5</x:v>
+        <x:v>46300.5</x:v>
       </x:c>
       <x:c r="D68" s="5" t="str">
         <x:v>BR</x:v>
@@ -16915,10 +16913,10 @@
         <x:v>Informado pelo usuário</x:v>
       </x:c>
       <x:c r="N68" s="5" t="str">
-        <x:v>Período estendido de 24/11 a 05/12/2026, permitindo até 3 jogos preparatórios.</x:v>
+        <x:v>Janela reservada de 05 a 13/10/2026 para realização de até 2 jogos amistosos.</x:v>
       </x:c>
       <x:c r="O68" s="5" t="str">
-        <x:v>Nov</x:v>
+        <x:v>Out</x:v>
       </x:c>
       <x:c r="P68" s="5" t="n">
         <x:v>2026</x:v>
@@ -16926,43 +16924,43 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="5" t="str">
-        <x:v>EVT-0011</x:v>
+        <x:v>EVT-0085</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C69" s="27" t="n">
-        <x:v>46357.5</x:v>
+        <x:v>46300.5</x:v>
       </x:c>
       <x:c r="D69" s="5" t="str">
         <x:v>BR</x:v>
       </x:c>
       <x:c r="E69" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
-        <x:v>Centro de Treinamento</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G69" s="5" t="str">
-        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina Sub-20</x:v>
       </x:c>
       <x:c r="H69" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I69" s="5" t="str"/>
       <x:c r="J69" s="5" t="str">
-        <x:v>A definir</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="K69" s="8"/>
       <x:c r="L69" s="8"/>
       <x:c r="M69" s="5" t="str">
-        <x:v>Informado pelo usuário</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N69" s="5" t="str">
-        <x:v>Definição do Team Base Camp prevista para dezembro de 2026. Data exata a definir.</x:v>
+        <x:v>Período de treinamentos da Seleção Brasileira Feminina Sub-20 previsto de 05 a 13/10/2026. A CBF não informou cidade nem local físico.</x:v>
       </x:c>
       <x:c r="O69" s="5" t="str">
-        <x:v>Dez</x:v>
+        <x:v>Out</x:v>
       </x:c>
       <x:c r="P69" s="5" t="n">
         <x:v>2026</x:v>
@@ -16970,43 +16968,43 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="5" t="str">
-        <x:v>EVT-0010</x:v>
+        <x:v>EVT-0086</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C70" s="27" t="n">
-        <x:v>46367.5</x:v>
+        <x:v>46312.5</x:v>
       </x:c>
       <x:c r="D70" s="5" t="str">
-        <x:v>RJ</x:v>
+        <x:v>MAR</x:v>
       </x:c>
       <x:c r="E70" s="5" t="str">
-        <x:v>Rio de Janeiro</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="F70" s="5" t="str">
-        <x:v>Sorteio Oficial</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G70" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>FIFA / CBF / Seleção Brasileira Feminina Sub-17</x:v>
       </x:c>
       <x:c r="H70" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I70" s="5" t="str"/>
       <x:c r="J70" s="5" t="str">
-        <x:v>Museu de Arte Moderna do Rio de Janeiro (MAM Rio)</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="K70" s="8"/>
       <x:c r="L70" s="8"/>
       <x:c r="M70" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/sorteio-grupos-copa-mundo-feminina-2027-data-local</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N70" s="5" t="str">
-        <x:v>Sorteio final dos grupos confirmado para 11/12/2026 no MAM Rio. O evento definirá os oito grupos e o caminho das 32 seleções na Copa do Mundo Feminina FIFA 2027.</x:v>
+        <x:v>Copa do Mundo Feminina Sub-17 da FIFA, disputada de 17/10 a 07/11/2026 no Marrocos. O Brasil integra grupo com Canadá, Noruega e uma seleção africana; a fonte consultada não especifica cidade nem estádio.</x:v>
       </x:c>
       <x:c r="O70" s="5" t="str">
-        <x:v>Dez</x:v>
+        <x:v>Out</x:v>
       </x:c>
       <x:c r="P70" s="5" t="n">
         <x:v>2026</x:v>
@@ -17014,101 +17012,103 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="5" t="str">
-        <x:v>EVT-0008</x:v>
+        <x:v>EVT-0087</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C71" s="27" t="n">
-        <x:v>46444.5</x:v>
+        <x:v>46340.5</x:v>
       </x:c>
       <x:c r="D71" s="5" t="str">
         <x:v>BR</x:v>
       </x:c>
       <x:c r="E71" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="F71" s="5" t="str">
-        <x:v>Amistosos da Seleção</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G71" s="5" t="str">
-        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina Sub-15</x:v>
       </x:c>
       <x:c r="H71" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I71" s="5" t="str"/>
       <x:c r="J71" s="5" t="str">
-        <x:v>A definir</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="K71" s="8"/>
       <x:c r="L71" s="8"/>
       <x:c r="M71" s="5" t="str">
-        <x:v>Informado pelo usuário</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N71" s="5" t="str">
-        <x:v>Primeira janela de amistosos de 2027, de 26/02 a 06/03, voltada aos testes táticos finais antes da convocação.</x:v>
+        <x:v>Torneio Brasil de Seleções previsto de 14 a 22/11/2026 como encerramento do calendário da Seleção Feminina Sub-15. A fonte não informa cidade, local físico ou tabela de jogos.</x:v>
       </x:c>
       <x:c r="O71" s="5" t="str">
-        <x:v>Fev</x:v>
+        <x:v>Nov</x:v>
       </x:c>
       <x:c r="P71" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="5" t="str">
-        <x:v>EVT-0009</x:v>
+        <x:v>EVT-0055</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C72" s="27" t="n">
-        <x:v>46482.5</x:v>
+        <x:v>46341.5</x:v>
       </x:c>
       <x:c r="D72" s="5" t="str">
-        <x:v>BR</x:v>
+        <x:v>SP</x:v>
       </x:c>
       <x:c r="E72" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo</x:v>
       </x:c>
       <x:c r="F72" s="5" t="str">
-        <x:v>Data FIFA / Convocação</x:v>
+        <x:v>Premiação</x:v>
       </x:c>
       <x:c r="G72" s="5" t="str">
-        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+        <x:v>TV Brasil / EBC / Petrobras</x:v>
       </x:c>
       <x:c r="H72" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I72" s="5" t="str"/>
+      <x:c r="I72" s="5" t="str">
+        <x:v>Petrobras</x:v>
+      </x:c>
       <x:c r="J72" s="5" t="str">
-        <x:v>A definir</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="K72" s="8"/>
       <x:c r="L72" s="8"/>
       <x:c r="M72" s="5" t="str">
-        <x:v>Informado pelo usuário</x:v>
+        <x:v>https://www.ebc.com.br/premiotvbrasilpetrobrasparaelas/</x:v>
       </x:c>
       <x:c r="N72" s="5" t="str">
-        <x:v>Última Data FIFA oficial antes do Mundial, de 05 a 13/04/2027. Período previsto para Arthur Elias fechar a lista oficial de convocadas.</x:v>
+        <x:v>Primeira edição do Prêmio TV Brasil Petrobras Para Elas, marcada para 15/11/2026, em São Paulo, com transmissão ao vivo pela TV Brasil e YouTube. A premiação reconhece atletas, treinadoras, clubes, departamentos e iniciativas relevantes para o fortalecimento do futebol feminino brasileiro. A fonte oficial confirma cidade e data, mas não informa o local físico.</x:v>
       </x:c>
       <x:c r="O72" s="5" t="str">
-        <x:v>Abr</x:v>
+        <x:v>Nov</x:v>
       </x:c>
       <x:c r="P72" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="5" t="str">
-        <x:v>EVT-0012</x:v>
+        <x:v>EVT-0007</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C73" s="27" t="n">
-        <x:v>46508.5</x:v>
+        <x:v>46350.5</x:v>
       </x:c>
       <x:c r="D73" s="5" t="str">
         <x:v>BR</x:v>
@@ -17117,7 +17117,7 @@
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F73" s="5" t="str">
-        <x:v>Preparação da Seleção</x:v>
+        <x:v>Amistosos da Seleção</x:v>
       </x:c>
       <x:c r="G73" s="5" t="str">
         <x:v>CBF / Seleção Brasileira Feminina</x:v>
@@ -17127,7 +17127,7 @@
       </x:c>
       <x:c r="I73" s="5" t="str"/>
       <x:c r="J73" s="5" t="str">
-        <x:v>Centro de treinamento a definir</x:v>
+        <x:v>A definir</x:v>
       </x:c>
       <x:c r="K73" s="8"/>
       <x:c r="L73" s="8"/>
@@ -17135,177 +17135,165 @@
         <x:v>Informado pelo usuário</x:v>
       </x:c>
       <x:c r="N73" s="5" t="str">
-        <x:v>Período de preparação fechada entre maio e junho de 2027, com concentração final e treinos intensivos sem interrupção de clubes.</x:v>
+        <x:v>Período estendido de 24/11 a 05/12/2026, permitindo até 3 jogos preparatórios.</x:v>
       </x:c>
       <x:c r="O73" s="5" t="str">
-        <x:v>Mai</x:v>
+        <x:v>Nov</x:v>
       </x:c>
       <x:c r="P73" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="5" t="str">
-        <x:v>EVT-0077</x:v>
+        <x:v>EVT-0088</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C74" s="27" t="n">
-        <x:v>46548.5</x:v>
+        <x:v>46350.5</x:v>
       </x:c>
       <x:c r="D74" s="5" t="str">
-        <x:v>RJ</x:v>
+        <x:v>BR</x:v>
       </x:c>
       <x:c r="E74" s="5" t="str">
-        <x:v>Rio de Janeiro</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="F74" s="5" t="str">
-        <x:v>Marco operacional</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G74" s="5" t="str">
-        <x:v>FIFA / administração do Maracanã</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina Sub-20</x:v>
       </x:c>
       <x:c r="H74" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I74" s="5" t="str"/>
       <x:c r="J74" s="5" t="str">
-        <x:v>Maracanã</x:v>
-      </x:c>
-      <x:c r="K74" s="8" t="n">
-        <x:v>-22.9122</x:v>
-      </x:c>
-      <x:c r="L74" s="8" t="n">
-        <x:v>-43.2302</x:v>
-      </x:c>
+        <x:v>Local a definir</x:v>
+      </x:c>
+      <x:c r="K74" s="8"/>
+      <x:c r="L74" s="8"/>
       <x:c r="M74" s="5" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N74" s="5" t="str">
-        <x:v>O Maracanã será o primeiro estádio entregue para uso exclusivo da FIFA, em 10/06/2027, 14 dias antes da abertura da Copa. As demais arenas terão início escalonado conforme a data de sua primeira partida; a fonte não publica aqui todas as datas individuais de entrega.</x:v>
+        <x:v>Janela de amistosos internacionais da Seleção Brasileira Feminina Sub-20 prevista entre 24/11 e 05/12/2026. Adversários, cidade e local físico ainda não foram divulgados.</x:v>
       </x:c>
       <x:c r="O74" s="5" t="str">
-        <x:v>Jun</x:v>
+        <x:v>Nov</x:v>
       </x:c>
       <x:c r="P74" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="5" t="str">
-        <x:v>EVT-0017</x:v>
+        <x:v>EVT-0011</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C75" s="27" t="n">
-        <x:v>46562.5</x:v>
+        <x:v>46357.5</x:v>
       </x:c>
       <x:c r="D75" s="5" t="str">
-        <x:v>RJ</x:v>
+        <x:v>BR</x:v>
       </x:c>
       <x:c r="E75" s="5" t="str">
-        <x:v>Rio de Janeiro</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
-        <x:v>Jogo da Copa</x:v>
+        <x:v>Centro de Treinamento</x:v>
       </x:c>
       <x:c r="G75" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina</x:v>
       </x:c>
       <x:c r="H75" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I75" s="5" t="str"/>
       <x:c r="J75" s="5" t="str">
-        <x:v>Maracanã</x:v>
-      </x:c>
-      <x:c r="K75" s="8" t="n">
-        <x:v>-22.9122</x:v>
-      </x:c>
-      <x:c r="L75" s="8" t="n">
-        <x:v>-43.2302</x:v>
-      </x:c>
+        <x:v>A definir</x:v>
+      </x:c>
+      <x:c r="K75" s="8"/>
+      <x:c r="L75" s="8"/>
       <x:c r="M75" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>Informado pelo usuário</x:v>
       </x:c>
       <x:c r="N75" s="5" t="str">
-        <x:v>Partida de abertura da Copa e estreia do Brasil no Grupo A; adversário será definido no sorteio final.</x:v>
+        <x:v>Definição do Team Base Camp prevista para dezembro de 2026. Data exata a definir.</x:v>
       </x:c>
       <x:c r="O75" s="5" t="str">
-        <x:v>Jun</x:v>
+        <x:v>Dez</x:v>
       </x:c>
       <x:c r="P75" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="5" t="str">
-        <x:v>EVT-0018</x:v>
+        <x:v>EVT-0089</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C76" s="27" t="n">
-        <x:v>46567.5</x:v>
+        <x:v>46362.5</x:v>
       </x:c>
       <x:c r="D76" s="5" t="str">
-        <x:v>SP</x:v>
+        <x:v>BR</x:v>
       </x:c>
       <x:c r="E76" s="5" t="str">
-        <x:v>São Paulo</x:v>
+        <x:v>Local a definir</x:v>
       </x:c>
       <x:c r="F76" s="5" t="str">
-        <x:v>Jogo da Copa</x:v>
+        <x:v>Seleções de Base</x:v>
       </x:c>
       <x:c r="G76" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina Sub-17</x:v>
       </x:c>
       <x:c r="H76" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I76" s="5" t="str"/>
       <x:c r="J76" s="5" t="str">
-        <x:v>Arena Itaquera</x:v>
-      </x:c>
-      <x:c r="K76" s="8" t="n">
-        <x:v>-23.5453</x:v>
-      </x:c>
-      <x:c r="L76" s="8" t="n">
-        <x:v>-46.4742</x:v>
-      </x:c>
+        <x:v>Local a definir</x:v>
+      </x:c>
+      <x:c r="K76" s="8"/>
+      <x:c r="L76" s="8"/>
       <x:c r="M76" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
       <x:c r="N76" s="5" t="str">
-        <x:v>Segundo jogo do Brasil na fase de grupos; adversário será definido no sorteio final.</x:v>
+        <x:v>Período de treinamento da Seleção Brasileira Feminina Sub-17 previsto de 06 a 12/12/2026. A CBF não informou cidade nem local físico.</x:v>
       </x:c>
       <x:c r="O76" s="5" t="str">
-        <x:v>Jun</x:v>
+        <x:v>Dez</x:v>
       </x:c>
       <x:c r="P76" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="5" t="str">
-        <x:v>EVT-0019</x:v>
+        <x:v>EVT-0010</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C77" s="27" t="n">
-        <x:v>46572.5</x:v>
+        <x:v>46367.5</x:v>
       </x:c>
       <x:c r="D77" s="5" t="str">
-        <x:v>DF</x:v>
+        <x:v>RJ</x:v>
       </x:c>
       <x:c r="E77" s="5" t="str">
-        <x:v>Brasília</x:v>
+        <x:v>Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F77" s="5" t="str">
-        <x:v>Jogo da Copa</x:v>
+        <x:v>Sorteio Oficial</x:v>
       </x:c>
       <x:c r="G77" s="5" t="str">
         <x:v>FIFA</x:v>
@@ -17315,200 +17303,394 @@
       </x:c>
       <x:c r="I77" s="5" t="str"/>
       <x:c r="J77" s="5" t="str">
-        <x:v>Estádio Nacional Mané Garrincha</x:v>
-      </x:c>
-      <x:c r="K77" s="8" t="n">
-        <x:v>-15.7835</x:v>
-      </x:c>
-      <x:c r="L77" s="8" t="n">
-        <x:v>-47.8992</x:v>
-      </x:c>
+        <x:v>Museu de Arte Moderna do Rio de Janeiro (MAM Rio)</x:v>
+      </x:c>
+      <x:c r="K77" s="8"/>
+      <x:c r="L77" s="8"/>
       <x:c r="M77" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/sorteio-grupos-copa-mundo-feminina-2027-data-local</x:v>
       </x:c>
       <x:c r="N77" s="5" t="str">
-        <x:v>Terceiro jogo do Brasil na fase de grupos; adversário será definido no sorteio final.</x:v>
+        <x:v>Sorteio final dos grupos confirmado para 11/12/2026 no MAM Rio. O evento definirá os oito grupos e o caminho das 32 seleções na Copa do Mundo Feminina FIFA 2027.</x:v>
       </x:c>
       <x:c r="O77" s="5" t="str">
-        <x:v>Jul</x:v>
+        <x:v>Dez</x:v>
       </x:c>
       <x:c r="P77" s="5" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="5" t="str">
-        <x:v>EVT-0020</x:v>
+        <x:v>EVT-0008</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="C78" s="27" t="n">
-        <x:v>46593.5</x:v>
+        <x:v>46444.5</x:v>
       </x:c>
       <x:c r="D78" s="5" t="str">
-        <x:v>RJ</x:v>
+        <x:v>BR</x:v>
       </x:c>
       <x:c r="E78" s="5" t="str">
-        <x:v>Rio de Janeiro</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F78" s="5" t="str">
-        <x:v>Final da Copa</x:v>
+        <x:v>Amistosos da Seleção</x:v>
       </x:c>
       <x:c r="G78" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>CBF / Seleção Brasileira Feminina</x:v>
       </x:c>
       <x:c r="H78" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I78" s="5" t="str"/>
       <x:c r="J78" s="5" t="str">
-        <x:v>Maracanã</x:v>
-      </x:c>
-      <x:c r="K78" s="8" t="n">
-        <x:v>-22.9122</x:v>
-      </x:c>
-      <x:c r="L78" s="8" t="n">
-        <x:v>-43.2302</x:v>
-      </x:c>
+        <x:v>A definir</x:v>
+      </x:c>
+      <x:c r="K78" s="8"/>
+      <x:c r="L78" s="8"/>
       <x:c r="M78" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>Informado pelo usuário</x:v>
       </x:c>
       <x:c r="N78" s="5" t="str">
-        <x:v>Final da Copa do Mundo Feminina da FIFA Brasil 2027.</x:v>
+        <x:v>Primeira janela de amistosos de 2027, de 26/02 a 06/03, voltada aos testes táticos finais antes da convocação.</x:v>
       </x:c>
       <x:c r="O78" s="5" t="str">
-        <x:v>Jul</x:v>
+        <x:v>Fev</x:v>
       </x:c>
       <x:c r="P78" s="5" t="n">
         <x:v>2027</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="5"/>
-      <x:c r="B79" s="5"/>
-      <x:c r="C79" s="6"/>
-      <x:c r="D79" s="5"/>
-      <x:c r="E79" s="5"/>
-      <x:c r="F79" s="5"/>
-      <x:c r="G79" s="5"/>
-      <x:c r="H79" s="7"/>
-      <x:c r="I79" s="5"/>
-      <x:c r="J79" s="5"/>
+      <x:c r="A79" s="5" t="str">
+        <x:v>EVT-0009</x:v>
+      </x:c>
+      <x:c r="B79" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C79" s="6" t="n">
+        <x:v>46482.5</x:v>
+      </x:c>
+      <x:c r="D79" s="5" t="str">
+        <x:v>BR</x:v>
+      </x:c>
+      <x:c r="E79" s="5" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="F79" s="5" t="str">
+        <x:v>Data FIFA / Convocação</x:v>
+      </x:c>
+      <x:c r="G79" s="5" t="str">
+        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+      </x:c>
+      <x:c r="H79" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I79" s="5" t="str"/>
+      <x:c r="J79" s="5" t="str">
+        <x:v>A definir</x:v>
+      </x:c>
       <x:c r="K79" s="8"/>
       <x:c r="L79" s="8"/>
-      <x:c r="M79" s="5"/>
-      <x:c r="N79" s="5"/>
-      <x:c r="O79" s="5"/>
-      <x:c r="P79" s="5"/>
+      <x:c r="M79" s="5" t="str">
+        <x:v>Informado pelo usuário</x:v>
+      </x:c>
+      <x:c r="N79" s="5" t="str">
+        <x:v>Última Data FIFA oficial antes do Mundial, de 05 a 13/04/2027. Período previsto para Arthur Elias fechar a lista oficial de convocadas.</x:v>
+      </x:c>
+      <x:c r="O79" s="5" t="str">
+        <x:v>Abr</x:v>
+      </x:c>
+      <x:c r="P79" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="5"/>
-      <x:c r="B80" s="5"/>
-      <x:c r="C80" s="6"/>
-      <x:c r="D80" s="5"/>
-      <x:c r="E80" s="5"/>
-      <x:c r="F80" s="5"/>
-      <x:c r="G80" s="5"/>
-      <x:c r="H80" s="7"/>
-      <x:c r="I80" s="5"/>
-      <x:c r="J80" s="5"/>
+      <x:c r="A80" s="5" t="str">
+        <x:v>EVT-0012</x:v>
+      </x:c>
+      <x:c r="B80" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C80" s="6" t="n">
+        <x:v>46508.5</x:v>
+      </x:c>
+      <x:c r="D80" s="5" t="str">
+        <x:v>BR</x:v>
+      </x:c>
+      <x:c r="E80" s="5" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="F80" s="5" t="str">
+        <x:v>Preparação da Seleção</x:v>
+      </x:c>
+      <x:c r="G80" s="5" t="str">
+        <x:v>CBF / Seleção Brasileira Feminina</x:v>
+      </x:c>
+      <x:c r="H80" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I80" s="5" t="str"/>
+      <x:c r="J80" s="5" t="str">
+        <x:v>Centro de treinamento a definir</x:v>
+      </x:c>
       <x:c r="K80" s="8"/>
       <x:c r="L80" s="8"/>
-      <x:c r="M80" s="5"/>
-      <x:c r="N80" s="5"/>
-      <x:c r="O80" s="5"/>
-      <x:c r="P80" s="5"/>
+      <x:c r="M80" s="5" t="str">
+        <x:v>Informado pelo usuário</x:v>
+      </x:c>
+      <x:c r="N80" s="5" t="str">
+        <x:v>Período de preparação fechada entre maio e junho de 2027, com concentração final e treinos intensivos sem interrupção de clubes.</x:v>
+      </x:c>
+      <x:c r="O80" s="5" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="P80" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="5"/>
-      <x:c r="B81" s="5"/>
-      <x:c r="C81" s="6"/>
-      <x:c r="D81" s="5"/>
-      <x:c r="E81" s="5"/>
-      <x:c r="F81" s="5"/>
-      <x:c r="G81" s="5"/>
-      <x:c r="H81" s="7"/>
-      <x:c r="I81" s="5"/>
-      <x:c r="J81" s="5"/>
-      <x:c r="K81" s="8"/>
-      <x:c r="L81" s="8"/>
-      <x:c r="M81" s="5"/>
-      <x:c r="N81" s="5"/>
-      <x:c r="O81" s="5"/>
-      <x:c r="P81" s="5"/>
+      <x:c r="A81" s="5" t="str">
+        <x:v>EVT-0077</x:v>
+      </x:c>
+      <x:c r="B81" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C81" s="6" t="n">
+        <x:v>46548.5</x:v>
+      </x:c>
+      <x:c r="D81" s="5" t="str">
+        <x:v>RJ</x:v>
+      </x:c>
+      <x:c r="E81" s="5" t="str">
+        <x:v>Rio de Janeiro</x:v>
+      </x:c>
+      <x:c r="F81" s="5" t="str">
+        <x:v>Marco operacional</x:v>
+      </x:c>
+      <x:c r="G81" s="5" t="str">
+        <x:v>FIFA / administração do Maracanã</x:v>
+      </x:c>
+      <x:c r="H81" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I81" s="5" t="str"/>
+      <x:c r="J81" s="5" t="str">
+        <x:v>Maracanã</x:v>
+      </x:c>
+      <x:c r="K81" s="8" t="n">
+        <x:v>-22.9122</x:v>
+      </x:c>
+      <x:c r="L81" s="8" t="n">
+        <x:v>-43.2302</x:v>
+      </x:c>
+      <x:c r="M81" s="5" t="str">
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+      </x:c>
+      <x:c r="N81" s="5" t="str">
+        <x:v>O Maracanã será o primeiro estádio entregue para uso exclusivo da FIFA, em 10/06/2027, 14 dias antes da abertura da Copa. As demais arenas terão início escalonado conforme a data de sua primeira partida; a fonte não publica aqui todas as datas individuais de entrega.</x:v>
+      </x:c>
+      <x:c r="O81" s="5" t="str">
+        <x:v>Jun</x:v>
+      </x:c>
+      <x:c r="P81" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="5"/>
-      <x:c r="B82" s="5"/>
-      <x:c r="C82" s="6"/>
-      <x:c r="D82" s="5"/>
-      <x:c r="E82" s="5"/>
-      <x:c r="F82" s="5"/>
-      <x:c r="G82" s="5"/>
-      <x:c r="H82" s="7"/>
-      <x:c r="I82" s="5"/>
-      <x:c r="J82" s="5"/>
-      <x:c r="K82" s="8"/>
-      <x:c r="L82" s="8"/>
-      <x:c r="M82" s="5"/>
-      <x:c r="N82" s="5"/>
-      <x:c r="O82" s="5"/>
-      <x:c r="P82" s="5"/>
+      <x:c r="A82" s="5" t="str">
+        <x:v>EVT-0017</x:v>
+      </x:c>
+      <x:c r="B82" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C82" s="6" t="n">
+        <x:v>46562.5</x:v>
+      </x:c>
+      <x:c r="D82" s="5" t="str">
+        <x:v>RJ</x:v>
+      </x:c>
+      <x:c r="E82" s="5" t="str">
+        <x:v>Rio de Janeiro</x:v>
+      </x:c>
+      <x:c r="F82" s="5" t="str">
+        <x:v>Jogo da Copa</x:v>
+      </x:c>
+      <x:c r="G82" s="5" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="H82" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I82" s="5" t="str"/>
+      <x:c r="J82" s="5" t="str">
+        <x:v>Maracanã</x:v>
+      </x:c>
+      <x:c r="K82" s="8" t="n">
+        <x:v>-22.9122</x:v>
+      </x:c>
+      <x:c r="L82" s="8" t="n">
+        <x:v>-43.2302</x:v>
+      </x:c>
+      <x:c r="M82" s="5" t="str">
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+      </x:c>
+      <x:c r="N82" s="5" t="str">
+        <x:v>Partida de abertura da Copa e estreia do Brasil no Grupo A; adversário será definido no sorteio final.</x:v>
+      </x:c>
+      <x:c r="O82" s="5" t="str">
+        <x:v>Jun</x:v>
+      </x:c>
+      <x:c r="P82" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="5"/>
-      <x:c r="B83" s="5"/>
-      <x:c r="C83" s="6"/>
-      <x:c r="D83" s="5"/>
-      <x:c r="E83" s="5"/>
-      <x:c r="F83" s="5"/>
-      <x:c r="G83" s="5"/>
-      <x:c r="H83" s="7"/>
-      <x:c r="I83" s="5"/>
-      <x:c r="J83" s="5"/>
-      <x:c r="K83" s="8"/>
-      <x:c r="L83" s="8"/>
-      <x:c r="M83" s="5"/>
-      <x:c r="N83" s="5"/>
-      <x:c r="O83" s="5"/>
-      <x:c r="P83" s="5"/>
+      <x:c r="A83" s="5" t="str">
+        <x:v>EVT-0018</x:v>
+      </x:c>
+      <x:c r="B83" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C83" s="6" t="n">
+        <x:v>46567.5</x:v>
+      </x:c>
+      <x:c r="D83" s="5" t="str">
+        <x:v>SP</x:v>
+      </x:c>
+      <x:c r="E83" s="5" t="str">
+        <x:v>São Paulo</x:v>
+      </x:c>
+      <x:c r="F83" s="5" t="str">
+        <x:v>Jogo da Copa</x:v>
+      </x:c>
+      <x:c r="G83" s="5" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="H83" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I83" s="5" t="str"/>
+      <x:c r="J83" s="5" t="str">
+        <x:v>Arena Itaquera</x:v>
+      </x:c>
+      <x:c r="K83" s="8" t="n">
+        <x:v>-23.5453</x:v>
+      </x:c>
+      <x:c r="L83" s="8" t="n">
+        <x:v>-46.4742</x:v>
+      </x:c>
+      <x:c r="M83" s="5" t="str">
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+      </x:c>
+      <x:c r="N83" s="5" t="str">
+        <x:v>Segundo jogo do Brasil na fase de grupos; adversário será definido no sorteio final.</x:v>
+      </x:c>
+      <x:c r="O83" s="5" t="str">
+        <x:v>Jun</x:v>
+      </x:c>
+      <x:c r="P83" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="5"/>
-      <x:c r="B84" s="5"/>
-      <x:c r="C84" s="6"/>
-      <x:c r="D84" s="5"/>
-      <x:c r="E84" s="5"/>
-      <x:c r="F84" s="5"/>
-      <x:c r="G84" s="5"/>
-      <x:c r="H84" s="7"/>
-      <x:c r="I84" s="5"/>
-      <x:c r="J84" s="5"/>
-      <x:c r="K84" s="8"/>
-      <x:c r="L84" s="8"/>
-      <x:c r="M84" s="5"/>
-      <x:c r="N84" s="5"/>
-      <x:c r="O84" s="5"/>
-      <x:c r="P84" s="5"/>
+      <x:c r="A84" s="5" t="str">
+        <x:v>EVT-0019</x:v>
+      </x:c>
+      <x:c r="B84" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C84" s="6" t="n">
+        <x:v>46572.5</x:v>
+      </x:c>
+      <x:c r="D84" s="5" t="str">
+        <x:v>DF</x:v>
+      </x:c>
+      <x:c r="E84" s="5" t="str">
+        <x:v>Brasília</x:v>
+      </x:c>
+      <x:c r="F84" s="5" t="str">
+        <x:v>Jogo da Copa</x:v>
+      </x:c>
+      <x:c r="G84" s="5" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="H84" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I84" s="5" t="str"/>
+      <x:c r="J84" s="5" t="str">
+        <x:v>Estádio Nacional Mané Garrincha</x:v>
+      </x:c>
+      <x:c r="K84" s="8" t="n">
+        <x:v>-15.7835</x:v>
+      </x:c>
+      <x:c r="L84" s="8" t="n">
+        <x:v>-47.8992</x:v>
+      </x:c>
+      <x:c r="M84" s="5" t="str">
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+      </x:c>
+      <x:c r="N84" s="5" t="str">
+        <x:v>Terceiro jogo do Brasil na fase de grupos; adversário será definido no sorteio final.</x:v>
+      </x:c>
+      <x:c r="O84" s="5" t="str">
+        <x:v>Jul</x:v>
+      </x:c>
+      <x:c r="P84" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="5"/>
-      <x:c r="B85" s="5"/>
-      <x:c r="C85" s="6"/>
-      <x:c r="D85" s="5"/>
-      <x:c r="E85" s="5"/>
-      <x:c r="F85" s="5"/>
-      <x:c r="G85" s="5"/>
-      <x:c r="H85" s="7"/>
-      <x:c r="I85" s="5"/>
-      <x:c r="J85" s="5"/>
-      <x:c r="K85" s="8"/>
-      <x:c r="L85" s="8"/>
-      <x:c r="M85" s="5"/>
-      <x:c r="N85" s="5"/>
-      <x:c r="O85" s="5"/>
-      <x:c r="P85" s="5"/>
+      <x:c r="A85" s="5" t="str">
+        <x:v>EVT-0020</x:v>
+      </x:c>
+      <x:c r="B85" s="5" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="C85" s="6" t="n">
+        <x:v>46593.5</x:v>
+      </x:c>
+      <x:c r="D85" s="5" t="str">
+        <x:v>RJ</x:v>
+      </x:c>
+      <x:c r="E85" s="5" t="str">
+        <x:v>Rio de Janeiro</x:v>
+      </x:c>
+      <x:c r="F85" s="5" t="str">
+        <x:v>Final da Copa</x:v>
+      </x:c>
+      <x:c r="G85" s="5" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="H85" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I85" s="5" t="str"/>
+      <x:c r="J85" s="5" t="str">
+        <x:v>Maracanã</x:v>
+      </x:c>
+      <x:c r="K85" s="8" t="n">
+        <x:v>-22.9122</x:v>
+      </x:c>
+      <x:c r="L85" s="8" t="n">
+        <x:v>-43.2302</x:v>
+      </x:c>
+      <x:c r="M85" s="5" t="str">
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+      </x:c>
+      <x:c r="N85" s="5" t="str">
+        <x:v>Final da Copa do Mundo Feminina da FIFA Brasil 2027.</x:v>
+      </x:c>
+      <x:c r="O85" s="5" t="str">
+        <x:v>Jul</x:v>
+      </x:c>
+      <x:c r="P85" s="5" t="n">
+        <x:v>2027</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="5"/>
@@ -24999,7 +25181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re696e867fb2640d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b7341aae2e5423f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25039,7 +25221,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str" cm="1">
-        <x:f t="array" ref="A2:A19" ca="1">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
+        <x:f t="array" ref="A2:A26" ca="1">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
         <x:v>EVT-0064</x:v>
       </x:c>
       <x:c r="B2" s="6">
@@ -25108,7 +25290,7 @@
     <x:row r="4">
       <x:c r="A4" s="5" t="str">
         <x:f ca="1"/>
-        <x:v>EVT-0022</x:v>
+        <x:v>EVT-0083</x:v>
       </x:c>
       <x:c r="B4" s="6">
         <x:f ca="1"/>
@@ -25142,7 +25324,7 @@
     <x:row r="5">
       <x:c r="A5" s="5" t="str">
         <x:f ca="1"/>
-        <x:v>EVT-0062</x:v>
+        <x:v>EVT-0022</x:v>
       </x:c>
       <x:c r="B5" s="6">
         <x:f ca="1"/>
@@ -25176,7 +25358,7 @@
     <x:row r="6">
       <x:c r="A6" s="5" t="str">
         <x:f ca="1"/>
-        <x:v>EVT-0074</x:v>
+        <x:v>EVT-0062</x:v>
       </x:c>
       <x:c r="B6" s="6">
         <x:f ca="1"/>
@@ -25210,7 +25392,7 @@
     <x:row r="7">
       <x:c r="A7" s="5" t="str">
         <x:f ca="1"/>
-        <x:v>EVT-0006</x:v>
+        <x:v>EVT-0084</x:v>
       </x:c>
       <x:c r="B7" s="6">
         <x:f ca="1"/>
@@ -25244,7 +25426,7 @@
     <x:row r="8">
       <x:c r="A8" s="5" t="str">
         <x:f ca="1"/>
-        <x:v>EVT-0055</x:v>
+        <x:v>EVT-0074</x:v>
       </x:c>
       <x:c r="B8" s="6">
         <x:f ca="1"/>
@@ -25277,7 +25459,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5" t="str">
-        <x:v>EVT-0007</x:v>
+        <x:v>EVT-0006</x:v>
       </x:c>
       <x:c r="B9" s="6"/>
       <x:c r="C9" s="5"/>
@@ -25289,7 +25471,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="str">
-        <x:v>EVT-0011</x:v>
+        <x:v>EVT-0085</x:v>
       </x:c>
       <x:c r="B10" s="6"/>
       <x:c r="C10" s="5"/>
@@ -25301,7 +25483,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5" t="str">
-        <x:v>EVT-0010</x:v>
+        <x:v>EVT-0086</x:v>
       </x:c>
       <x:c r="B11" s="6"/>
       <x:c r="C11" s="5"/>
@@ -25313,7 +25495,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5" t="str">
-        <x:v>EVT-0008</x:v>
+        <x:v>EVT-0087</x:v>
       </x:c>
       <x:c r="B12" s="6"/>
       <x:c r="C12" s="5"/>
@@ -25325,7 +25507,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5" t="str">
-        <x:v>EVT-0009</x:v>
+        <x:v>EVT-0055</x:v>
       </x:c>
       <x:c r="B13" s="6"/>
       <x:c r="C13" s="5"/>
@@ -25337,7 +25519,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5" t="str">
-        <x:v>EVT-0012</x:v>
+        <x:v>EVT-0007</x:v>
       </x:c>
       <x:c r="B14" s="6"/>
       <x:c r="C14" s="5"/>
@@ -25349,7 +25531,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="5" t="str">
-        <x:v>EVT-0077</x:v>
+        <x:v>EVT-0088</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="5"/>
@@ -25361,7 +25543,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="5" t="str">
-        <x:v>EVT-0017</x:v>
+        <x:v>EVT-0011</x:v>
       </x:c>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="5"/>
@@ -25373,48 +25555,62 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="str">
-        <x:v>EVT-0018</x:v>
+        <x:v>EVT-0089</x:v>
       </x:c>
       <x:c r="B17" s="6"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="5" t="str">
-        <x:v>EVT-0019</x:v>
+        <x:v>EVT-0010</x:v>
       </x:c>
       <x:c r="B18" s="6"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5" t="str">
+        <x:v>EVT-0008</x:v>
+      </x:c>
+      <x:c r="B19" s="6"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="5" t="str">
+        <x:v>EVT-0009</x:v>
+      </x:c>
+      <x:c r="B20" s="6"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="5" t="str">
+        <x:v>EVT-0012</x:v>
+      </x:c>
+      <x:c r="B21" s="6"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="5" t="str">
+        <x:v>EVT-0077</x:v>
+      </x:c>
+      <x:c r="B22" s="6"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="5" t="str">
+        <x:v>EVT-0017</x:v>
+      </x:c>
+      <x:c r="B23" s="6"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="5" t="str">
+        <x:v>EVT-0018</x:v>
+      </x:c>
+      <x:c r="B24" s="6"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="5" t="str">
+        <x:v>EVT-0019</x:v>
+      </x:c>
+      <x:c r="B25" s="6"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="5" t="str">
         <x:v>EVT-0020</x:v>
       </x:c>
-      <x:c r="B19" s="6"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="5"/>
-      <x:c r="B20" s="6"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="5"/>
-      <x:c r="B21" s="6"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="5"/>
-      <x:c r="B22" s="6"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="5"/>
-      <x:c r="B23" s="6"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="5"/>
-      <x:c r="B24" s="6"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="5"/>
-      <x:c r="B25" s="6"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="5"/>
       <x:c r="B26" s="6"/>
     </x:row>
     <x:row r="27">
@@ -26966,7 +27162,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb708f81d3044530"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ae3d6a0dde4efa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27324,7 +27520,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68b0a085888a4256"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bdc5521d57549b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27431,28 +27627,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="128.25">
@@ -27460,28 +27656,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27489,28 +27685,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
-        <x:v>ge</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H6" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="5" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27547,19 +27743,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G8" s="5" t="str">
         <x:v>Positivo</x:v>
@@ -27568,7 +27764,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="5" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -27576,19 +27772,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G9" s="5" t="str">
         <x:v>Positivo</x:v>
@@ -27597,7 +27793,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="5" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -27605,28 +27801,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>UOL</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -27634,19 +27830,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
         <x:v>Positivo</x:v>
@@ -27655,7 +27851,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="5" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -27663,28 +27859,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C12" s="5" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="5" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="5" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -27895,19 +28091,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C20" s="5" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E20" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G20" s="5" t="str">
         <x:v>Neutro</x:v>
@@ -27916,7 +28112,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="5" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -27924,19 +28120,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C21" s="5" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E21" s="5" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G21" s="5" t="str">
         <x:v>Neutro</x:v>
@@ -27945,7 +28141,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="5" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -27953,28 +28149,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C22" s="5" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D22" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E22" s="5" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F22" s="5" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G22" s="5" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="5" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -27982,28 +28178,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B23" s="5" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C23" s="5" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D23" s="5" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="5" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F23" s="5" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G23" s="5" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H23" s="5" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="5" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28011,19 +28207,19 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="5" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D24" s="5" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="5" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F24" s="5" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G24" s="5" t="str">
         <x:v>Positivo</x:v>
@@ -28032,7 +28228,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="5" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28069,28 +28265,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B26" s="5" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C26" s="5" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D26" s="5" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E26" s="5" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F26" s="5" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G26" s="5" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="5" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28098,57 +28294,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B27" s="5" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D27" s="5" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E27" s="5" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F27" s="5" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G27" s="5" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="5" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="5" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="27" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B28" s="5" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E28" s="5" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F28" s="5" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G28" s="5" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H28" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="5" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28156,115 +28352,115 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B29" s="5" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D29" s="5" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="5" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F29" s="5" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G29" s="5" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H29" s="5" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="5" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="27" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B30" s="5" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C30" s="5" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D30" s="5" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E30" s="5" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F30" s="5" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G30" s="5" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="5" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="5" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="27" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B31" s="5" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D31" s="5" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="5" t="str">
-        <x:v>ge</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G31" s="5" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="5" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="5" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="27" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B32" s="5" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C32" s="5" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="5" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G32" s="5" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H32" s="5" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="5" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28272,102 +28468,174 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B33" s="5" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="5" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D33" s="5" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="5" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F33" s="5" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G33" s="5" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H33" s="5" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I33" s="5" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="27" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B34" s="5" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D34" s="5" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E34" s="5" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F34" s="5" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G34" s="5" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="5" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="5" t="str">
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="6" t="n">
+        <x:v>46239.5</x:v>
+      </x:c>
+      <x:c r="B35" s="5" t="str">
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+      </x:c>
+      <x:c r="C35" s="5" t="str">
+        <x:v>Legado / futebol feminino</x:v>
+      </x:c>
+      <x:c r="D35" s="5" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="E35" s="5" t="str">
+        <x:v>O Liberal</x:v>
+      </x:c>
+      <x:c r="F35" s="5" t="str">
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+      </x:c>
+      <x:c r="G35" s="5" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H35" s="5" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I35" s="5" t="str">
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="6" t="n">
+        <x:v>46238.5</x:v>
+      </x:c>
+      <x:c r="B36" s="5" t="str">
+        <x:v>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</x:v>
+      </x:c>
+      <x:c r="C36" s="5" t="str">
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+      </x:c>
+      <x:c r="D36" s="5" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="E36" s="5" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="F36" s="5" t="str">
+        <x:v>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</x:v>
+      </x:c>
+      <x:c r="G36" s="5" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H36" s="5" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I36" s="5" t="str">
+        <x:v>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="6" t="n">
+        <x:v>46238.5</x:v>
+      </x:c>
+      <x:c r="B37" s="5" t="str">
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+      </x:c>
+      <x:c r="C37" s="5" t="str">
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+      </x:c>
+      <x:c r="D37" s="5" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="E37" s="5" t="str">
+        <x:v>Máquina do Esporte</x:v>
+      </x:c>
+      <x:c r="F37" s="5" t="str">
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+      </x:c>
+      <x:c r="G37" s="5" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H37" s="5" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I37" s="5" t="str">
         <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="6"/>
-      <x:c r="B35" s="5"/>
-      <x:c r="C35" s="5"/>
-      <x:c r="D35" s="5"/>
-      <x:c r="E35" s="5"/>
-      <x:c r="F35" s="5"/>
-      <x:c r="G35" s="5"/>
-      <x:c r="H35" s="5"/>
-      <x:c r="I35" s="5"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="6"/>
-      <x:c r="B36" s="5"/>
-      <x:c r="C36" s="5"/>
-      <x:c r="D36" s="5"/>
-      <x:c r="E36" s="5"/>
-      <x:c r="F36" s="5"/>
-      <x:c r="G36" s="5"/>
-      <x:c r="H36" s="5"/>
-      <x:c r="I36" s="5"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="6"/>
-      <x:c r="B37" s="5"/>
-      <x:c r="C37" s="5"/>
-      <x:c r="D37" s="5"/>
-      <x:c r="E37" s="5"/>
-      <x:c r="F37" s="5"/>
-      <x:c r="G37" s="5"/>
-      <x:c r="H37" s="5"/>
-      <x:c r="I37" s="5"/>
-    </x:row>
     <x:row r="38">
-      <x:c r="A38" s="6"/>
-      <x:c r="B38" s="5"/>
-      <x:c r="C38" s="5"/>
-      <x:c r="D38" s="5"/>
-      <x:c r="E38" s="5"/>
-      <x:c r="F38" s="5"/>
-      <x:c r="G38" s="5"/>
-      <x:c r="H38" s="5"/>
-      <x:c r="I38" s="5"/>
+      <x:c r="A38" s="6" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B38" s="5" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C38" s="5" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D38" s="5" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E38" s="5" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F38" s="5" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G38" s="5" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H38" s="5" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I38" s="5" t="str">
+        <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="6"/>
@@ -33462,7 +33730,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa82039835764421"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2f1350e7a7438e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34317,7 +34585,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea0f68856a6c41cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42e52e9d84a047b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35150,7 +35418,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae5303c3120d426a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf47387a18f364bd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35473,7 +35741,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d613678871c4467"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00963512d5ef4bd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona atualização da Seleção Feminina Sub-20 na Polônia
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -1345,7 +1345,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I40" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I41" headerRowCount="1">
   <tableColumns count="9">
     <tableColumn id="1" name="Data"/>
     <tableColumn id="2" name="Título"/>
@@ -29538,27 +29538,27 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
+          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>Tour da Taça / ativações / EVT-0090</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -29568,42 +29568,42 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
+          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" s="1">
       <c r="A3" s="30" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
+          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Cultura / turismo / alimentação / Salvador</t>
+          <t>Tour da Taça / ativações / EVT-0090</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>A TARDE</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
+          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -29613,12 +29613,12 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
+          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -29673,42 +29673,42 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
+          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Sorteio / governança / premiação / EVT-0010</t>
+          <t>Cultura / turismo / alimentação / Salvador</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>A TARDE</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
+          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
+          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
         </is>
       </c>
     </row>
@@ -29718,27 +29718,27 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
+          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Calendário continental / clubes / organização</t>
+          <t>Sorteio / governança / premiação / EVT-0010</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>América do Sul / Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Máquina do Esporte</t>
         </is>
       </c>
       <c r="F6" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -29753,7 +29753,7 @@
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
+          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
         </is>
       </c>
     </row>
@@ -29763,32 +29763,32 @@
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
+          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Negócios / audiência / patrocínios</t>
+          <t>Calendário continental / clubes / organização</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>América do Sul / Brasil</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>MKT Esportivo</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
+          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
@@ -29798,7 +29798,7 @@
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
+          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
         </is>
       </c>
     </row>
@@ -29808,87 +29808,87 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
+          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação / Porto Alegre</t>
+          <t>Negócios / audiência / patrocínios</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>GZH</t>
+          <t>MKT Esportivo</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
+          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
+          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
+          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Calendário / estádios / EVT-0077</t>
+          <t>Seleção Brasileira / preparação / Porto Alegre</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>GZH</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
+          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
+          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
         </is>
       </c>
     </row>
@@ -29898,27 +29898,27 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
+          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
+          <t>Calendário / estádios / EVT-0077</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
@@ -29928,12 +29928,12 @@
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
         <is>
-          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
+          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
         </is>
       </c>
     </row>
@@ -29943,27 +29943,27 @@
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
+          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado / EVT-0021</t>
+          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>TV Brasil</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
+          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -29978,7 +29978,7 @@
       </c>
       <c r="I11" s="23" t="inlineStr">
         <is>
-          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
+          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
         </is>
       </c>
     </row>
@@ -29988,27 +29988,27 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
+          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Turismo / hotelaria / economia local</t>
+          <t>Elas Jogam Summit / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>TurisNews</t>
+          <t>TV Brasil</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
+          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="I12" s="23" t="inlineStr">
         <is>
-          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
+          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
         </is>
       </c>
     </row>
@@ -30033,12 +30033,12 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
+          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Sustentabilidade / Fortaleza</t>
+          <t>Turismo / hotelaria / economia local</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
@@ -30048,12 +30048,12 @@
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>Agência Sebrae de Notícias</t>
+          <t>TurisNews</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
+          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
@@ -30068,7 +30068,7 @@
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
+          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
         </is>
       </c>
     </row>
@@ -30078,27 +30078,27 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
+          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / calendário / EVT-0010</t>
+          <t>Sustentabilidade / Fortaleza</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Agência Sebrae de Notícias</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
+          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -30108,42 +30108,42 @@
       </c>
       <c r="H14" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I14" s="23" t="inlineStr">
         <is>
-          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
+          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
+          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / negócios</t>
+          <t>Sorteio / calendário / EVT-0010</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>Exame</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -30158,7 +30158,7 @@
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
+          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
         </is>
       </c>
     </row>
@@ -30168,27 +30168,27 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
+          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Tributação / organização / políticas públicas</t>
+          <t>Patrocínio / negócios</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Governo do Estado do Rio de Janeiro</t>
+          <t>Exame</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
+          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
@@ -30203,37 +30203,37 @@
       </c>
       <c r="I16" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
+          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="29" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
+          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
+          <t>Tributação / organização / políticas públicas</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Correio</t>
+          <t>Governo do Estado do Rio de Janeiro</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
+          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -30243,42 +30243,42 @@
       </c>
       <c r="H17" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I17" s="23" t="inlineStr">
         <is>
-          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
+          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="29" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
+          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>Correio</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
+          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -30293,37 +30293,37 @@
       </c>
       <c r="I18" s="23" t="inlineStr">
         <is>
-          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
+          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="29" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
+          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
+          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -30338,7 +30338,7 @@
       </c>
       <c r="I19" s="23" t="inlineStr">
         <is>
-          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
+          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
         </is>
       </c>
     </row>
@@ -30348,12 +30348,12 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
+          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / relacionamento</t>
+          <t>Seleção Brasileira / preparação</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
@@ -30363,17 +30363,17 @@
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H20" s="23" t="inlineStr">
@@ -30383,7 +30383,7 @@
       </c>
       <c r="I20" s="23" t="inlineStr">
         <is>
-          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
+          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
         </is>
       </c>
     </row>
@@ -30393,12 +30393,12 @@
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
+          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sedes</t>
+          <t>Ingressos / relacionamento</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
@@ -30408,27 +30408,27 @@
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
+          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
         </is>
       </c>
     </row>
@@ -30438,12 +30438,12 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
+          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Investimentos públicos / segurança / infraestrutura</t>
+          <t>Calendário / sedes</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
@@ -30453,17 +30453,17 @@
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
+          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
@@ -30473,7 +30473,7 @@
       </c>
       <c r="I22" s="23" t="inlineStr">
         <is>
-          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
+          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
         </is>
       </c>
     </row>
@@ -30483,12 +30483,12 @@
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
+          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / sorteio</t>
+          <t>Investimentos públicos / segurança / infraestrutura</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -30498,12 +30498,12 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -30518,27 +30518,27 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
+          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="29" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
+          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Repescagem / sorteio</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>Brasil / Polônia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr">
@@ -30548,22 +30548,22 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I24" s="23" t="inlineStr">
         <is>
-          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
+          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
         </is>
       </c>
     </row>
@@ -30573,42 +30573,42 @@
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
+          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasil / Polônia</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
+          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H25" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I25" s="23" t="inlineStr">
         <is>
-          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
+          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
         </is>
       </c>
     </row>
@@ -30618,12 +30618,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
+          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Varejo / consumo / oportunidades comerciais</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
@@ -30633,57 +30633,57 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Revista Super Negócios / ASSERJ</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
+          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
         <is>
-          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
+          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
+          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Elas em Ação / legado / EVT-0081</t>
+          <t>Varejo / consumo / oportunidades comerciais</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>FSports</t>
+          <t>Revista Super Negócios / ASSERJ</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
+          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -30698,37 +30698,37 @@
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
+          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
+          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15 Feminina</t>
+          <t>Elas em Ação / legado / EVT-0081</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>Assunção/PRY</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>FSports</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
+          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -30743,7 +30743,7 @@
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
+          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
         </is>
       </c>
     </row>
@@ -30753,27 +30753,27 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
+          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>Operação / cidade-sede</t>
+          <t>Seleções de Base / Sub-15 Feminina</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Assunção/PRY</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>Tribuna Online</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -30783,12 +30783,12 @@
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
+          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
         </is>
       </c>
     </row>
@@ -30798,72 +30798,72 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
+          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
+          <t>Operação / cidade-sede</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Tribuna Online</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
+          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
         </is>
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
+          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="29" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
+          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sorteio</t>
+          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -30873,12 +30873,12 @@
       </c>
       <c r="H31" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
+          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
         </is>
       </c>
     </row>
@@ -30888,32 +30888,32 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
+          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / ativações</t>
+          <t>Calendário / sorteio</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H32" s="23" t="inlineStr">
@@ -30923,37 +30923,37 @@
       </c>
       <c r="I32" s="23" t="inlineStr">
         <is>
-          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
+          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="29" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
+          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
+          <t>Patrocínio / ativações</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
+          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
@@ -30963,27 +30963,27 @@
       </c>
       <c r="H33" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
+          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="29" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
+          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
@@ -30993,17 +30993,17 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H34" s="23" t="inlineStr">
@@ -31013,22 +31013,22 @@
       </c>
       <c r="I34" s="23" t="inlineStr">
         <is>
-          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
+          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>46239</v>
+        <v>46246</v>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
+          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Calendário / competições nacionais</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
@@ -31038,12 +31038,12 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
+          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -31053,12 +31053,12 @@
       </c>
       <c r="H35" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I35" s="23" t="inlineStr">
         <is>
-          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
+          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
         </is>
       </c>
     </row>
@@ -31068,42 +31068,42 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
+          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Calendário / competições nacionais</t>
         </is>
       </c>
       <c r="D36" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>Donas FC</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H36" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I36" s="23" t="inlineStr">
         <is>
-          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
+          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
         </is>
       </c>
     </row>
@@ -31113,12 +31113,12 @@
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
+          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
@@ -31128,12 +31128,12 @@
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>O Liberal</t>
+          <t>Donas FC</t>
         </is>
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
+          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
@@ -31148,37 +31148,37 @@
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
+          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</t>
+          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Legado / futebol feminino</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>O Liberal</t>
         </is>
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</t>
+          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -31193,7 +31193,7 @@
       </c>
       <c r="I38" s="23" t="inlineStr">
         <is>
-          <t>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</t>
+          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
         </is>
       </c>
     </row>
@@ -31203,32 +31203,32 @@
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
+          <t>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D39" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E39" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
+          <t>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</t>
         </is>
       </c>
       <c r="G39" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H39" s="23" t="inlineStr">
@@ -31238,65 +31238,99 @@
       </c>
       <c r="I39" s="23" t="inlineStr">
         <is>
-          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
+          <t>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>São Paulo/SP</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Máquina do Esporte</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>Neutro</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>46199</v>
       </c>
-      <c r="B40" s="23" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</t>
         </is>
       </c>
-      <c r="C40" s="23" t="inlineStr">
+      <c r="C41" s="23" t="inlineStr">
         <is>
           <t>Seleções de Base / calendário 2026</t>
         </is>
       </c>
-      <c r="D40" s="23" t="inlineStr">
+      <c r="D41" s="23" t="inlineStr">
         <is>
           <t>Brasil e exterior</t>
         </is>
       </c>
-      <c r="E40" s="23" t="inlineStr">
+      <c r="E41" s="23" t="inlineStr">
         <is>
           <t>CBF</t>
         </is>
       </c>
-      <c r="F40" s="23" t="inlineStr">
+      <c r="F41" s="23" t="inlineStr">
         <is>
           <t>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</t>
         </is>
       </c>
-      <c r="G40" s="23" t="inlineStr">
+      <c r="G41" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
-      <c r="H40" s="23" t="inlineStr">
+      <c r="H41" s="23" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="I40" s="23" t="inlineStr">
+      <c r="I41" s="23" t="inlineStr">
         <is>
           <t>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
-      <c r="I41" s="23" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>

</xml_diff>

<commit_message>
Adiciona notícia sobre Mundial Feminino Sub-20
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R375c79606a044a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R73e26bd71ad84eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R8b4fa5fcd54a41bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rbbdcea2c0fed4ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R2fb1ff27b5874e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R1f8dec3bb1ec400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rac4d014c37104b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rc745e6e531554752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R8a8ff2521cf84c77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Re3da242b40e44cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rde2109a727e94368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R486dc48558c54b4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rc40d197e09c6462e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd20305bbc27d4b18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Ra79b3c053a0b40d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R937184d7c41040ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R4c03ce71f1f34ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rbca2b502d2f447af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Re95dc9489aad4abd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R06797080c28c4ef0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rb844b47412cf4321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R5d6c95714aac49d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rcca70ff54e1e4993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R4c08a87968974e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R231f08a6a999400d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rff61dc1c0bbd4965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R08a9c593535f47d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R5211d548faa64e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R510002b7dd854e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R9b01c4b8f13c4e08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R7f7ff121835b47fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R419a9a2294764ba4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Ra270f7f147344721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R052f3a833c6947e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R64a7ec911d494913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rf89677e16eb64fd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -146,7 +146,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
@@ -206,6 +206,10 @@
     <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1134,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5ce090496ac4cde"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfca893327ecc4880"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1164,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6eea2d7424d642b5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8acbc2b6868341df"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf50db3e3a5484e19"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8f32db8203b141f3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1224,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R57a525948abc4f78"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe63de4956184cb4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1259,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2bdca2dc56f142b2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40d0b987a3874d0b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1383,7 +1387,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I42" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I43" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2959,7 +2963,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d5a291d62f4a69"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc0ff8e496548b2"/>
 </x:worksheet>
 </file>
 
@@ -5248,7 +5252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R821cd750aa904ef7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb77ab4f3109c4ad3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7556,7 +7560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ff65f6c51344a61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd37778a7b657461a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8188,7 +8192,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a895b589ba342d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29e81d3c91c947a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12378,9 +12382,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dcfbd1856ff40e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43444668f0fb4af4"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea4838bab5cd49bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R491433af8c3b4cf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12671,7 +12675,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R385f45b154254ad8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5f72f7eb1a9488d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27250,7 +27254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra98dd87f9a8e4672"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9934bc7621d44423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29150,7 +29154,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71bfc99edc7c4fed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a09f2fb248c4324"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29562,7 +29566,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58431f6cd4264c91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15da873538f491d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29625,52 +29629,52 @@
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="150.75" customHeight="1">
-      <x:c r="A2" s="30" t="n">
-        <x:v>46260</x:v>
+      <x:c r="A2" s="31" t="n">
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Polônia / Internacional</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote aos torneios da FIFA após receber garantias sobre o abandono do plano de financiamento privado. O recuo reduz o risco de impacto sobre a Copa do Mundo Feminina Sub-20 de 2026, competição em que a Seleção Brasileira estreia em 5 de setembro na Polônia.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
-      <x:c r="A3" s="30" t="n">
-        <x:v>46260</x:v>
+      <x:c r="A3" s="31" t="n">
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -29679,85 +29683,85 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
-      <x:c r="A4" s="30" t="n">
-        <x:v>46260</x:v>
+      <x:c r="A4" s="31" t="n">
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
-      <x:c r="A5" s="30" t="n">
-        <x:v>46260</x:v>
+      <x:c r="A5" s="31" t="n">
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="n">
-        <x:v>46259</x:v>
+      <x:c r="A6" s="32" t="n">
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29766,56 +29770,56 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="32" t="n">
+        <x:v>46259.5</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>Salvador/BA</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>A TARDE</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="str">
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="str">
         <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="n">
-        <x:v>46259</x:v>
-      </x:c>
-      <x:c r="B7" s="23" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="32" t="n">
+        <x:v>46259.5</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
         <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
-      <x:c r="C7" s="23" t="str">
+      <x:c r="C8" s="23" t="str">
         <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
-      <x:c r="D7" s="23" t="str">
+      <x:c r="D8" s="23" t="str">
         <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
-      <x:c r="E7" s="23" t="str">
+      <x:c r="E8" s="23" t="str">
         <x:v>Máquina do Esporte</x:v>
       </x:c>
-      <x:c r="F7" s="23" t="str">
+      <x:c r="F8" s="23" t="str">
         <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
-      </x:c>
-      <x:c r="G7" s="23" t="str">
-        <x:v>Neutro</x:v>
-      </x:c>
-      <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="n">
-        <x:v>46259</x:v>
-      </x:c>
-      <x:c r="B8" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
-      </x:c>
-      <x:c r="C8" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
-      </x:c>
-      <x:c r="D8" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
-      </x:c>
-      <x:c r="E8" s="23" t="str">
-        <x:v>ge</x:v>
-      </x:c>
-      <x:c r="F8" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -29824,143 +29828,143 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="n">
-        <x:v>46259</x:v>
+      <x:c r="A9" s="32" t="n">
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="32" t="n">
+        <x:v>46259.5</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>Negócios / audiência / patrocínios</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>MKT Esportivo</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="str">
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I10" s="23" t="str">
         <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="n">
-        <x:v>46259</x:v>
-      </x:c>
-      <x:c r="B10" s="23" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="32" t="n">
+        <x:v>46259.5</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
         <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
-      <x:c r="C10" s="23" t="str">
+      <x:c r="C11" s="23" t="str">
         <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
-      <x:c r="D10" s="23" t="str">
+      <x:c r="D11" s="23" t="str">
         <x:v>Porto Alegre/RS</x:v>
       </x:c>
-      <x:c r="E10" s="23" t="str">
+      <x:c r="E11" s="23" t="str">
         <x:v>GZH</x:v>
       </x:c>
-      <x:c r="F10" s="23" t="str">
+      <x:c r="F11" s="23" t="str">
         <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
-      <x:c r="G10" s="23" t="str">
+      <x:c r="G11" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
-      <x:c r="H10" s="23" t="str">
+      <x:c r="H11" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
-      <x:c r="I10" s="23" t="str">
+      <x:c r="I11" s="23" t="str">
         <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="n">
-        <x:v>46258</x:v>
-      </x:c>
-      <x:c r="B11" s="23" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="32" t="n">
+        <x:v>46258.5</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
         <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
-      <x:c r="C11" s="23" t="str">
+      <x:c r="C12" s="23" t="str">
         <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
-      <x:c r="D11" s="23" t="str">
+      <x:c r="D12" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="E11" s="23" t="str">
+      <x:c r="E12" s="23" t="str">
         <x:v>UOL</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="str">
+      <x:c r="F12" s="23" t="str">
         <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
-      </x:c>
-      <x:c r="G11" s="23" t="str">
-        <x:v>Positivo</x:v>
-      </x:c>
-      <x:c r="H11" s="23" t="str">
-        <x:v>Alto</x:v>
-      </x:c>
-      <x:c r="I11" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="n">
-        <x:v>46258</x:v>
-      </x:c>
-      <x:c r="B12" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
-      </x:c>
-      <x:c r="C12" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="str">
-        <x:v>CBF</x:v>
-      </x:c>
-      <x:c r="F12" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="29" t="n">
-        <x:v>46258</x:v>
+      <x:c r="A13" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29969,27 +29973,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29" t="n">
-        <x:v>46258</x:v>
+      <x:c r="A14" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29998,27 +30002,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29" t="n">
-        <x:v>46258</x:v>
+      <x:c r="A15" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30027,56 +30031,56 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="n">
-        <x:v>46258</x:v>
+      <x:c r="A16" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="n">
-        <x:v>46257</x:v>
+      <x:c r="A17" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30085,27 +30089,27 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="29" t="n">
-        <x:v>46257</x:v>
+      <x:c r="A18" s="32" t="n">
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30114,56 +30118,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="n">
-        <x:v>46256</x:v>
+      <x:c r="A19" s="32" t="n">
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="n">
-        <x:v>46255</x:v>
+      <x:c r="A20" s="32" t="n">
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30172,27 +30176,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="29" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A21" s="32" t="n">
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30201,114 +30205,114 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A22" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="29" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A23" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A24" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A25" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -30317,114 +30321,114 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="29" t="n">
-        <x:v>46253</x:v>
+      <x:c r="A26" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H26" s="23" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="str">
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="32" t="n">
+        <x:v>46253.5</x:v>
+      </x:c>
+      <x:c r="B27" s="23" t="str">
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="str">
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="str">
+        <x:v>Brasil / Polônia</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="str">
+        <x:v>FIFA</x:v>
+      </x:c>
+      <x:c r="F27" s="23" t="str">
         <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
-      <x:c r="G26" s="23" t="str">
+      <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
-      <x:c r="H26" s="23" t="str">
+      <x:c r="H27" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
-      <x:c r="I26" s="23" t="str">
+      <x:c r="I27" s="23" t="str">
         <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="29" t="n">
-        <x:v>46253</x:v>
-      </x:c>
-      <x:c r="B27" s="23" t="str">
+    <x:row r="28">
+      <x:c r="A28" s="32" t="n">
+        <x:v>46253.5</x:v>
+      </x:c>
+      <x:c r="B28" s="23" t="str">
         <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
-      <x:c r="C27" s="23" t="str">
+      <x:c r="C28" s="23" t="str">
         <x:v>Políticas públicas / educação</x:v>
-      </x:c>
-      <x:c r="D27" s="23" t="str">
-        <x:v>Brasil</x:v>
-      </x:c>
-      <x:c r="E27" s="23" t="str">
-        <x:v>UOL</x:v>
-      </x:c>
-      <x:c r="F27" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
-      </x:c>
-      <x:c r="G27" s="23" t="str">
-        <x:v>Neutro</x:v>
-      </x:c>
-      <x:c r="H27" s="23" t="str">
-        <x:v>Alto</x:v>
-      </x:c>
-      <x:c r="I27" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="29" t="n">
-        <x:v>46253</x:v>
-      </x:c>
-      <x:c r="B28" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
-      </x:c>
-      <x:c r="C28" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
+        <x:v>UOL</x:v>
+      </x:c>
+      <x:c r="F28" s="23" t="str">
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+      </x:c>
+      <x:c r="G28" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H28" s="23" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I28" s="23" t="str">
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="32" t="n">
+        <x:v>46253.5</x:v>
+      </x:c>
+      <x:c r="B29" s="23" t="str">
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="str">
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="str">
         <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
-      <x:c r="F28" s="23" t="str">
+      <x:c r="F29" s="23" t="str">
         <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
-      </x:c>
-      <x:c r="G28" s="23" t="str">
-        <x:v>Positivo</x:v>
-      </x:c>
-      <x:c r="H28" s="23" t="str">
-        <x:v>Médio</x:v>
-      </x:c>
-      <x:c r="I28" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="29" t="n">
-        <x:v>46252</x:v>
-      </x:c>
-      <x:c r="B29" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
-      </x:c>
-      <x:c r="C29" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="str">
-        <x:v>FSports</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30433,27 +30437,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="29" t="n">
-        <x:v>46251</x:v>
+      <x:c r="A30" s="32" t="n">
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30462,259 +30466,259 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="29" t="n">
-        <x:v>46251</x:v>
+      <x:c r="A31" s="32" t="n">
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I31" s="23" t="str">
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="32" t="n">
+        <x:v>46251.5</x:v>
+      </x:c>
+      <x:c r="B32" s="23" t="str">
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+      </x:c>
+      <x:c r="C32" s="23" t="str">
+        <x:v>Operação / cidade-sede</x:v>
+      </x:c>
+      <x:c r="D32" s="23" t="str">
+        <x:v>Recife/PE</x:v>
+      </x:c>
+      <x:c r="E32" s="23" t="str">
+        <x:v>Tribuna Online</x:v>
+      </x:c>
+      <x:c r="F32" s="23" t="str">
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+      </x:c>
+      <x:c r="G32" s="23" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H32" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I31" s="23" t="str">
+      <x:c r="I32" s="23" t="str">
         <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="29" t="n">
-        <x:v>46251</x:v>
-      </x:c>
-      <x:c r="B32" s="23" t="str">
+    <x:row r="33">
+      <x:c r="A33" s="32" t="n">
+        <x:v>46251.5</x:v>
+      </x:c>
+      <x:c r="B33" s="23" t="str">
         <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
-      <x:c r="C32" s="23" t="str">
+      <x:c r="C33" s="23" t="str">
         <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
-      <x:c r="D32" s="23" t="str">
+      <x:c r="D33" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
-      <x:c r="E32" s="23" t="str">
+      <x:c r="E33" s="23" t="str">
         <x:v>UOL</x:v>
       </x:c>
-      <x:c r="F32" s="23" t="str">
+      <x:c r="F33" s="23" t="str">
         <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
-      </x:c>
-      <x:c r="G32" s="23" t="str">
-        <x:v>Neutro</x:v>
-      </x:c>
-      <x:c r="H32" s="23" t="str">
-        <x:v>Médio</x:v>
-      </x:c>
-      <x:c r="I32" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="29" t="n">
-        <x:v>46248</x:v>
-      </x:c>
-      <x:c r="B33" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
-      </x:c>
-      <x:c r="C33" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="str">
-        <x:v>Brasil</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="str">
-        <x:v>ge</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="29" t="n">
-        <x:v>46248</x:v>
+      <x:c r="A34" s="32" t="n">
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="6" t="n">
-        <x:v>46247</x:v>
+      <x:c r="A35" s="32" t="n">
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="6" t="n">
-        <x:v>46246</x:v>
+      <x:c r="A36" s="32" t="n">
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="6" t="n">
-        <x:v>46239</x:v>
+      <x:c r="A37" s="32" t="n">
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I37" s="23" t="str">
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="32" t="n">
+        <x:v>46239.5</x:v>
+      </x:c>
+      <x:c r="B38" s="23" t="str">
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+      </x:c>
+      <x:c r="C38" s="23" t="str">
+        <x:v>Calendário / competições nacionais</x:v>
+      </x:c>
+      <x:c r="D38" s="23" t="str">
+        <x:v>Brasil</x:v>
+      </x:c>
+      <x:c r="E38" s="23" t="str">
+        <x:v>ge</x:v>
+      </x:c>
+      <x:c r="F38" s="23" t="str">
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+      </x:c>
+      <x:c r="G38" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H38" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I37" s="23" t="str">
+      <x:c r="I38" s="23" t="str">
         <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="6" t="n">
-        <x:v>46239</x:v>
-      </x:c>
-      <x:c r="B38" s="23" t="str">
+    <x:row r="39">
+      <x:c r="A39" s="32" t="n">
+        <x:v>46239.5</x:v>
+      </x:c>
+      <x:c r="B39" s="23" t="str">
         <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
-      <x:c r="C38" s="23" t="str">
+      <x:c r="C39" s="23" t="str">
         <x:v>Elas Jogam Summit / legado</x:v>
-      </x:c>
-      <x:c r="D38" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
-      </x:c>
-      <x:c r="E38" s="23" t="str">
-        <x:v>Donas FC</x:v>
-      </x:c>
-      <x:c r="F38" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
-      </x:c>
-      <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
-      </x:c>
-      <x:c r="H38" s="23" t="str">
-        <x:v>Médio</x:v>
-      </x:c>
-      <x:c r="I38" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="6" t="n">
-        <x:v>46239</x:v>
-      </x:c>
-      <x:c r="B39" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
-      </x:c>
-      <x:c r="C39" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30723,27 +30727,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="6" t="n">
-        <x:v>46238</x:v>
+      <x:c r="A40" s="32" t="n">
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -30752,77 +30756,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="6" t="n">
-        <x:v>46238</x:v>
+      <x:c r="A41" s="32" t="n">
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="6" t="n">
-        <x:v>46199</x:v>
+      <x:c r="A42" s="32" t="n">
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I42" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B43" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C43" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D43" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E43" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F43" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G43" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H43" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I42" s="23" t="str">
+      <x:c r="I43" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="6" t="n"/>
-      <x:c r="B43" s="23" t="n"/>
-      <x:c r="C43" s="23" t="n"/>
-      <x:c r="D43" s="23" t="n"/>
-      <x:c r="E43" s="23" t="n"/>
-      <x:c r="F43" s="23" t="n"/>
-      <x:c r="G43" s="23" t="n"/>
-      <x:c r="H43" s="23" t="n"/>
-      <x:c r="I43" s="23" t="n"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="6" t="n"/>
@@ -35862,7 +35884,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R396d8c260d834e4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aeffd3300df4e12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36765,7 +36787,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9f2cb28f4e24667"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d8f9607a7c4880"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37644,7 +37666,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c7b508d103f4f66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc02d4a3dd3d4239"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38067,7 +38089,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a692b4ae1b14d7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e3562645f6441dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona análise da preparação da Seleção Feminina Sub-20
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rbc1ab59a5cdc47c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R558c4609f888485d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R5f55377a5bb142b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R43d379ccf4824174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R309f1ae529bd4942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Rd9618b74657c4a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R3c4c16c65aa7483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R60a835390a714501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R098cca200082415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R379049ca556c4643"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R21fa23cde5f64046"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R3c90939e27da48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rdd4586110cbc473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R03c9b68d182444f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Ra57886afb3874502"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R877046f4fb694daa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rb417126701b64a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R7f3599532b67422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R48d70f18d2694277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rf0066205874f4946"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R108c34a760ad4833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R66415930b8be4219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rcdb1b5bcbdb04877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R093c6db3556b4cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R77f17575e5b44a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rfc9f4db4dda04cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R453385f6f26247bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rdeeade0744654106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R3553ebc536914c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R26d0fa8939664ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rab715d8a63724241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd27f1d6955a546d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rb0813f338bde44ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rb66e2cfc12654b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rd58f112cf51d43b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R6f1b2964cf5a4525"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -146,7 +146,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
@@ -206,6 +206,10 @@
     <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1134,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0c1a05a1401544f4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R224362d9feb44ac7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1164,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra26c16a86bcf423b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52310fcb1c274e95"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba2cdb145547499e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R21ac8e901fa3444d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1224,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2c9721890f2a470c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7d0ad3bafca477b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1259,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R106eb6ea3940439e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7eeece6a58d34be6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1383,7 +1387,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I42" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I43" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2959,7 +2963,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5c4678d8d74f2a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra79a2a21e8d04da1"/>
 </x:worksheet>
 </file>
 
@@ -5248,7 +5252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6942a28ef90a49f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref66c7a6ef424191"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7556,7 +7560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33bbb236761f4854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05fe3924cea04a43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8188,7 +8192,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad00e59200b74d7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c682ee034fc414d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12378,9 +12382,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce838828195240b1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7b9db7df724051"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e1274a1a2f34daf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9582a53ec2da4a16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12671,7 +12675,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac49c41b71a405d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R024bf478f1264df3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25222,7 +25226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a460c9306b446b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R952fe1b16d5643f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27122,7 +27126,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b11f9af1914da6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb5aaea26e5e4ccc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27534,7 +27538,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf3987d03f904312"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb679921e615b45b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27597,36 +27601,36 @@
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="150.75" customHeight="1">
-      <x:c r="A2" s="30" t="n">
+      <x:c r="A2" s="31" t="n">
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
-      <x:c r="A3" s="30" t="n">
+      <x:c r="A3" s="31" t="n">
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
@@ -27655,52 +27659,52 @@
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
-      <x:c r="A4" s="30" t="n">
-        <x:v>46260.5</x:v>
+      <x:c r="A4" s="31" t="n">
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
-      <x:c r="A5" s="30" t="n">
+      <x:c r="A5" s="31" t="n">
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27709,85 +27713,85 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="n">
+      <x:c r="A6" s="32" t="n">
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="n">
+      <x:c r="A7" s="32" t="n">
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="n">
+      <x:c r="A8" s="32" t="n">
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27796,230 +27800,230 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="n">
+      <x:c r="A9" s="32" t="n">
+        <x:v>46260.5</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>Internacional</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>Folha de S.Paulo / AFP</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="str">
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="str">
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="32" t="n">
         <x:v>46259.5</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
-      </x:c>
-      <x:c r="C9" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
-      </x:c>
-      <x:c r="D9" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
-      </x:c>
-      <x:c r="E9" s="23" t="str">
-        <x:v>A TARDE</x:v>
-      </x:c>
-      <x:c r="F9" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
-      </x:c>
-      <x:c r="G9" s="23" t="str">
-        <x:v>Positivo</x:v>
-      </x:c>
-      <x:c r="H9" s="23" t="str">
-        <x:v>Médio</x:v>
-      </x:c>
-      <x:c r="I9" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="n">
-        <x:v>46259.5</x:v>
-      </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="n">
+      <x:c r="A11" s="32" t="n">
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="29" t="n">
+      <x:c r="A12" s="32" t="n">
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="29" t="n">
+      <x:c r="A13" s="32" t="n">
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29" t="n">
-        <x:v>46258.5</x:v>
+      <x:c r="A14" s="32" t="n">
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29" t="n">
+      <x:c r="A15" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
         <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="n">
+      <x:c r="A16" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28028,11 +28032,11 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="n">
+      <x:c r="A17" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
@@ -28061,23 +28065,23 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="29" t="n">
+      <x:c r="A18" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28086,56 +28090,56 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="n">
+      <x:c r="A19" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
         <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="n">
-        <x:v>46257.5</x:v>
+      <x:c r="A20" s="32" t="n">
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28144,11 +28148,11 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="29" t="n">
+      <x:c r="A21" s="32" t="n">
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
@@ -28177,52 +28181,52 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29" t="n">
-        <x:v>46256.5</x:v>
+      <x:c r="A22" s="32" t="n">
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="29" t="n">
-        <x:v>46255.5</x:v>
+      <x:c r="A23" s="32" t="n">
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28231,27 +28235,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29" t="n">
-        <x:v>46254.5</x:v>
+      <x:c r="A24" s="32" t="n">
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28260,143 +28264,143 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29" t="n">
+      <x:c r="A25" s="32" t="n">
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="29" t="n">
+      <x:c r="A26" s="32" t="n">
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="29" t="n">
+      <x:c r="A27" s="32" t="n">
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="29" t="n">
+      <x:c r="A28" s="32" t="n">
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H28" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="29" t="n">
-        <x:v>46253.5</x:v>
+      <x:c r="A29" s="32" t="n">
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28405,85 +28409,85 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="29" t="n">
+      <x:c r="A30" s="32" t="n">
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="29" t="n">
+      <x:c r="A31" s="32" t="n">
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="29" t="n">
-        <x:v>46252.5</x:v>
+      <x:c r="A32" s="32" t="n">
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28492,27 +28496,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29" t="n">
-        <x:v>46251.5</x:v>
+      <x:c r="A33" s="32" t="n">
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28521,98 +28525,98 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="32" t="n">
+        <x:v>46251.5</x:v>
+      </x:c>
+      <x:c r="B34" s="23" t="str">
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+      </x:c>
+      <x:c r="C34" s="23" t="str">
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+      </x:c>
+      <x:c r="D34" s="23" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="E34" s="23" t="str">
+        <x:v>UOL</x:v>
+      </x:c>
+      <x:c r="F34" s="23" t="str">
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+      </x:c>
+      <x:c r="G34" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H34" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I34" s="23" t="str">
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="32" t="n">
+        <x:v>46251.5</x:v>
+      </x:c>
+      <x:c r="B35" s="23" t="str">
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+      </x:c>
+      <x:c r="C35" s="23" t="str">
+        <x:v>Operação / cidade-sede</x:v>
+      </x:c>
+      <x:c r="D35" s="23" t="str">
+        <x:v>Recife/PE</x:v>
+      </x:c>
+      <x:c r="E35" s="23" t="str">
+        <x:v>Tribuna Online</x:v>
+      </x:c>
+      <x:c r="F35" s="23" t="str">
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+      </x:c>
+      <x:c r="G35" s="23" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H35" s="23" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="I35" s="23" t="str">
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="32" t="n">
+        <x:v>46251.5</x:v>
+      </x:c>
+      <x:c r="B36" s="23" t="str">
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+      </x:c>
+      <x:c r="C36" s="23" t="str">
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+      </x:c>
+      <x:c r="D36" s="23" t="str">
+        <x:v>Assunção/PRY</x:v>
+      </x:c>
+      <x:c r="E36" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F36" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+      </x:c>
+      <x:c r="G36" s="23" t="str">
+        <x:v>Positivo</x:v>
+      </x:c>
+      <x:c r="H36" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I36" s="23" t="str">
         <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="29" t="n">
-        <x:v>46251.5</x:v>
-      </x:c>
-      <x:c r="B34" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
-      </x:c>
-      <x:c r="C34" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="str">
-        <x:v>Recife/PE</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
-      </x:c>
-      <x:c r="G34" s="23" t="str">
-        <x:v>Positivo</x:v>
-      </x:c>
-      <x:c r="H34" s="23" t="str">
-        <x:v>Alto</x:v>
-      </x:c>
-      <x:c r="I34" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="6" t="n">
-        <x:v>46251.5</x:v>
-      </x:c>
-      <x:c r="B35" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
-      </x:c>
-      <x:c r="C35" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
-      </x:c>
-      <x:c r="D35" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="str">
-        <x:v>UOL</x:v>
-      </x:c>
-      <x:c r="F35" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
-      </x:c>
-      <x:c r="G35" s="23" t="str">
-        <x:v>Neutro</x:v>
-      </x:c>
-      <x:c r="H35" s="23" t="str">
-        <x:v>Médio</x:v>
-      </x:c>
-      <x:c r="I35" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="6" t="n">
-        <x:v>46248.5</x:v>
-      </x:c>
-      <x:c r="B36" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
-      </x:c>
-      <x:c r="C36" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
-      </x:c>
-      <x:c r="D36" s="23" t="str">
-        <x:v>Brasil</x:v>
-      </x:c>
-      <x:c r="E36" s="23" t="str">
-        <x:v>ge</x:v>
-      </x:c>
-      <x:c r="F36" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
-      </x:c>
-      <x:c r="G36" s="23" t="str">
-        <x:v>Neutro</x:v>
-      </x:c>
-      <x:c r="H36" s="23" t="str">
-        <x:v>Alto</x:v>
-      </x:c>
-      <x:c r="I36" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
-      </x:c>
-    </x:row>
     <x:row r="37">
-      <x:c r="A37" s="6" t="n">
+      <x:c r="A37" s="32" t="n">
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
@@ -28641,110 +28645,110 @@
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="6" t="n">
-        <x:v>46247.5</x:v>
+      <x:c r="A38" s="32" t="n">
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="6" t="n">
-        <x:v>46246.5</x:v>
+      <x:c r="A39" s="32" t="n">
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="6" t="n">
-        <x:v>46239.5</x:v>
+      <x:c r="A40" s="32" t="n">
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="6" t="n">
+      <x:c r="A41" s="32" t="n">
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28753,27 +28757,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="6" t="n">
+      <x:c r="A42" s="32" t="n">
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28782,40 +28786,40 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="6" t="n">
-        <x:v>46238.5</x:v>
+      <x:c r="A43" s="32" t="n">
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Camilla Orlando projeta Brasil Sub-20 ofensivo no Mundial</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/camilla-orlando-treinadora-brasil-sub-20-entrevista-agosto-2026</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A treinadora Camilla Orlando detalhou à FIFA a preparação da Seleção Brasileira Feminina Sub-20 e afirmou que a equipe pretende buscar o gol e reproduzir princípios da Seleção principal no Mundial da Polônia.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="6" t="n">
+      <x:c r="A44" s="32" t="n">
         <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
@@ -28844,7 +28848,7 @@
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="6" t="n">
+      <x:c r="A45" s="32" t="n">
         <x:v>46199.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
@@ -28873,7 +28877,7 @@
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="6" t="n"/>
+      <x:c r="A46" s="32" t="n"/>
       <x:c r="B46" s="23" t="n"/>
       <x:c r="C46" s="23" t="n"/>
       <x:c r="D46" s="23" t="n"/>
@@ -33888,7 +33892,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63277f38f53d4ad8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b3ccca1b1d24c1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34791,7 +34795,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a88435131044594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910a5a1104e2403e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35670,7 +35674,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra02f8567a79442e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R772cd13ff3744af2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36093,7 +36097,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94401c57fa1a47e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2908d4f350b34365"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona medidas de proteção às mulheres para a Copa 2027 em Salvador
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R48d70f18d2694277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rf0066205874f4946"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R108c34a760ad4833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R66415930b8be4219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rcdb1b5bcbdb04877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R093c6db3556b4cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R77f17575e5b44a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rfc9f4db4dda04cd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R453385f6f26247bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rdeeade0744654106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R3553ebc536914c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R26d0fa8939664ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rab715d8a63724241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd27f1d6955a546d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rb0813f338bde44ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rb66e2cfc12654b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rd58f112cf51d43b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R6f1b2964cf5a4525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Ra45d5a80dceb465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R4c258a994ed84df5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rd790441b5c7d49f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rd88014db6f3e4c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R48144a2d0c0948f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Rec398d4f73284bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R3cd00c8ab5bc4d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rb8875e4c92644f00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R2a8e0c22797146d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R3ea844244d7542da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Recd62d89547c4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rb711e75659b14e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R060e40d6020c47bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rf3993facb10f4a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R166ed06f0e164a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R5607d68f53484cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R066e4336b9b64774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R54078e0c4d284310"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R224362d9feb44ac7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R11cd64a99f4741be"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52310fcb1c274e95"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec9470bbf9ad4d78"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R21ac8e901fa3444d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3738a5c31fd448be"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7d0ad3bafca477b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R177362106b694103"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7eeece6a58d34be6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabdff90761d6429b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,7 +1387,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I43" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I44" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2963,7 +2963,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra79a2a21e8d04da1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3034f15373b74066"/>
 </x:worksheet>
 </file>
 
@@ -5252,7 +5252,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref66c7a6ef424191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3a0adb4f35f40d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7560,7 +7560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05fe3924cea04a43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135a6dfb99de4d26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8192,7 +8192,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c682ee034fc414d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75fc705b49ab453a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12382,9 +12382,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7b9db7df724051"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19467df31d9e4123"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9582a53ec2da4a16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6804a0601a8041bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12675,7 +12675,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R024bf478f1264df3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00fc4522fe5434a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25226,7 +25226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R952fe1b16d5643f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b845ea4d89e4f9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27126,7 +27126,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb5aaea26e5e4ccc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80ed06c0e08d4ec6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27538,7 +27538,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb679921e615b45b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07a5dafb1f548c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27605,28 +27605,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
@@ -27634,28 +27634,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27663,48 +27663,48 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
       <x:c r="A5" s="31" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27713,7 +27713,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27721,28 +27721,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27750,19 +27750,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27771,7 +27771,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -27779,19 +27779,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27800,7 +27800,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -27808,57 +27808,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -27866,28 +27866,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -27895,19 +27895,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -27916,7 +27916,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -27924,19 +27924,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -27945,7 +27945,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -27953,57 +27953,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28011,28 +28011,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28040,19 +28040,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28061,7 +28061,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28098,19 +28098,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28119,7 +28119,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28127,48 +28127,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
         <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28177,7 +28177,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28211,51 +28211,51 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28264,36 +28264,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28301,28 +28301,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28330,28 +28330,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28359,28 +28359,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H28" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28388,57 +28388,57 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28446,28 +28446,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28475,48 +28475,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28525,36 +28525,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28562,28 +28562,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28591,39 +28591,39 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
@@ -28632,16 +28632,16 @@
         <x:v>UOL</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28675,89 +28675,89 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -28765,28 +28765,28 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -28794,57 +28794,57 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -33892,7 +33892,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b3ccca1b1d24c1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34526460b02e45f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34795,7 +34795,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910a5a1104e2403e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c004669031b4127"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35674,7 +35674,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R772cd13ff3744af2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra698a6dc924044fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36097,7 +36097,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2908d4f350b34365"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a80dc7d8054105"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Remove notícia duplicada e sincroniza planilha
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Ra45d5a80dceb465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R4c258a994ed84df5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rd790441b5c7d49f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rd88014db6f3e4c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R48144a2d0c0948f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Rec398d4f73284bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R3cd00c8ab5bc4d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rb8875e4c92644f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R2a8e0c22797146d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R3ea844244d7542da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Recd62d89547c4f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rb711e75659b14e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R060e40d6020c47bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rf3993facb10f4a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R166ed06f0e164a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R5607d68f53484cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R066e4336b9b64774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R54078e0c4d284310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R466c76ffa7a345e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R684fd1ca9c4b45bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Refb9a20472dd4465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rc83268b0fdb141e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R56f0255bd705412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R5e52aa2429cc4bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rc235af7f8ca84129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5ba24e109cd24200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rb0f0ef9923194f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R1fd332f9318e4b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R031fddd5a6cb4ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Re6a68e7f6ace4a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R4f28c0e102844981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R749c2f1418874b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R0247607662f84d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R47d9eb3c2de042ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R2f206fbf24134adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R29a973dc711e48ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R11cd64a99f4741be"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R11a99a24ce114481"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec9470bbf9ad4d78"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfacd497295f14338"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3738a5c31fd448be"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48f61a83e8014d67"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R177362106b694103"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf196b58698df4559"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabdff90761d6429b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25a689e36e0e4229"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,7 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I44" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I46"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2963,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3034f15373b74066"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4de84697034dc7"/>
 </x:worksheet>
 </file>
 
@@ -5252,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3a0adb4f35f40d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe7a25df30bc4122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7560,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135a6dfb99de4d26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reac15c6d5bdb42e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8192,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75fc705b49ab453a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ddc1fc14c514d97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12382,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19467df31d9e4123"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14db8528a18a4046"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6804a0601a8041bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445df68e09244239"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12675,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00fc4522fe5434a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6423d04ce334ae5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25226,7 +25227,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b845ea4d89e4f9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1210e3efed544d27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27126,7 +27127,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80ed06c0e08d4ec6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72c7b655527a4d04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27538,7 +27539,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07a5dafb1f548c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06f369a6ef3d456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27634,28 +27635,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27692,28 +27693,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27721,28 +27722,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27750,28 +27751,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -27808,28 +27809,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -27837,28 +27838,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -27866,28 +27867,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -27895,28 +27896,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -27953,28 +27954,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -27982,28 +27983,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28011,19 +28012,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
         <x:v>UOL</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28032,7 +28033,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28040,19 +28041,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28061,7 +28062,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28069,19 +28070,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28090,7 +28091,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28098,19 +28099,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28119,7 +28120,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28127,19 +28128,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28148,7 +28149,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28156,19 +28157,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
         <x:v>UOL</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28177,7 +28178,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28185,19 +28186,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28206,7 +28207,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28214,19 +28215,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28235,7 +28236,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28301,28 +28302,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28330,28 +28331,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28388,28 +28389,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28417,28 +28418,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28446,19 +28447,19 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28467,7 +28468,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28504,19 +28505,19 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28525,7 +28526,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28562,28 +28563,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28620,28 +28621,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28649,28 +28650,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28678,28 +28679,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -28765,28 +28766,28 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -28823,1763 +28824,1781 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I45" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B46" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G46" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H46" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I45" s="23" t="str">
+      <x:c r="I46" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="32" t="n"/>
-      <x:c r="B46" s="23" t="n"/>
-      <x:c r="C46" s="23" t="n"/>
-      <x:c r="D46" s="23" t="n"/>
-      <x:c r="E46" s="23" t="n"/>
-      <x:c r="F46" s="23" t="n"/>
-      <x:c r="G46" s="23" t="n"/>
-      <x:c r="H46" s="23" t="n"/>
-      <x:c r="I46" s="23" t="n"/>
-    </x:row>
     <x:row r="47">
-      <x:c r="A47" s="6" t="n"/>
-      <x:c r="B47" s="23" t="n"/>
-      <x:c r="C47" s="23" t="n"/>
-      <x:c r="D47" s="23" t="n"/>
-      <x:c r="E47" s="23" t="n"/>
-      <x:c r="F47" s="23" t="n"/>
-      <x:c r="G47" s="23" t="n"/>
-      <x:c r="H47" s="23" t="n"/>
-      <x:c r="I47" s="23" t="n"/>
+      <x:c r="A47" s="6"/>
+      <x:c r="B47" s="23"/>
+      <x:c r="C47" s="23"/>
+      <x:c r="D47" s="23"/>
+      <x:c r="E47" s="23"/>
+      <x:c r="F47" s="23"/>
+      <x:c r="G47" s="23"/>
+      <x:c r="H47" s="23"/>
+      <x:c r="I47" s="23"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="6" t="n"/>
-      <x:c r="B48" s="23" t="n"/>
-      <x:c r="C48" s="23" t="n"/>
-      <x:c r="D48" s="23" t="n"/>
-      <x:c r="E48" s="23" t="n"/>
-      <x:c r="F48" s="23" t="n"/>
-      <x:c r="G48" s="23" t="n"/>
-      <x:c r="H48" s="23" t="n"/>
-      <x:c r="I48" s="23" t="n"/>
+      <x:c r="A48" s="6"/>
+      <x:c r="B48" s="23"/>
+      <x:c r="C48" s="23"/>
+      <x:c r="D48" s="23"/>
+      <x:c r="E48" s="23"/>
+      <x:c r="F48" s="23"/>
+      <x:c r="G48" s="23"/>
+      <x:c r="H48" s="23"/>
+      <x:c r="I48" s="23"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="6" t="n"/>
-      <x:c r="B49" s="23" t="n"/>
-      <x:c r="C49" s="23" t="n"/>
-      <x:c r="D49" s="23" t="n"/>
-      <x:c r="E49" s="23" t="n"/>
-      <x:c r="F49" s="23" t="n"/>
-      <x:c r="G49" s="23" t="n"/>
-      <x:c r="H49" s="23" t="n"/>
-      <x:c r="I49" s="23" t="n"/>
+      <x:c r="A49" s="6"/>
+      <x:c r="B49" s="23"/>
+      <x:c r="C49" s="23"/>
+      <x:c r="D49" s="23"/>
+      <x:c r="E49" s="23"/>
+      <x:c r="F49" s="23"/>
+      <x:c r="G49" s="23"/>
+      <x:c r="H49" s="23"/>
+      <x:c r="I49" s="23"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="6" t="n"/>
-      <x:c r="B50" s="23" t="n"/>
-      <x:c r="C50" s="23" t="n"/>
-      <x:c r="D50" s="23" t="n"/>
-      <x:c r="E50" s="23" t="n"/>
-      <x:c r="F50" s="23" t="n"/>
-      <x:c r="G50" s="23" t="n"/>
-      <x:c r="H50" s="23" t="n"/>
-      <x:c r="I50" s="23" t="n"/>
+      <x:c r="A50" s="6"/>
+      <x:c r="B50" s="23"/>
+      <x:c r="C50" s="23"/>
+      <x:c r="D50" s="23"/>
+      <x:c r="E50" s="23"/>
+      <x:c r="F50" s="23"/>
+      <x:c r="G50" s="23"/>
+      <x:c r="H50" s="23"/>
+      <x:c r="I50" s="23"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="6" t="n"/>
-      <x:c r="B51" s="23" t="n"/>
-      <x:c r="C51" s="23" t="n"/>
-      <x:c r="D51" s="23" t="n"/>
-      <x:c r="E51" s="23" t="n"/>
-      <x:c r="F51" s="23" t="n"/>
-      <x:c r="G51" s="23" t="n"/>
-      <x:c r="H51" s="23" t="n"/>
-      <x:c r="I51" s="23" t="n"/>
+      <x:c r="A51" s="6"/>
+      <x:c r="B51" s="23"/>
+      <x:c r="C51" s="23"/>
+      <x:c r="D51" s="23"/>
+      <x:c r="E51" s="23"/>
+      <x:c r="F51" s="23"/>
+      <x:c r="G51" s="23"/>
+      <x:c r="H51" s="23"/>
+      <x:c r="I51" s="23"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="6" t="n"/>
-      <x:c r="B52" s="23" t="n"/>
-      <x:c r="C52" s="23" t="n"/>
-      <x:c r="D52" s="23" t="n"/>
-      <x:c r="E52" s="23" t="n"/>
-      <x:c r="F52" s="23" t="n"/>
-      <x:c r="G52" s="23" t="n"/>
-      <x:c r="H52" s="23" t="n"/>
-      <x:c r="I52" s="23" t="n"/>
+      <x:c r="A52" s="6"/>
+      <x:c r="B52" s="23"/>
+      <x:c r="C52" s="23"/>
+      <x:c r="D52" s="23"/>
+      <x:c r="E52" s="23"/>
+      <x:c r="F52" s="23"/>
+      <x:c r="G52" s="23"/>
+      <x:c r="H52" s="23"/>
+      <x:c r="I52" s="23"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="6" t="n"/>
-      <x:c r="B53" s="23" t="n"/>
-      <x:c r="C53" s="23" t="n"/>
-      <x:c r="D53" s="23" t="n"/>
-      <x:c r="E53" s="23" t="n"/>
-      <x:c r="F53" s="23" t="n"/>
-      <x:c r="G53" s="23" t="n"/>
-      <x:c r="H53" s="23" t="n"/>
-      <x:c r="I53" s="23" t="n"/>
+      <x:c r="A53" s="6"/>
+      <x:c r="B53" s="23"/>
+      <x:c r="C53" s="23"/>
+      <x:c r="D53" s="23"/>
+      <x:c r="E53" s="23"/>
+      <x:c r="F53" s="23"/>
+      <x:c r="G53" s="23"/>
+      <x:c r="H53" s="23"/>
+      <x:c r="I53" s="23"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="6" t="n"/>
-      <x:c r="B54" s="23" t="n"/>
-      <x:c r="C54" s="23" t="n"/>
-      <x:c r="D54" s="23" t="n"/>
-      <x:c r="E54" s="23" t="n"/>
-      <x:c r="F54" s="23" t="n"/>
-      <x:c r="G54" s="23" t="n"/>
-      <x:c r="H54" s="23" t="n"/>
-      <x:c r="I54" s="23" t="n"/>
+      <x:c r="A54" s="6"/>
+      <x:c r="B54" s="23"/>
+      <x:c r="C54" s="23"/>
+      <x:c r="D54" s="23"/>
+      <x:c r="E54" s="23"/>
+      <x:c r="F54" s="23"/>
+      <x:c r="G54" s="23"/>
+      <x:c r="H54" s="23"/>
+      <x:c r="I54" s="23"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="6" t="n"/>
-      <x:c r="B55" s="23" t="n"/>
-      <x:c r="C55" s="23" t="n"/>
-      <x:c r="D55" s="23" t="n"/>
-      <x:c r="E55" s="23" t="n"/>
-      <x:c r="F55" s="23" t="n"/>
-      <x:c r="G55" s="23" t="n"/>
-      <x:c r="H55" s="23" t="n"/>
-      <x:c r="I55" s="23" t="n"/>
+      <x:c r="A55" s="6"/>
+      <x:c r="B55" s="23"/>
+      <x:c r="C55" s="23"/>
+      <x:c r="D55" s="23"/>
+      <x:c r="E55" s="23"/>
+      <x:c r="F55" s="23"/>
+      <x:c r="G55" s="23"/>
+      <x:c r="H55" s="23"/>
+      <x:c r="I55" s="23"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="6" t="n"/>
-      <x:c r="B56" s="23" t="n"/>
-      <x:c r="C56" s="23" t="n"/>
-      <x:c r="D56" s="23" t="n"/>
-      <x:c r="E56" s="23" t="n"/>
-      <x:c r="F56" s="23" t="n"/>
-      <x:c r="G56" s="23" t="n"/>
-      <x:c r="H56" s="23" t="n"/>
-      <x:c r="I56" s="23" t="n"/>
+      <x:c r="A56" s="6"/>
+      <x:c r="B56" s="23"/>
+      <x:c r="C56" s="23"/>
+      <x:c r="D56" s="23"/>
+      <x:c r="E56" s="23"/>
+      <x:c r="F56" s="23"/>
+      <x:c r="G56" s="23"/>
+      <x:c r="H56" s="23"/>
+      <x:c r="I56" s="23"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="6" t="n"/>
-      <x:c r="B57" s="23" t="n"/>
-      <x:c r="C57" s="23" t="n"/>
-      <x:c r="D57" s="23" t="n"/>
-      <x:c r="E57" s="23" t="n"/>
-      <x:c r="F57" s="23" t="n"/>
-      <x:c r="G57" s="23" t="n"/>
-      <x:c r="H57" s="23" t="n"/>
-      <x:c r="I57" s="23" t="n"/>
+      <x:c r="A57" s="6"/>
+      <x:c r="B57" s="23"/>
+      <x:c r="C57" s="23"/>
+      <x:c r="D57" s="23"/>
+      <x:c r="E57" s="23"/>
+      <x:c r="F57" s="23"/>
+      <x:c r="G57" s="23"/>
+      <x:c r="H57" s="23"/>
+      <x:c r="I57" s="23"/>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="6" t="n"/>
-      <x:c r="B58" s="23" t="n"/>
-      <x:c r="C58" s="23" t="n"/>
-      <x:c r="D58" s="23" t="n"/>
-      <x:c r="E58" s="23" t="n"/>
-      <x:c r="F58" s="23" t="n"/>
-      <x:c r="G58" s="23" t="n"/>
-      <x:c r="H58" s="23" t="n"/>
-      <x:c r="I58" s="23" t="n"/>
+      <x:c r="A58" s="6"/>
+      <x:c r="B58" s="23"/>
+      <x:c r="C58" s="23"/>
+      <x:c r="D58" s="23"/>
+      <x:c r="E58" s="23"/>
+      <x:c r="F58" s="23"/>
+      <x:c r="G58" s="23"/>
+      <x:c r="H58" s="23"/>
+      <x:c r="I58" s="23"/>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="6" t="n"/>
-      <x:c r="B59" s="23" t="n"/>
-      <x:c r="C59" s="23" t="n"/>
-      <x:c r="D59" s="23" t="n"/>
-      <x:c r="E59" s="23" t="n"/>
-      <x:c r="F59" s="23" t="n"/>
-      <x:c r="G59" s="23" t="n"/>
-      <x:c r="H59" s="23" t="n"/>
-      <x:c r="I59" s="23" t="n"/>
+      <x:c r="A59" s="6"/>
+      <x:c r="B59" s="23"/>
+      <x:c r="C59" s="23"/>
+      <x:c r="D59" s="23"/>
+      <x:c r="E59" s="23"/>
+      <x:c r="F59" s="23"/>
+      <x:c r="G59" s="23"/>
+      <x:c r="H59" s="23"/>
+      <x:c r="I59" s="23"/>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="6" t="n"/>
-      <x:c r="B60" s="23" t="n"/>
-      <x:c r="C60" s="23" t="n"/>
-      <x:c r="D60" s="23" t="n"/>
-      <x:c r="E60" s="23" t="n"/>
-      <x:c r="F60" s="23" t="n"/>
-      <x:c r="G60" s="23" t="n"/>
-      <x:c r="H60" s="23" t="n"/>
-      <x:c r="I60" s="23" t="n"/>
+      <x:c r="A60" s="6"/>
+      <x:c r="B60" s="23"/>
+      <x:c r="C60" s="23"/>
+      <x:c r="D60" s="23"/>
+      <x:c r="E60" s="23"/>
+      <x:c r="F60" s="23"/>
+      <x:c r="G60" s="23"/>
+      <x:c r="H60" s="23"/>
+      <x:c r="I60" s="23"/>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="6" t="n"/>
-      <x:c r="B61" s="23" t="n"/>
-      <x:c r="C61" s="23" t="n"/>
-      <x:c r="D61" s="23" t="n"/>
-      <x:c r="E61" s="23" t="n"/>
-      <x:c r="F61" s="23" t="n"/>
-      <x:c r="G61" s="23" t="n"/>
-      <x:c r="H61" s="23" t="n"/>
-      <x:c r="I61" s="23" t="n"/>
+      <x:c r="A61" s="6"/>
+      <x:c r="B61" s="23"/>
+      <x:c r="C61" s="23"/>
+      <x:c r="D61" s="23"/>
+      <x:c r="E61" s="23"/>
+      <x:c r="F61" s="23"/>
+      <x:c r="G61" s="23"/>
+      <x:c r="H61" s="23"/>
+      <x:c r="I61" s="23"/>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="6" t="n"/>
-      <x:c r="B62" s="23" t="n"/>
-      <x:c r="C62" s="23" t="n"/>
-      <x:c r="D62" s="23" t="n"/>
-      <x:c r="E62" s="23" t="n"/>
-      <x:c r="F62" s="23" t="n"/>
-      <x:c r="G62" s="23" t="n"/>
-      <x:c r="H62" s="23" t="n"/>
-      <x:c r="I62" s="23" t="n"/>
+      <x:c r="A62" s="6"/>
+      <x:c r="B62" s="23"/>
+      <x:c r="C62" s="23"/>
+      <x:c r="D62" s="23"/>
+      <x:c r="E62" s="23"/>
+      <x:c r="F62" s="23"/>
+      <x:c r="G62" s="23"/>
+      <x:c r="H62" s="23"/>
+      <x:c r="I62" s="23"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="6" t="n"/>
-      <x:c r="B63" s="23" t="n"/>
-      <x:c r="C63" s="23" t="n"/>
-      <x:c r="D63" s="23" t="n"/>
-      <x:c r="E63" s="23" t="n"/>
-      <x:c r="F63" s="23" t="n"/>
-      <x:c r="G63" s="23" t="n"/>
-      <x:c r="H63" s="23" t="n"/>
-      <x:c r="I63" s="23" t="n"/>
+      <x:c r="A63" s="6"/>
+      <x:c r="B63" s="23"/>
+      <x:c r="C63" s="23"/>
+      <x:c r="D63" s="23"/>
+      <x:c r="E63" s="23"/>
+      <x:c r="F63" s="23"/>
+      <x:c r="G63" s="23"/>
+      <x:c r="H63" s="23"/>
+      <x:c r="I63" s="23"/>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="6" t="n"/>
-      <x:c r="B64" s="23" t="n"/>
-      <x:c r="C64" s="23" t="n"/>
-      <x:c r="D64" s="23" t="n"/>
-      <x:c r="E64" s="23" t="n"/>
-      <x:c r="F64" s="23" t="n"/>
-      <x:c r="G64" s="23" t="n"/>
-      <x:c r="H64" s="23" t="n"/>
-      <x:c r="I64" s="23" t="n"/>
+      <x:c r="A64" s="6"/>
+      <x:c r="B64" s="23"/>
+      <x:c r="C64" s="23"/>
+      <x:c r="D64" s="23"/>
+      <x:c r="E64" s="23"/>
+      <x:c r="F64" s="23"/>
+      <x:c r="G64" s="23"/>
+      <x:c r="H64" s="23"/>
+      <x:c r="I64" s="23"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="6" t="n"/>
-      <x:c r="B65" s="23" t="n"/>
-      <x:c r="C65" s="23" t="n"/>
-      <x:c r="D65" s="23" t="n"/>
-      <x:c r="E65" s="23" t="n"/>
-      <x:c r="F65" s="23" t="n"/>
-      <x:c r="G65" s="23" t="n"/>
-      <x:c r="H65" s="23" t="n"/>
-      <x:c r="I65" s="23" t="n"/>
+      <x:c r="A65" s="6"/>
+      <x:c r="B65" s="23"/>
+      <x:c r="C65" s="23"/>
+      <x:c r="D65" s="23"/>
+      <x:c r="E65" s="23"/>
+      <x:c r="F65" s="23"/>
+      <x:c r="G65" s="23"/>
+      <x:c r="H65" s="23"/>
+      <x:c r="I65" s="23"/>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="6" t="n"/>
-      <x:c r="B66" s="23" t="n"/>
-      <x:c r="C66" s="23" t="n"/>
-      <x:c r="D66" s="23" t="n"/>
-      <x:c r="E66" s="23" t="n"/>
-      <x:c r="F66" s="23" t="n"/>
-      <x:c r="G66" s="23" t="n"/>
-      <x:c r="H66" s="23" t="n"/>
-      <x:c r="I66" s="23" t="n"/>
+      <x:c r="A66" s="6"/>
+      <x:c r="B66" s="23"/>
+      <x:c r="C66" s="23"/>
+      <x:c r="D66" s="23"/>
+      <x:c r="E66" s="23"/>
+      <x:c r="F66" s="23"/>
+      <x:c r="G66" s="23"/>
+      <x:c r="H66" s="23"/>
+      <x:c r="I66" s="23"/>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="6" t="n"/>
-      <x:c r="B67" s="23" t="n"/>
-      <x:c r="C67" s="23" t="n"/>
-      <x:c r="D67" s="23" t="n"/>
-      <x:c r="E67" s="23" t="n"/>
-      <x:c r="F67" s="23" t="n"/>
-      <x:c r="G67" s="23" t="n"/>
-      <x:c r="H67" s="23" t="n"/>
-      <x:c r="I67" s="23" t="n"/>
+      <x:c r="A67" s="6"/>
+      <x:c r="B67" s="23"/>
+      <x:c r="C67" s="23"/>
+      <x:c r="D67" s="23"/>
+      <x:c r="E67" s="23"/>
+      <x:c r="F67" s="23"/>
+      <x:c r="G67" s="23"/>
+      <x:c r="H67" s="23"/>
+      <x:c r="I67" s="23"/>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="6" t="n"/>
-      <x:c r="B68" s="23" t="n"/>
-      <x:c r="C68" s="23" t="n"/>
-      <x:c r="D68" s="23" t="n"/>
-      <x:c r="E68" s="23" t="n"/>
-      <x:c r="F68" s="23" t="n"/>
-      <x:c r="G68" s="23" t="n"/>
-      <x:c r="H68" s="23" t="n"/>
-      <x:c r="I68" s="23" t="n"/>
+      <x:c r="A68" s="6"/>
+      <x:c r="B68" s="23"/>
+      <x:c r="C68" s="23"/>
+      <x:c r="D68" s="23"/>
+      <x:c r="E68" s="23"/>
+      <x:c r="F68" s="23"/>
+      <x:c r="G68" s="23"/>
+      <x:c r="H68" s="23"/>
+      <x:c r="I68" s="23"/>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="6" t="n"/>
-      <x:c r="B69" s="23" t="n"/>
-      <x:c r="C69" s="23" t="n"/>
-      <x:c r="D69" s="23" t="n"/>
-      <x:c r="E69" s="23" t="n"/>
-      <x:c r="F69" s="23" t="n"/>
-      <x:c r="G69" s="23" t="n"/>
-      <x:c r="H69" s="23" t="n"/>
-      <x:c r="I69" s="23" t="n"/>
+      <x:c r="A69" s="6"/>
+      <x:c r="B69" s="23"/>
+      <x:c r="C69" s="23"/>
+      <x:c r="D69" s="23"/>
+      <x:c r="E69" s="23"/>
+      <x:c r="F69" s="23"/>
+      <x:c r="G69" s="23"/>
+      <x:c r="H69" s="23"/>
+      <x:c r="I69" s="23"/>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="6" t="n"/>
-      <x:c r="B70" s="23" t="n"/>
-      <x:c r="C70" s="23" t="n"/>
-      <x:c r="D70" s="23" t="n"/>
-      <x:c r="E70" s="23" t="n"/>
-      <x:c r="F70" s="23" t="n"/>
-      <x:c r="G70" s="23" t="n"/>
-      <x:c r="H70" s="23" t="n"/>
-      <x:c r="I70" s="23" t="n"/>
+      <x:c r="A70" s="6"/>
+      <x:c r="B70" s="23"/>
+      <x:c r="C70" s="23"/>
+      <x:c r="D70" s="23"/>
+      <x:c r="E70" s="23"/>
+      <x:c r="F70" s="23"/>
+      <x:c r="G70" s="23"/>
+      <x:c r="H70" s="23"/>
+      <x:c r="I70" s="23"/>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="6" t="n"/>
-      <x:c r="B71" s="23" t="n"/>
-      <x:c r="C71" s="23" t="n"/>
-      <x:c r="D71" s="23" t="n"/>
-      <x:c r="E71" s="23" t="n"/>
-      <x:c r="F71" s="23" t="n"/>
-      <x:c r="G71" s="23" t="n"/>
-      <x:c r="H71" s="23" t="n"/>
-      <x:c r="I71" s="23" t="n"/>
+      <x:c r="A71" s="6"/>
+      <x:c r="B71" s="23"/>
+      <x:c r="C71" s="23"/>
+      <x:c r="D71" s="23"/>
+      <x:c r="E71" s="23"/>
+      <x:c r="F71" s="23"/>
+      <x:c r="G71" s="23"/>
+      <x:c r="H71" s="23"/>
+      <x:c r="I71" s="23"/>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="6" t="n"/>
-      <x:c r="B72" s="23" t="n"/>
-      <x:c r="C72" s="23" t="n"/>
-      <x:c r="D72" s="23" t="n"/>
-      <x:c r="E72" s="23" t="n"/>
-      <x:c r="F72" s="23" t="n"/>
-      <x:c r="G72" s="23" t="n"/>
-      <x:c r="H72" s="23" t="n"/>
-      <x:c r="I72" s="23" t="n"/>
+      <x:c r="A72" s="6"/>
+      <x:c r="B72" s="23"/>
+      <x:c r="C72" s="23"/>
+      <x:c r="D72" s="23"/>
+      <x:c r="E72" s="23"/>
+      <x:c r="F72" s="23"/>
+      <x:c r="G72" s="23"/>
+      <x:c r="H72" s="23"/>
+      <x:c r="I72" s="23"/>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="6" t="n"/>
-      <x:c r="B73" s="23" t="n"/>
-      <x:c r="C73" s="23" t="n"/>
-      <x:c r="D73" s="23" t="n"/>
-      <x:c r="E73" s="23" t="n"/>
-      <x:c r="F73" s="23" t="n"/>
-      <x:c r="G73" s="23" t="n"/>
-      <x:c r="H73" s="23" t="n"/>
-      <x:c r="I73" s="23" t="n"/>
+      <x:c r="A73" s="6"/>
+      <x:c r="B73" s="23"/>
+      <x:c r="C73" s="23"/>
+      <x:c r="D73" s="23"/>
+      <x:c r="E73" s="23"/>
+      <x:c r="F73" s="23"/>
+      <x:c r="G73" s="23"/>
+      <x:c r="H73" s="23"/>
+      <x:c r="I73" s="23"/>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="6" t="n"/>
-      <x:c r="B74" s="23" t="n"/>
-      <x:c r="C74" s="23" t="n"/>
-      <x:c r="D74" s="23" t="n"/>
-      <x:c r="E74" s="23" t="n"/>
-      <x:c r="F74" s="23" t="n"/>
-      <x:c r="G74" s="23" t="n"/>
-      <x:c r="H74" s="23" t="n"/>
-      <x:c r="I74" s="23" t="n"/>
+      <x:c r="A74" s="6"/>
+      <x:c r="B74" s="23"/>
+      <x:c r="C74" s="23"/>
+      <x:c r="D74" s="23"/>
+      <x:c r="E74" s="23"/>
+      <x:c r="F74" s="23"/>
+      <x:c r="G74" s="23"/>
+      <x:c r="H74" s="23"/>
+      <x:c r="I74" s="23"/>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="6" t="n"/>
-      <x:c r="B75" s="23" t="n"/>
-      <x:c r="C75" s="23" t="n"/>
-      <x:c r="D75" s="23" t="n"/>
-      <x:c r="E75" s="23" t="n"/>
-      <x:c r="F75" s="23" t="n"/>
-      <x:c r="G75" s="23" t="n"/>
-      <x:c r="H75" s="23" t="n"/>
-      <x:c r="I75" s="23" t="n"/>
+      <x:c r="A75" s="6"/>
+      <x:c r="B75" s="23"/>
+      <x:c r="C75" s="23"/>
+      <x:c r="D75" s="23"/>
+      <x:c r="E75" s="23"/>
+      <x:c r="F75" s="23"/>
+      <x:c r="G75" s="23"/>
+      <x:c r="H75" s="23"/>
+      <x:c r="I75" s="23"/>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="6" t="n"/>
-      <x:c r="B76" s="23" t="n"/>
-      <x:c r="C76" s="23" t="n"/>
-      <x:c r="D76" s="23" t="n"/>
-      <x:c r="E76" s="23" t="n"/>
-      <x:c r="F76" s="23" t="n"/>
-      <x:c r="G76" s="23" t="n"/>
-      <x:c r="H76" s="23" t="n"/>
-      <x:c r="I76" s="23" t="n"/>
+      <x:c r="A76" s="6"/>
+      <x:c r="B76" s="23"/>
+      <x:c r="C76" s="23"/>
+      <x:c r="D76" s="23"/>
+      <x:c r="E76" s="23"/>
+      <x:c r="F76" s="23"/>
+      <x:c r="G76" s="23"/>
+      <x:c r="H76" s="23"/>
+      <x:c r="I76" s="23"/>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="6" t="n"/>
-      <x:c r="B77" s="23" t="n"/>
-      <x:c r="C77" s="23" t="n"/>
-      <x:c r="D77" s="23" t="n"/>
-      <x:c r="E77" s="23" t="n"/>
-      <x:c r="F77" s="23" t="n"/>
-      <x:c r="G77" s="23" t="n"/>
-      <x:c r="H77" s="23" t="n"/>
-      <x:c r="I77" s="23" t="n"/>
+      <x:c r="A77" s="6"/>
+      <x:c r="B77" s="23"/>
+      <x:c r="C77" s="23"/>
+      <x:c r="D77" s="23"/>
+      <x:c r="E77" s="23"/>
+      <x:c r="F77" s="23"/>
+      <x:c r="G77" s="23"/>
+      <x:c r="H77" s="23"/>
+      <x:c r="I77" s="23"/>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="6" t="n"/>
-      <x:c r="B78" s="23" t="n"/>
-      <x:c r="C78" s="23" t="n"/>
-      <x:c r="D78" s="23" t="n"/>
-      <x:c r="E78" s="23" t="n"/>
-      <x:c r="F78" s="23" t="n"/>
-      <x:c r="G78" s="23" t="n"/>
-      <x:c r="H78" s="23" t="n"/>
-      <x:c r="I78" s="23" t="n"/>
+      <x:c r="A78" s="6"/>
+      <x:c r="B78" s="23"/>
+      <x:c r="C78" s="23"/>
+      <x:c r="D78" s="23"/>
+      <x:c r="E78" s="23"/>
+      <x:c r="F78" s="23"/>
+      <x:c r="G78" s="23"/>
+      <x:c r="H78" s="23"/>
+      <x:c r="I78" s="23"/>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="6" t="n"/>
-      <x:c r="B79" s="23" t="n"/>
-      <x:c r="C79" s="23" t="n"/>
-      <x:c r="D79" s="23" t="n"/>
-      <x:c r="E79" s="23" t="n"/>
-      <x:c r="F79" s="23" t="n"/>
-      <x:c r="G79" s="23" t="n"/>
-      <x:c r="H79" s="23" t="n"/>
-      <x:c r="I79" s="23" t="n"/>
+      <x:c r="A79" s="6"/>
+      <x:c r="B79" s="23"/>
+      <x:c r="C79" s="23"/>
+      <x:c r="D79" s="23"/>
+      <x:c r="E79" s="23"/>
+      <x:c r="F79" s="23"/>
+      <x:c r="G79" s="23"/>
+      <x:c r="H79" s="23"/>
+      <x:c r="I79" s="23"/>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="6" t="n"/>
-      <x:c r="B80" s="23" t="n"/>
-      <x:c r="C80" s="23" t="n"/>
-      <x:c r="D80" s="23" t="n"/>
-      <x:c r="E80" s="23" t="n"/>
-      <x:c r="F80" s="23" t="n"/>
-      <x:c r="G80" s="23" t="n"/>
-      <x:c r="H80" s="23" t="n"/>
-      <x:c r="I80" s="23" t="n"/>
+      <x:c r="A80" s="6"/>
+      <x:c r="B80" s="23"/>
+      <x:c r="C80" s="23"/>
+      <x:c r="D80" s="23"/>
+      <x:c r="E80" s="23"/>
+      <x:c r="F80" s="23"/>
+      <x:c r="G80" s="23"/>
+      <x:c r="H80" s="23"/>
+      <x:c r="I80" s="23"/>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="6" t="n"/>
-      <x:c r="B81" s="23" t="n"/>
-      <x:c r="C81" s="23" t="n"/>
-      <x:c r="D81" s="23" t="n"/>
-      <x:c r="E81" s="23" t="n"/>
-      <x:c r="F81" s="23" t="n"/>
-      <x:c r="G81" s="23" t="n"/>
-      <x:c r="H81" s="23" t="n"/>
-      <x:c r="I81" s="23" t="n"/>
+      <x:c r="A81" s="6"/>
+      <x:c r="B81" s="23"/>
+      <x:c r="C81" s="23"/>
+      <x:c r="D81" s="23"/>
+      <x:c r="E81" s="23"/>
+      <x:c r="F81" s="23"/>
+      <x:c r="G81" s="23"/>
+      <x:c r="H81" s="23"/>
+      <x:c r="I81" s="23"/>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="6" t="n"/>
-      <x:c r="B82" s="23" t="n"/>
-      <x:c r="C82" s="23" t="n"/>
-      <x:c r="D82" s="23" t="n"/>
-      <x:c r="E82" s="23" t="n"/>
-      <x:c r="F82" s="23" t="n"/>
-      <x:c r="G82" s="23" t="n"/>
-      <x:c r="H82" s="23" t="n"/>
-      <x:c r="I82" s="23" t="n"/>
+      <x:c r="A82" s="6"/>
+      <x:c r="B82" s="23"/>
+      <x:c r="C82" s="23"/>
+      <x:c r="D82" s="23"/>
+      <x:c r="E82" s="23"/>
+      <x:c r="F82" s="23"/>
+      <x:c r="G82" s="23"/>
+      <x:c r="H82" s="23"/>
+      <x:c r="I82" s="23"/>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="6" t="n"/>
-      <x:c r="B83" s="23" t="n"/>
-      <x:c r="C83" s="23" t="n"/>
-      <x:c r="D83" s="23" t="n"/>
-      <x:c r="E83" s="23" t="n"/>
-      <x:c r="F83" s="23" t="n"/>
-      <x:c r="G83" s="23" t="n"/>
-      <x:c r="H83" s="23" t="n"/>
-      <x:c r="I83" s="23" t="n"/>
+      <x:c r="A83" s="6"/>
+      <x:c r="B83" s="23"/>
+      <x:c r="C83" s="23"/>
+      <x:c r="D83" s="23"/>
+      <x:c r="E83" s="23"/>
+      <x:c r="F83" s="23"/>
+      <x:c r="G83" s="23"/>
+      <x:c r="H83" s="23"/>
+      <x:c r="I83" s="23"/>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="6" t="n"/>
-      <x:c r="B84" s="23" t="n"/>
-      <x:c r="C84" s="23" t="n"/>
-      <x:c r="D84" s="23" t="n"/>
-      <x:c r="E84" s="23" t="n"/>
-      <x:c r="F84" s="23" t="n"/>
-      <x:c r="G84" s="23" t="n"/>
-      <x:c r="H84" s="23" t="n"/>
-      <x:c r="I84" s="23" t="n"/>
+      <x:c r="A84" s="6"/>
+      <x:c r="B84" s="23"/>
+      <x:c r="C84" s="23"/>
+      <x:c r="D84" s="23"/>
+      <x:c r="E84" s="23"/>
+      <x:c r="F84" s="23"/>
+      <x:c r="G84" s="23"/>
+      <x:c r="H84" s="23"/>
+      <x:c r="I84" s="23"/>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="6" t="n"/>
-      <x:c r="B85" s="23" t="n"/>
-      <x:c r="C85" s="23" t="n"/>
-      <x:c r="D85" s="23" t="n"/>
-      <x:c r="E85" s="23" t="n"/>
-      <x:c r="F85" s="23" t="n"/>
-      <x:c r="G85" s="23" t="n"/>
-      <x:c r="H85" s="23" t="n"/>
-      <x:c r="I85" s="23" t="n"/>
+      <x:c r="A85" s="6"/>
+      <x:c r="B85" s="23"/>
+      <x:c r="C85" s="23"/>
+      <x:c r="D85" s="23"/>
+      <x:c r="E85" s="23"/>
+      <x:c r="F85" s="23"/>
+      <x:c r="G85" s="23"/>
+      <x:c r="H85" s="23"/>
+      <x:c r="I85" s="23"/>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="6" t="n"/>
-      <x:c r="B86" s="23" t="n"/>
-      <x:c r="C86" s="23" t="n"/>
-      <x:c r="D86" s="23" t="n"/>
-      <x:c r="E86" s="23" t="n"/>
-      <x:c r="F86" s="23" t="n"/>
-      <x:c r="G86" s="23" t="n"/>
-      <x:c r="H86" s="23" t="n"/>
-      <x:c r="I86" s="23" t="n"/>
+      <x:c r="A86" s="6"/>
+      <x:c r="B86" s="23"/>
+      <x:c r="C86" s="23"/>
+      <x:c r="D86" s="23"/>
+      <x:c r="E86" s="23"/>
+      <x:c r="F86" s="23"/>
+      <x:c r="G86" s="23"/>
+      <x:c r="H86" s="23"/>
+      <x:c r="I86" s="23"/>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="6" t="n"/>
-      <x:c r="B87" s="23" t="n"/>
-      <x:c r="C87" s="23" t="n"/>
-      <x:c r="D87" s="23" t="n"/>
-      <x:c r="E87" s="23" t="n"/>
-      <x:c r="F87" s="23" t="n"/>
-      <x:c r="G87" s="23" t="n"/>
-      <x:c r="H87" s="23" t="n"/>
-      <x:c r="I87" s="23" t="n"/>
+      <x:c r="A87" s="6"/>
+      <x:c r="B87" s="23"/>
+      <x:c r="C87" s="23"/>
+      <x:c r="D87" s="23"/>
+      <x:c r="E87" s="23"/>
+      <x:c r="F87" s="23"/>
+      <x:c r="G87" s="23"/>
+      <x:c r="H87" s="23"/>
+      <x:c r="I87" s="23"/>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="6" t="n"/>
-      <x:c r="B88" s="23" t="n"/>
-      <x:c r="C88" s="23" t="n"/>
-      <x:c r="D88" s="23" t="n"/>
-      <x:c r="E88" s="23" t="n"/>
-      <x:c r="F88" s="23" t="n"/>
-      <x:c r="G88" s="23" t="n"/>
-      <x:c r="H88" s="23" t="n"/>
-      <x:c r="I88" s="23" t="n"/>
+      <x:c r="A88" s="6"/>
+      <x:c r="B88" s="23"/>
+      <x:c r="C88" s="23"/>
+      <x:c r="D88" s="23"/>
+      <x:c r="E88" s="23"/>
+      <x:c r="F88" s="23"/>
+      <x:c r="G88" s="23"/>
+      <x:c r="H88" s="23"/>
+      <x:c r="I88" s="23"/>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="6" t="n"/>
-      <x:c r="B89" s="23" t="n"/>
-      <x:c r="C89" s="23" t="n"/>
-      <x:c r="D89" s="23" t="n"/>
-      <x:c r="E89" s="23" t="n"/>
-      <x:c r="F89" s="23" t="n"/>
-      <x:c r="G89" s="23" t="n"/>
-      <x:c r="H89" s="23" t="n"/>
-      <x:c r="I89" s="23" t="n"/>
+      <x:c r="A89" s="6"/>
+      <x:c r="B89" s="23"/>
+      <x:c r="C89" s="23"/>
+      <x:c r="D89" s="23"/>
+      <x:c r="E89" s="23"/>
+      <x:c r="F89" s="23"/>
+      <x:c r="G89" s="23"/>
+      <x:c r="H89" s="23"/>
+      <x:c r="I89" s="23"/>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="6" t="n"/>
-      <x:c r="B90" s="23" t="n"/>
-      <x:c r="C90" s="23" t="n"/>
-      <x:c r="D90" s="23" t="n"/>
-      <x:c r="E90" s="23" t="n"/>
-      <x:c r="F90" s="23" t="n"/>
-      <x:c r="G90" s="23" t="n"/>
-      <x:c r="H90" s="23" t="n"/>
-      <x:c r="I90" s="23" t="n"/>
+      <x:c r="A90" s="6"/>
+      <x:c r="B90" s="23"/>
+      <x:c r="C90" s="23"/>
+      <x:c r="D90" s="23"/>
+      <x:c r="E90" s="23"/>
+      <x:c r="F90" s="23"/>
+      <x:c r="G90" s="23"/>
+      <x:c r="H90" s="23"/>
+      <x:c r="I90" s="23"/>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="6" t="n"/>
-      <x:c r="B91" s="23" t="n"/>
-      <x:c r="C91" s="23" t="n"/>
-      <x:c r="D91" s="23" t="n"/>
-      <x:c r="E91" s="23" t="n"/>
-      <x:c r="F91" s="23" t="n"/>
-      <x:c r="G91" s="23" t="n"/>
-      <x:c r="H91" s="23" t="n"/>
-      <x:c r="I91" s="23" t="n"/>
+      <x:c r="A91" s="6"/>
+      <x:c r="B91" s="23"/>
+      <x:c r="C91" s="23"/>
+      <x:c r="D91" s="23"/>
+      <x:c r="E91" s="23"/>
+      <x:c r="F91" s="23"/>
+      <x:c r="G91" s="23"/>
+      <x:c r="H91" s="23"/>
+      <x:c r="I91" s="23"/>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="6" t="n"/>
-      <x:c r="B92" s="23" t="n"/>
-      <x:c r="C92" s="23" t="n"/>
-      <x:c r="D92" s="23" t="n"/>
-      <x:c r="E92" s="23" t="n"/>
-      <x:c r="F92" s="23" t="n"/>
-      <x:c r="G92" s="23" t="n"/>
-      <x:c r="H92" s="23" t="n"/>
-      <x:c r="I92" s="23" t="n"/>
+      <x:c r="A92" s="6"/>
+      <x:c r="B92" s="23"/>
+      <x:c r="C92" s="23"/>
+      <x:c r="D92" s="23"/>
+      <x:c r="E92" s="23"/>
+      <x:c r="F92" s="23"/>
+      <x:c r="G92" s="23"/>
+      <x:c r="H92" s="23"/>
+      <x:c r="I92" s="23"/>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" s="6" t="n"/>
-      <x:c r="B93" s="23" t="n"/>
-      <x:c r="C93" s="23" t="n"/>
-      <x:c r="D93" s="23" t="n"/>
-      <x:c r="E93" s="23" t="n"/>
-      <x:c r="F93" s="23" t="n"/>
-      <x:c r="G93" s="23" t="n"/>
-      <x:c r="H93" s="23" t="n"/>
-      <x:c r="I93" s="23" t="n"/>
+      <x:c r="A93" s="6"/>
+      <x:c r="B93" s="23"/>
+      <x:c r="C93" s="23"/>
+      <x:c r="D93" s="23"/>
+      <x:c r="E93" s="23"/>
+      <x:c r="F93" s="23"/>
+      <x:c r="G93" s="23"/>
+      <x:c r="H93" s="23"/>
+      <x:c r="I93" s="23"/>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" s="6" t="n"/>
-      <x:c r="B94" s="23" t="n"/>
-      <x:c r="C94" s="23" t="n"/>
-      <x:c r="D94" s="23" t="n"/>
-      <x:c r="E94" s="23" t="n"/>
-      <x:c r="F94" s="23" t="n"/>
-      <x:c r="G94" s="23" t="n"/>
-      <x:c r="H94" s="23" t="n"/>
-      <x:c r="I94" s="23" t="n"/>
+      <x:c r="A94" s="6"/>
+      <x:c r="B94" s="23"/>
+      <x:c r="C94" s="23"/>
+      <x:c r="D94" s="23"/>
+      <x:c r="E94" s="23"/>
+      <x:c r="F94" s="23"/>
+      <x:c r="G94" s="23"/>
+      <x:c r="H94" s="23"/>
+      <x:c r="I94" s="23"/>
     </x:row>
     <x:row r="95">
-      <x:c r="A95" s="6" t="n"/>
-      <x:c r="B95" s="23" t="n"/>
-      <x:c r="C95" s="23" t="n"/>
-      <x:c r="D95" s="23" t="n"/>
-      <x:c r="E95" s="23" t="n"/>
-      <x:c r="F95" s="23" t="n"/>
-      <x:c r="G95" s="23" t="n"/>
-      <x:c r="H95" s="23" t="n"/>
-      <x:c r="I95" s="23" t="n"/>
+      <x:c r="A95" s="6"/>
+      <x:c r="B95" s="23"/>
+      <x:c r="C95" s="23"/>
+      <x:c r="D95" s="23"/>
+      <x:c r="E95" s="23"/>
+      <x:c r="F95" s="23"/>
+      <x:c r="G95" s="23"/>
+      <x:c r="H95" s="23"/>
+      <x:c r="I95" s="23"/>
     </x:row>
     <x:row r="96">
-      <x:c r="A96" s="6" t="n"/>
-      <x:c r="B96" s="23" t="n"/>
-      <x:c r="C96" s="23" t="n"/>
-      <x:c r="D96" s="23" t="n"/>
-      <x:c r="E96" s="23" t="n"/>
-      <x:c r="F96" s="23" t="n"/>
-      <x:c r="G96" s="23" t="n"/>
-      <x:c r="H96" s="23" t="n"/>
-      <x:c r="I96" s="23" t="n"/>
+      <x:c r="A96" s="6"/>
+      <x:c r="B96" s="23"/>
+      <x:c r="C96" s="23"/>
+      <x:c r="D96" s="23"/>
+      <x:c r="E96" s="23"/>
+      <x:c r="F96" s="23"/>
+      <x:c r="G96" s="23"/>
+      <x:c r="H96" s="23"/>
+      <x:c r="I96" s="23"/>
     </x:row>
     <x:row r="97">
-      <x:c r="A97" s="6" t="n"/>
-      <x:c r="B97" s="23" t="n"/>
-      <x:c r="C97" s="23" t="n"/>
-      <x:c r="D97" s="23" t="n"/>
-      <x:c r="E97" s="23" t="n"/>
-      <x:c r="F97" s="23" t="n"/>
-      <x:c r="G97" s="23" t="n"/>
-      <x:c r="H97" s="23" t="n"/>
-      <x:c r="I97" s="23" t="n"/>
+      <x:c r="A97" s="6"/>
+      <x:c r="B97" s="23"/>
+      <x:c r="C97" s="23"/>
+      <x:c r="D97" s="23"/>
+      <x:c r="E97" s="23"/>
+      <x:c r="F97" s="23"/>
+      <x:c r="G97" s="23"/>
+      <x:c r="H97" s="23"/>
+      <x:c r="I97" s="23"/>
     </x:row>
     <x:row r="98">
-      <x:c r="A98" s="6" t="n"/>
-      <x:c r="B98" s="23" t="n"/>
-      <x:c r="C98" s="23" t="n"/>
-      <x:c r="D98" s="23" t="n"/>
-      <x:c r="E98" s="23" t="n"/>
-      <x:c r="F98" s="23" t="n"/>
-      <x:c r="G98" s="23" t="n"/>
-      <x:c r="H98" s="23" t="n"/>
-      <x:c r="I98" s="23" t="n"/>
+      <x:c r="A98" s="6"/>
+      <x:c r="B98" s="23"/>
+      <x:c r="C98" s="23"/>
+      <x:c r="D98" s="23"/>
+      <x:c r="E98" s="23"/>
+      <x:c r="F98" s="23"/>
+      <x:c r="G98" s="23"/>
+      <x:c r="H98" s="23"/>
+      <x:c r="I98" s="23"/>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="6" t="n"/>
-      <x:c r="B99" s="23" t="n"/>
-      <x:c r="C99" s="23" t="n"/>
-      <x:c r="D99" s="23" t="n"/>
-      <x:c r="E99" s="23" t="n"/>
-      <x:c r="F99" s="23" t="n"/>
-      <x:c r="G99" s="23" t="n"/>
-      <x:c r="H99" s="23" t="n"/>
-      <x:c r="I99" s="23" t="n"/>
+      <x:c r="A99" s="6"/>
+      <x:c r="B99" s="23"/>
+      <x:c r="C99" s="23"/>
+      <x:c r="D99" s="23"/>
+      <x:c r="E99" s="23"/>
+      <x:c r="F99" s="23"/>
+      <x:c r="G99" s="23"/>
+      <x:c r="H99" s="23"/>
+      <x:c r="I99" s="23"/>
     </x:row>
     <x:row r="100">
-      <x:c r="A100" s="6" t="n"/>
-      <x:c r="B100" s="23" t="n"/>
-      <x:c r="C100" s="23" t="n"/>
-      <x:c r="D100" s="23" t="n"/>
-      <x:c r="E100" s="23" t="n"/>
-      <x:c r="F100" s="23" t="n"/>
-      <x:c r="G100" s="23" t="n"/>
-      <x:c r="H100" s="23" t="n"/>
-      <x:c r="I100" s="23" t="n"/>
+      <x:c r="A100" s="6"/>
+      <x:c r="B100" s="23"/>
+      <x:c r="C100" s="23"/>
+      <x:c r="D100" s="23"/>
+      <x:c r="E100" s="23"/>
+      <x:c r="F100" s="23"/>
+      <x:c r="G100" s="23"/>
+      <x:c r="H100" s="23"/>
+      <x:c r="I100" s="23"/>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="6" t="n"/>
-      <x:c r="B101" s="23" t="n"/>
-      <x:c r="C101" s="23" t="n"/>
-      <x:c r="D101" s="23" t="n"/>
-      <x:c r="E101" s="23" t="n"/>
-      <x:c r="F101" s="23" t="n"/>
-      <x:c r="G101" s="23" t="n"/>
-      <x:c r="H101" s="23" t="n"/>
-      <x:c r="I101" s="23" t="n"/>
+      <x:c r="A101" s="6"/>
+      <x:c r="B101" s="23"/>
+      <x:c r="C101" s="23"/>
+      <x:c r="D101" s="23"/>
+      <x:c r="E101" s="23"/>
+      <x:c r="F101" s="23"/>
+      <x:c r="G101" s="23"/>
+      <x:c r="H101" s="23"/>
+      <x:c r="I101" s="23"/>
     </x:row>
     <x:row r="102">
-      <x:c r="A102" s="6" t="n"/>
-      <x:c r="B102" s="23" t="n"/>
-      <x:c r="C102" s="23" t="n"/>
-      <x:c r="D102" s="23" t="n"/>
-      <x:c r="E102" s="23" t="n"/>
-      <x:c r="F102" s="23" t="n"/>
-      <x:c r="G102" s="23" t="n"/>
-      <x:c r="H102" s="23" t="n"/>
-      <x:c r="I102" s="23" t="n"/>
+      <x:c r="A102" s="6"/>
+      <x:c r="B102" s="23"/>
+      <x:c r="C102" s="23"/>
+      <x:c r="D102" s="23"/>
+      <x:c r="E102" s="23"/>
+      <x:c r="F102" s="23"/>
+      <x:c r="G102" s="23"/>
+      <x:c r="H102" s="23"/>
+      <x:c r="I102" s="23"/>
     </x:row>
     <x:row r="103">
-      <x:c r="A103" s="6" t="n"/>
-      <x:c r="B103" s="23" t="n"/>
-      <x:c r="C103" s="23" t="n"/>
-      <x:c r="D103" s="23" t="n"/>
-      <x:c r="E103" s="23" t="n"/>
-      <x:c r="F103" s="23" t="n"/>
-      <x:c r="G103" s="23" t="n"/>
-      <x:c r="H103" s="23" t="n"/>
-      <x:c r="I103" s="23" t="n"/>
+      <x:c r="A103" s="6"/>
+      <x:c r="B103" s="23"/>
+      <x:c r="C103" s="23"/>
+      <x:c r="D103" s="23"/>
+      <x:c r="E103" s="23"/>
+      <x:c r="F103" s="23"/>
+      <x:c r="G103" s="23"/>
+      <x:c r="H103" s="23"/>
+      <x:c r="I103" s="23"/>
     </x:row>
     <x:row r="104">
-      <x:c r="A104" s="6" t="n"/>
-      <x:c r="B104" s="23" t="n"/>
-      <x:c r="C104" s="23" t="n"/>
-      <x:c r="D104" s="23" t="n"/>
-      <x:c r="E104" s="23" t="n"/>
-      <x:c r="F104" s="23" t="n"/>
-      <x:c r="G104" s="23" t="n"/>
-      <x:c r="H104" s="23" t="n"/>
-      <x:c r="I104" s="23" t="n"/>
+      <x:c r="A104" s="6"/>
+      <x:c r="B104" s="23"/>
+      <x:c r="C104" s="23"/>
+      <x:c r="D104" s="23"/>
+      <x:c r="E104" s="23"/>
+      <x:c r="F104" s="23"/>
+      <x:c r="G104" s="23"/>
+      <x:c r="H104" s="23"/>
+      <x:c r="I104" s="23"/>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="6" t="n"/>
-      <x:c r="B105" s="23" t="n"/>
-      <x:c r="C105" s="23" t="n"/>
-      <x:c r="D105" s="23" t="n"/>
-      <x:c r="E105" s="23" t="n"/>
-      <x:c r="F105" s="23" t="n"/>
-      <x:c r="G105" s="23" t="n"/>
-      <x:c r="H105" s="23" t="n"/>
-      <x:c r="I105" s="23" t="n"/>
+      <x:c r="A105" s="6"/>
+      <x:c r="B105" s="23"/>
+      <x:c r="C105" s="23"/>
+      <x:c r="D105" s="23"/>
+      <x:c r="E105" s="23"/>
+      <x:c r="F105" s="23"/>
+      <x:c r="G105" s="23"/>
+      <x:c r="H105" s="23"/>
+      <x:c r="I105" s="23"/>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="6" t="n"/>
-      <x:c r="B106" s="23" t="n"/>
-      <x:c r="C106" s="23" t="n"/>
-      <x:c r="D106" s="23" t="n"/>
-      <x:c r="E106" s="23" t="n"/>
-      <x:c r="F106" s="23" t="n"/>
-      <x:c r="G106" s="23" t="n"/>
-      <x:c r="H106" s="23" t="n"/>
-      <x:c r="I106" s="23" t="n"/>
+      <x:c r="A106" s="6"/>
+      <x:c r="B106" s="23"/>
+      <x:c r="C106" s="23"/>
+      <x:c r="D106" s="23"/>
+      <x:c r="E106" s="23"/>
+      <x:c r="F106" s="23"/>
+      <x:c r="G106" s="23"/>
+      <x:c r="H106" s="23"/>
+      <x:c r="I106" s="23"/>
     </x:row>
     <x:row r="107">
-      <x:c r="A107" s="6" t="n"/>
-      <x:c r="B107" s="23" t="n"/>
-      <x:c r="C107" s="23" t="n"/>
-      <x:c r="D107" s="23" t="n"/>
-      <x:c r="E107" s="23" t="n"/>
-      <x:c r="F107" s="23" t="n"/>
-      <x:c r="G107" s="23" t="n"/>
-      <x:c r="H107" s="23" t="n"/>
-      <x:c r="I107" s="23" t="n"/>
+      <x:c r="A107" s="6"/>
+      <x:c r="B107" s="23"/>
+      <x:c r="C107" s="23"/>
+      <x:c r="D107" s="23"/>
+      <x:c r="E107" s="23"/>
+      <x:c r="F107" s="23"/>
+      <x:c r="G107" s="23"/>
+      <x:c r="H107" s="23"/>
+      <x:c r="I107" s="23"/>
     </x:row>
     <x:row r="108">
-      <x:c r="A108" s="6" t="n"/>
-      <x:c r="B108" s="23" t="n"/>
-      <x:c r="C108" s="23" t="n"/>
-      <x:c r="D108" s="23" t="n"/>
-      <x:c r="E108" s="23" t="n"/>
-      <x:c r="F108" s="23" t="n"/>
-      <x:c r="G108" s="23" t="n"/>
-      <x:c r="H108" s="23" t="n"/>
-      <x:c r="I108" s="23" t="n"/>
+      <x:c r="A108" s="6"/>
+      <x:c r="B108" s="23"/>
+      <x:c r="C108" s="23"/>
+      <x:c r="D108" s="23"/>
+      <x:c r="E108" s="23"/>
+      <x:c r="F108" s="23"/>
+      <x:c r="G108" s="23"/>
+      <x:c r="H108" s="23"/>
+      <x:c r="I108" s="23"/>
     </x:row>
     <x:row r="109">
-      <x:c r="A109" s="6" t="n"/>
-      <x:c r="B109" s="23" t="n"/>
-      <x:c r="C109" s="23" t="n"/>
-      <x:c r="D109" s="23" t="n"/>
-      <x:c r="E109" s="23" t="n"/>
-      <x:c r="F109" s="23" t="n"/>
-      <x:c r="G109" s="23" t="n"/>
-      <x:c r="H109" s="23" t="n"/>
-      <x:c r="I109" s="23" t="n"/>
+      <x:c r="A109" s="6"/>
+      <x:c r="B109" s="23"/>
+      <x:c r="C109" s="23"/>
+      <x:c r="D109" s="23"/>
+      <x:c r="E109" s="23"/>
+      <x:c r="F109" s="23"/>
+      <x:c r="G109" s="23"/>
+      <x:c r="H109" s="23"/>
+      <x:c r="I109" s="23"/>
     </x:row>
     <x:row r="110">
-      <x:c r="A110" s="6" t="n"/>
-      <x:c r="B110" s="23" t="n"/>
-      <x:c r="C110" s="23" t="n"/>
-      <x:c r="D110" s="23" t="n"/>
-      <x:c r="E110" s="23" t="n"/>
-      <x:c r="F110" s="23" t="n"/>
-      <x:c r="G110" s="23" t="n"/>
-      <x:c r="H110" s="23" t="n"/>
-      <x:c r="I110" s="23" t="n"/>
+      <x:c r="A110" s="6"/>
+      <x:c r="B110" s="23"/>
+      <x:c r="C110" s="23"/>
+      <x:c r="D110" s="23"/>
+      <x:c r="E110" s="23"/>
+      <x:c r="F110" s="23"/>
+      <x:c r="G110" s="23"/>
+      <x:c r="H110" s="23"/>
+      <x:c r="I110" s="23"/>
     </x:row>
     <x:row r="111">
-      <x:c r="A111" s="6" t="n"/>
-      <x:c r="B111" s="23" t="n"/>
-      <x:c r="C111" s="23" t="n"/>
-      <x:c r="D111" s="23" t="n"/>
-      <x:c r="E111" s="23" t="n"/>
-      <x:c r="F111" s="23" t="n"/>
-      <x:c r="G111" s="23" t="n"/>
-      <x:c r="H111" s="23" t="n"/>
-      <x:c r="I111" s="23" t="n"/>
+      <x:c r="A111" s="6"/>
+      <x:c r="B111" s="23"/>
+      <x:c r="C111" s="23"/>
+      <x:c r="D111" s="23"/>
+      <x:c r="E111" s="23"/>
+      <x:c r="F111" s="23"/>
+      <x:c r="G111" s="23"/>
+      <x:c r="H111" s="23"/>
+      <x:c r="I111" s="23"/>
     </x:row>
     <x:row r="112">
-      <x:c r="A112" s="6" t="n"/>
-      <x:c r="B112" s="23" t="n"/>
-      <x:c r="C112" s="23" t="n"/>
-      <x:c r="D112" s="23" t="n"/>
-      <x:c r="E112" s="23" t="n"/>
-      <x:c r="F112" s="23" t="n"/>
-      <x:c r="G112" s="23" t="n"/>
-      <x:c r="H112" s="23" t="n"/>
-      <x:c r="I112" s="23" t="n"/>
+      <x:c r="A112" s="6"/>
+      <x:c r="B112" s="23"/>
+      <x:c r="C112" s="23"/>
+      <x:c r="D112" s="23"/>
+      <x:c r="E112" s="23"/>
+      <x:c r="F112" s="23"/>
+      <x:c r="G112" s="23"/>
+      <x:c r="H112" s="23"/>
+      <x:c r="I112" s="23"/>
     </x:row>
     <x:row r="113">
-      <x:c r="A113" s="6" t="n"/>
-      <x:c r="B113" s="23" t="n"/>
-      <x:c r="C113" s="23" t="n"/>
-      <x:c r="D113" s="23" t="n"/>
-      <x:c r="E113" s="23" t="n"/>
-      <x:c r="F113" s="23" t="n"/>
-      <x:c r="G113" s="23" t="n"/>
-      <x:c r="H113" s="23" t="n"/>
-      <x:c r="I113" s="23" t="n"/>
+      <x:c r="A113" s="6"/>
+      <x:c r="B113" s="23"/>
+      <x:c r="C113" s="23"/>
+      <x:c r="D113" s="23"/>
+      <x:c r="E113" s="23"/>
+      <x:c r="F113" s="23"/>
+      <x:c r="G113" s="23"/>
+      <x:c r="H113" s="23"/>
+      <x:c r="I113" s="23"/>
     </x:row>
     <x:row r="114">
-      <x:c r="A114" s="6" t="n"/>
-      <x:c r="B114" s="23" t="n"/>
-      <x:c r="C114" s="23" t="n"/>
-      <x:c r="D114" s="23" t="n"/>
-      <x:c r="E114" s="23" t="n"/>
-      <x:c r="F114" s="23" t="n"/>
-      <x:c r="G114" s="23" t="n"/>
-      <x:c r="H114" s="23" t="n"/>
-      <x:c r="I114" s="23" t="n"/>
+      <x:c r="A114" s="6"/>
+      <x:c r="B114" s="23"/>
+      <x:c r="C114" s="23"/>
+      <x:c r="D114" s="23"/>
+      <x:c r="E114" s="23"/>
+      <x:c r="F114" s="23"/>
+      <x:c r="G114" s="23"/>
+      <x:c r="H114" s="23"/>
+      <x:c r="I114" s="23"/>
     </x:row>
     <x:row r="115">
-      <x:c r="A115" s="6" t="n"/>
-      <x:c r="B115" s="23" t="n"/>
-      <x:c r="C115" s="23" t="n"/>
-      <x:c r="D115" s="23" t="n"/>
-      <x:c r="E115" s="23" t="n"/>
-      <x:c r="F115" s="23" t="n"/>
-      <x:c r="G115" s="23" t="n"/>
-      <x:c r="H115" s="23" t="n"/>
-      <x:c r="I115" s="23" t="n"/>
+      <x:c r="A115" s="6"/>
+      <x:c r="B115" s="23"/>
+      <x:c r="C115" s="23"/>
+      <x:c r="D115" s="23"/>
+      <x:c r="E115" s="23"/>
+      <x:c r="F115" s="23"/>
+      <x:c r="G115" s="23"/>
+      <x:c r="H115" s="23"/>
+      <x:c r="I115" s="23"/>
     </x:row>
     <x:row r="116">
-      <x:c r="A116" s="6" t="n"/>
-      <x:c r="B116" s="23" t="n"/>
-      <x:c r="C116" s="23" t="n"/>
-      <x:c r="D116" s="23" t="n"/>
-      <x:c r="E116" s="23" t="n"/>
-      <x:c r="F116" s="23" t="n"/>
-      <x:c r="G116" s="23" t="n"/>
-      <x:c r="H116" s="23" t="n"/>
-      <x:c r="I116" s="23" t="n"/>
+      <x:c r="A116" s="6"/>
+      <x:c r="B116" s="23"/>
+      <x:c r="C116" s="23"/>
+      <x:c r="D116" s="23"/>
+      <x:c r="E116" s="23"/>
+      <x:c r="F116" s="23"/>
+      <x:c r="G116" s="23"/>
+      <x:c r="H116" s="23"/>
+      <x:c r="I116" s="23"/>
     </x:row>
     <x:row r="117">
-      <x:c r="A117" s="6" t="n"/>
-      <x:c r="B117" s="23" t="n"/>
-      <x:c r="C117" s="23" t="n"/>
-      <x:c r="D117" s="23" t="n"/>
-      <x:c r="E117" s="23" t="n"/>
-      <x:c r="F117" s="23" t="n"/>
-      <x:c r="G117" s="23" t="n"/>
-      <x:c r="H117" s="23" t="n"/>
-      <x:c r="I117" s="23" t="n"/>
+      <x:c r="A117" s="6"/>
+      <x:c r="B117" s="23"/>
+      <x:c r="C117" s="23"/>
+      <x:c r="D117" s="23"/>
+      <x:c r="E117" s="23"/>
+      <x:c r="F117" s="23"/>
+      <x:c r="G117" s="23"/>
+      <x:c r="H117" s="23"/>
+      <x:c r="I117" s="23"/>
     </x:row>
     <x:row r="118">
-      <x:c r="A118" s="6" t="n"/>
-      <x:c r="B118" s="23" t="n"/>
-      <x:c r="C118" s="23" t="n"/>
-      <x:c r="D118" s="23" t="n"/>
-      <x:c r="E118" s="23" t="n"/>
-      <x:c r="F118" s="23" t="n"/>
-      <x:c r="G118" s="23" t="n"/>
-      <x:c r="H118" s="23" t="n"/>
-      <x:c r="I118" s="23" t="n"/>
+      <x:c r="A118" s="6"/>
+      <x:c r="B118" s="23"/>
+      <x:c r="C118" s="23"/>
+      <x:c r="D118" s="23"/>
+      <x:c r="E118" s="23"/>
+      <x:c r="F118" s="23"/>
+      <x:c r="G118" s="23"/>
+      <x:c r="H118" s="23"/>
+      <x:c r="I118" s="23"/>
     </x:row>
     <x:row r="119">
-      <x:c r="A119" s="6" t="n"/>
-      <x:c r="B119" s="23" t="n"/>
-      <x:c r="C119" s="23" t="n"/>
-      <x:c r="D119" s="23" t="n"/>
-      <x:c r="E119" s="23" t="n"/>
-      <x:c r="F119" s="23" t="n"/>
-      <x:c r="G119" s="23" t="n"/>
-      <x:c r="H119" s="23" t="n"/>
-      <x:c r="I119" s="23" t="n"/>
+      <x:c r="A119" s="6"/>
+      <x:c r="B119" s="23"/>
+      <x:c r="C119" s="23"/>
+      <x:c r="D119" s="23"/>
+      <x:c r="E119" s="23"/>
+      <x:c r="F119" s="23"/>
+      <x:c r="G119" s="23"/>
+      <x:c r="H119" s="23"/>
+      <x:c r="I119" s="23"/>
     </x:row>
     <x:row r="120">
-      <x:c r="A120" s="6" t="n"/>
-      <x:c r="B120" s="23" t="n"/>
-      <x:c r="C120" s="23" t="n"/>
-      <x:c r="D120" s="23" t="n"/>
-      <x:c r="E120" s="23" t="n"/>
-      <x:c r="F120" s="23" t="n"/>
-      <x:c r="G120" s="23" t="n"/>
-      <x:c r="H120" s="23" t="n"/>
-      <x:c r="I120" s="23" t="n"/>
+      <x:c r="A120" s="6"/>
+      <x:c r="B120" s="23"/>
+      <x:c r="C120" s="23"/>
+      <x:c r="D120" s="23"/>
+      <x:c r="E120" s="23"/>
+      <x:c r="F120" s="23"/>
+      <x:c r="G120" s="23"/>
+      <x:c r="H120" s="23"/>
+      <x:c r="I120" s="23"/>
     </x:row>
     <x:row r="121">
-      <x:c r="A121" s="6" t="n"/>
-      <x:c r="B121" s="23" t="n"/>
-      <x:c r="C121" s="23" t="n"/>
-      <x:c r="D121" s="23" t="n"/>
-      <x:c r="E121" s="23" t="n"/>
-      <x:c r="F121" s="23" t="n"/>
-      <x:c r="G121" s="23" t="n"/>
-      <x:c r="H121" s="23" t="n"/>
-      <x:c r="I121" s="23" t="n"/>
+      <x:c r="A121" s="6"/>
+      <x:c r="B121" s="23"/>
+      <x:c r="C121" s="23"/>
+      <x:c r="D121" s="23"/>
+      <x:c r="E121" s="23"/>
+      <x:c r="F121" s="23"/>
+      <x:c r="G121" s="23"/>
+      <x:c r="H121" s="23"/>
+      <x:c r="I121" s="23"/>
     </x:row>
     <x:row r="122">
-      <x:c r="A122" s="6" t="n"/>
-      <x:c r="B122" s="23" t="n"/>
-      <x:c r="C122" s="23" t="n"/>
-      <x:c r="D122" s="23" t="n"/>
-      <x:c r="E122" s="23" t="n"/>
-      <x:c r="F122" s="23" t="n"/>
-      <x:c r="G122" s="23" t="n"/>
-      <x:c r="H122" s="23" t="n"/>
-      <x:c r="I122" s="23" t="n"/>
+      <x:c r="A122" s="6"/>
+      <x:c r="B122" s="23"/>
+      <x:c r="C122" s="23"/>
+      <x:c r="D122" s="23"/>
+      <x:c r="E122" s="23"/>
+      <x:c r="F122" s="23"/>
+      <x:c r="G122" s="23"/>
+      <x:c r="H122" s="23"/>
+      <x:c r="I122" s="23"/>
     </x:row>
     <x:row r="123">
-      <x:c r="A123" s="6" t="n"/>
-      <x:c r="B123" s="23" t="n"/>
-      <x:c r="C123" s="23" t="n"/>
-      <x:c r="D123" s="23" t="n"/>
-      <x:c r="E123" s="23" t="n"/>
-      <x:c r="F123" s="23" t="n"/>
-      <x:c r="G123" s="23" t="n"/>
-      <x:c r="H123" s="23" t="n"/>
-      <x:c r="I123" s="23" t="n"/>
+      <x:c r="A123" s="6"/>
+      <x:c r="B123" s="23"/>
+      <x:c r="C123" s="23"/>
+      <x:c r="D123" s="23"/>
+      <x:c r="E123" s="23"/>
+      <x:c r="F123" s="23"/>
+      <x:c r="G123" s="23"/>
+      <x:c r="H123" s="23"/>
+      <x:c r="I123" s="23"/>
     </x:row>
     <x:row r="124">
-      <x:c r="A124" s="6" t="n"/>
-      <x:c r="B124" s="23" t="n"/>
-      <x:c r="C124" s="23" t="n"/>
-      <x:c r="D124" s="23" t="n"/>
-      <x:c r="E124" s="23" t="n"/>
-      <x:c r="F124" s="23" t="n"/>
-      <x:c r="G124" s="23" t="n"/>
-      <x:c r="H124" s="23" t="n"/>
-      <x:c r="I124" s="23" t="n"/>
+      <x:c r="A124" s="6"/>
+      <x:c r="B124" s="23"/>
+      <x:c r="C124" s="23"/>
+      <x:c r="D124" s="23"/>
+      <x:c r="E124" s="23"/>
+      <x:c r="F124" s="23"/>
+      <x:c r="G124" s="23"/>
+      <x:c r="H124" s="23"/>
+      <x:c r="I124" s="23"/>
     </x:row>
     <x:row r="125">
-      <x:c r="A125" s="6" t="n"/>
-      <x:c r="B125" s="23" t="n"/>
-      <x:c r="C125" s="23" t="n"/>
-      <x:c r="D125" s="23" t="n"/>
-      <x:c r="E125" s="23" t="n"/>
-      <x:c r="F125" s="23" t="n"/>
-      <x:c r="G125" s="23" t="n"/>
-      <x:c r="H125" s="23" t="n"/>
-      <x:c r="I125" s="23" t="n"/>
+      <x:c r="A125" s="6"/>
+      <x:c r="B125" s="23"/>
+      <x:c r="C125" s="23"/>
+      <x:c r="D125" s="23"/>
+      <x:c r="E125" s="23"/>
+      <x:c r="F125" s="23"/>
+      <x:c r="G125" s="23"/>
+      <x:c r="H125" s="23"/>
+      <x:c r="I125" s="23"/>
     </x:row>
     <x:row r="126">
-      <x:c r="A126" s="6" t="n"/>
-      <x:c r="B126" s="23" t="n"/>
-      <x:c r="C126" s="23" t="n"/>
-      <x:c r="D126" s="23" t="n"/>
-      <x:c r="E126" s="23" t="n"/>
-      <x:c r="F126" s="23" t="n"/>
-      <x:c r="G126" s="23" t="n"/>
-      <x:c r="H126" s="23" t="n"/>
-      <x:c r="I126" s="23" t="n"/>
+      <x:c r="A126" s="6"/>
+      <x:c r="B126" s="23"/>
+      <x:c r="C126" s="23"/>
+      <x:c r="D126" s="23"/>
+      <x:c r="E126" s="23"/>
+      <x:c r="F126" s="23"/>
+      <x:c r="G126" s="23"/>
+      <x:c r="H126" s="23"/>
+      <x:c r="I126" s="23"/>
     </x:row>
     <x:row r="127">
-      <x:c r="A127" s="6" t="n"/>
-      <x:c r="B127" s="23" t="n"/>
-      <x:c r="C127" s="23" t="n"/>
-      <x:c r="D127" s="23" t="n"/>
-      <x:c r="E127" s="23" t="n"/>
-      <x:c r="F127" s="23" t="n"/>
-      <x:c r="G127" s="23" t="n"/>
-      <x:c r="H127" s="23" t="n"/>
-      <x:c r="I127" s="23" t="n"/>
+      <x:c r="A127" s="6"/>
+      <x:c r="B127" s="23"/>
+      <x:c r="C127" s="23"/>
+      <x:c r="D127" s="23"/>
+      <x:c r="E127" s="23"/>
+      <x:c r="F127" s="23"/>
+      <x:c r="G127" s="23"/>
+      <x:c r="H127" s="23"/>
+      <x:c r="I127" s="23"/>
     </x:row>
     <x:row r="128">
-      <x:c r="A128" s="6" t="n"/>
-      <x:c r="B128" s="23" t="n"/>
-      <x:c r="C128" s="23" t="n"/>
-      <x:c r="D128" s="23" t="n"/>
-      <x:c r="E128" s="23" t="n"/>
-      <x:c r="F128" s="23" t="n"/>
-      <x:c r="G128" s="23" t="n"/>
-      <x:c r="H128" s="23" t="n"/>
-      <x:c r="I128" s="23" t="n"/>
+      <x:c r="A128" s="6"/>
+      <x:c r="B128" s="23"/>
+      <x:c r="C128" s="23"/>
+      <x:c r="D128" s="23"/>
+      <x:c r="E128" s="23"/>
+      <x:c r="F128" s="23"/>
+      <x:c r="G128" s="23"/>
+      <x:c r="H128" s="23"/>
+      <x:c r="I128" s="23"/>
     </x:row>
     <x:row r="129">
-      <x:c r="A129" s="6" t="n"/>
-      <x:c r="B129" s="23" t="n"/>
-      <x:c r="C129" s="23" t="n"/>
-      <x:c r="D129" s="23" t="n"/>
-      <x:c r="E129" s="23" t="n"/>
-      <x:c r="F129" s="23" t="n"/>
-      <x:c r="G129" s="23" t="n"/>
-      <x:c r="H129" s="23" t="n"/>
-      <x:c r="I129" s="23" t="n"/>
+      <x:c r="A129" s="6"/>
+      <x:c r="B129" s="23"/>
+      <x:c r="C129" s="23"/>
+      <x:c r="D129" s="23"/>
+      <x:c r="E129" s="23"/>
+      <x:c r="F129" s="23"/>
+      <x:c r="G129" s="23"/>
+      <x:c r="H129" s="23"/>
+      <x:c r="I129" s="23"/>
     </x:row>
     <x:row r="130">
-      <x:c r="A130" s="6" t="n"/>
-      <x:c r="B130" s="23" t="n"/>
-      <x:c r="C130" s="23" t="n"/>
-      <x:c r="D130" s="23" t="n"/>
-      <x:c r="E130" s="23" t="n"/>
-      <x:c r="F130" s="23" t="n"/>
-      <x:c r="G130" s="23" t="n"/>
-      <x:c r="H130" s="23" t="n"/>
-      <x:c r="I130" s="23" t="n"/>
+      <x:c r="A130" s="6"/>
+      <x:c r="B130" s="23"/>
+      <x:c r="C130" s="23"/>
+      <x:c r="D130" s="23"/>
+      <x:c r="E130" s="23"/>
+      <x:c r="F130" s="23"/>
+      <x:c r="G130" s="23"/>
+      <x:c r="H130" s="23"/>
+      <x:c r="I130" s="23"/>
     </x:row>
     <x:row r="131">
-      <x:c r="A131" s="6" t="n"/>
-      <x:c r="B131" s="23" t="n"/>
-      <x:c r="C131" s="23" t="n"/>
-      <x:c r="D131" s="23" t="n"/>
-      <x:c r="E131" s="23" t="n"/>
-      <x:c r="F131" s="23" t="n"/>
-      <x:c r="G131" s="23" t="n"/>
-      <x:c r="H131" s="23" t="n"/>
-      <x:c r="I131" s="23" t="n"/>
+      <x:c r="A131" s="6"/>
+      <x:c r="B131" s="23"/>
+      <x:c r="C131" s="23"/>
+      <x:c r="D131" s="23"/>
+      <x:c r="E131" s="23"/>
+      <x:c r="F131" s="23"/>
+      <x:c r="G131" s="23"/>
+      <x:c r="H131" s="23"/>
+      <x:c r="I131" s="23"/>
     </x:row>
     <x:row r="132">
-      <x:c r="A132" s="6" t="n"/>
-      <x:c r="B132" s="23" t="n"/>
-      <x:c r="C132" s="23" t="n"/>
-      <x:c r="D132" s="23" t="n"/>
-      <x:c r="E132" s="23" t="n"/>
-      <x:c r="F132" s="23" t="n"/>
-      <x:c r="G132" s="23" t="n"/>
-      <x:c r="H132" s="23" t="n"/>
-      <x:c r="I132" s="23" t="n"/>
+      <x:c r="A132" s="6"/>
+      <x:c r="B132" s="23"/>
+      <x:c r="C132" s="23"/>
+      <x:c r="D132" s="23"/>
+      <x:c r="E132" s="23"/>
+      <x:c r="F132" s="23"/>
+      <x:c r="G132" s="23"/>
+      <x:c r="H132" s="23"/>
+      <x:c r="I132" s="23"/>
     </x:row>
     <x:row r="133">
-      <x:c r="A133" s="6" t="n"/>
-      <x:c r="B133" s="23" t="n"/>
-      <x:c r="C133" s="23" t="n"/>
-      <x:c r="D133" s="23" t="n"/>
-      <x:c r="E133" s="23" t="n"/>
-      <x:c r="F133" s="23" t="n"/>
-      <x:c r="G133" s="23" t="n"/>
-      <x:c r="H133" s="23" t="n"/>
-      <x:c r="I133" s="23" t="n"/>
+      <x:c r="A133" s="6"/>
+      <x:c r="B133" s="23"/>
+      <x:c r="C133" s="23"/>
+      <x:c r="D133" s="23"/>
+      <x:c r="E133" s="23"/>
+      <x:c r="F133" s="23"/>
+      <x:c r="G133" s="23"/>
+      <x:c r="H133" s="23"/>
+      <x:c r="I133" s="23"/>
     </x:row>
     <x:row r="134">
-      <x:c r="A134" s="6" t="n"/>
-      <x:c r="B134" s="23" t="n"/>
-      <x:c r="C134" s="23" t="n"/>
-      <x:c r="D134" s="23" t="n"/>
-      <x:c r="E134" s="23" t="n"/>
-      <x:c r="F134" s="23" t="n"/>
-      <x:c r="G134" s="23" t="n"/>
-      <x:c r="H134" s="23" t="n"/>
-      <x:c r="I134" s="23" t="n"/>
+      <x:c r="A134" s="6"/>
+      <x:c r="B134" s="23"/>
+      <x:c r="C134" s="23"/>
+      <x:c r="D134" s="23"/>
+      <x:c r="E134" s="23"/>
+      <x:c r="F134" s="23"/>
+      <x:c r="G134" s="23"/>
+      <x:c r="H134" s="23"/>
+      <x:c r="I134" s="23"/>
     </x:row>
     <x:row r="135">
-      <x:c r="A135" s="6" t="n"/>
-      <x:c r="B135" s="23" t="n"/>
-      <x:c r="C135" s="23" t="n"/>
-      <x:c r="D135" s="23" t="n"/>
-      <x:c r="E135" s="23" t="n"/>
-      <x:c r="F135" s="23" t="n"/>
-      <x:c r="G135" s="23" t="n"/>
-      <x:c r="H135" s="23" t="n"/>
-      <x:c r="I135" s="23" t="n"/>
+      <x:c r="A135" s="6"/>
+      <x:c r="B135" s="23"/>
+      <x:c r="C135" s="23"/>
+      <x:c r="D135" s="23"/>
+      <x:c r="E135" s="23"/>
+      <x:c r="F135" s="23"/>
+      <x:c r="G135" s="23"/>
+      <x:c r="H135" s="23"/>
+      <x:c r="I135" s="23"/>
     </x:row>
     <x:row r="136">
-      <x:c r="A136" s="6" t="n"/>
-      <x:c r="B136" s="23" t="n"/>
-      <x:c r="C136" s="23" t="n"/>
-      <x:c r="D136" s="23" t="n"/>
-      <x:c r="E136" s="23" t="n"/>
-      <x:c r="F136" s="23" t="n"/>
-      <x:c r="G136" s="23" t="n"/>
-      <x:c r="H136" s="23" t="n"/>
-      <x:c r="I136" s="23" t="n"/>
+      <x:c r="A136" s="6"/>
+      <x:c r="B136" s="23"/>
+      <x:c r="C136" s="23"/>
+      <x:c r="D136" s="23"/>
+      <x:c r="E136" s="23"/>
+      <x:c r="F136" s="23"/>
+      <x:c r="G136" s="23"/>
+      <x:c r="H136" s="23"/>
+      <x:c r="I136" s="23"/>
     </x:row>
     <x:row r="137">
-      <x:c r="A137" s="6" t="n"/>
-      <x:c r="B137" s="23" t="n"/>
-      <x:c r="C137" s="23" t="n"/>
-      <x:c r="D137" s="23" t="n"/>
-      <x:c r="E137" s="23" t="n"/>
-      <x:c r="F137" s="23" t="n"/>
-      <x:c r="G137" s="23" t="n"/>
-      <x:c r="H137" s="23" t="n"/>
-      <x:c r="I137" s="23" t="n"/>
+      <x:c r="A137" s="6"/>
+      <x:c r="B137" s="23"/>
+      <x:c r="C137" s="23"/>
+      <x:c r="D137" s="23"/>
+      <x:c r="E137" s="23"/>
+      <x:c r="F137" s="23"/>
+      <x:c r="G137" s="23"/>
+      <x:c r="H137" s="23"/>
+      <x:c r="I137" s="23"/>
     </x:row>
     <x:row r="138">
-      <x:c r="A138" s="6" t="n"/>
-      <x:c r="B138" s="23" t="n"/>
-      <x:c r="C138" s="23" t="n"/>
-      <x:c r="D138" s="23" t="n"/>
-      <x:c r="E138" s="23" t="n"/>
-      <x:c r="F138" s="23" t="n"/>
-      <x:c r="G138" s="23" t="n"/>
-      <x:c r="H138" s="23" t="n"/>
-      <x:c r="I138" s="23" t="n"/>
+      <x:c r="A138" s="6"/>
+      <x:c r="B138" s="23"/>
+      <x:c r="C138" s="23"/>
+      <x:c r="D138" s="23"/>
+      <x:c r="E138" s="23"/>
+      <x:c r="F138" s="23"/>
+      <x:c r="G138" s="23"/>
+      <x:c r="H138" s="23"/>
+      <x:c r="I138" s="23"/>
     </x:row>
     <x:row r="139">
-      <x:c r="A139" s="6" t="n"/>
-      <x:c r="B139" s="23" t="n"/>
-      <x:c r="C139" s="23" t="n"/>
-      <x:c r="D139" s="23" t="n"/>
-      <x:c r="E139" s="23" t="n"/>
-      <x:c r="F139" s="23" t="n"/>
-      <x:c r="G139" s="23" t="n"/>
-      <x:c r="H139" s="23" t="n"/>
-      <x:c r="I139" s="23" t="n"/>
+      <x:c r="A139" s="6"/>
+      <x:c r="B139" s="23"/>
+      <x:c r="C139" s="23"/>
+      <x:c r="D139" s="23"/>
+      <x:c r="E139" s="23"/>
+      <x:c r="F139" s="23"/>
+      <x:c r="G139" s="23"/>
+      <x:c r="H139" s="23"/>
+      <x:c r="I139" s="23"/>
     </x:row>
     <x:row r="140">
-      <x:c r="A140" s="6" t="n"/>
-      <x:c r="B140" s="23" t="n"/>
-      <x:c r="C140" s="23" t="n"/>
-      <x:c r="D140" s="23" t="n"/>
-      <x:c r="E140" s="23" t="n"/>
-      <x:c r="F140" s="23" t="n"/>
-      <x:c r="G140" s="23" t="n"/>
-      <x:c r="H140" s="23" t="n"/>
-      <x:c r="I140" s="23" t="n"/>
+      <x:c r="A140" s="6"/>
+      <x:c r="B140" s="23"/>
+      <x:c r="C140" s="23"/>
+      <x:c r="D140" s="23"/>
+      <x:c r="E140" s="23"/>
+      <x:c r="F140" s="23"/>
+      <x:c r="G140" s="23"/>
+      <x:c r="H140" s="23"/>
+      <x:c r="I140" s="23"/>
     </x:row>
     <x:row r="141">
-      <x:c r="A141" s="6" t="n"/>
-      <x:c r="B141" s="23" t="n"/>
-      <x:c r="C141" s="23" t="n"/>
-      <x:c r="D141" s="23" t="n"/>
-      <x:c r="E141" s="23" t="n"/>
-      <x:c r="F141" s="23" t="n"/>
-      <x:c r="G141" s="23" t="n"/>
-      <x:c r="H141" s="23" t="n"/>
-      <x:c r="I141" s="23" t="n"/>
+      <x:c r="A141" s="6"/>
+      <x:c r="B141" s="23"/>
+      <x:c r="C141" s="23"/>
+      <x:c r="D141" s="23"/>
+      <x:c r="E141" s="23"/>
+      <x:c r="F141" s="23"/>
+      <x:c r="G141" s="23"/>
+      <x:c r="H141" s="23"/>
+      <x:c r="I141" s="23"/>
     </x:row>
     <x:row r="142">
-      <x:c r="A142" s="6" t="n"/>
-      <x:c r="B142" s="23" t="n"/>
-      <x:c r="C142" s="23" t="n"/>
-      <x:c r="D142" s="23" t="n"/>
-      <x:c r="E142" s="23" t="n"/>
-      <x:c r="F142" s="23" t="n"/>
-      <x:c r="G142" s="23" t="n"/>
-      <x:c r="H142" s="23" t="n"/>
-      <x:c r="I142" s="23" t="n"/>
+      <x:c r="A142" s="6"/>
+      <x:c r="B142" s="23"/>
+      <x:c r="C142" s="23"/>
+      <x:c r="D142" s="23"/>
+      <x:c r="E142" s="23"/>
+      <x:c r="F142" s="23"/>
+      <x:c r="G142" s="23"/>
+      <x:c r="H142" s="23"/>
+      <x:c r="I142" s="23"/>
     </x:row>
     <x:row r="143">
-      <x:c r="A143" s="6" t="n"/>
-      <x:c r="B143" s="23" t="n"/>
-      <x:c r="C143" s="23" t="n"/>
-      <x:c r="D143" s="23" t="n"/>
-      <x:c r="E143" s="23" t="n"/>
-      <x:c r="F143" s="23" t="n"/>
-      <x:c r="G143" s="23" t="n"/>
-      <x:c r="H143" s="23" t="n"/>
-      <x:c r="I143" s="23" t="n"/>
+      <x:c r="A143" s="6"/>
+      <x:c r="B143" s="23"/>
+      <x:c r="C143" s="23"/>
+      <x:c r="D143" s="23"/>
+      <x:c r="E143" s="23"/>
+      <x:c r="F143" s="23"/>
+      <x:c r="G143" s="23"/>
+      <x:c r="H143" s="23"/>
+      <x:c r="I143" s="23"/>
     </x:row>
     <x:row r="144">
-      <x:c r="A144" s="6" t="n"/>
-      <x:c r="B144" s="23" t="n"/>
-      <x:c r="C144" s="23" t="n"/>
-      <x:c r="D144" s="23" t="n"/>
-      <x:c r="E144" s="23" t="n"/>
-      <x:c r="F144" s="23" t="n"/>
-      <x:c r="G144" s="23" t="n"/>
-      <x:c r="H144" s="23" t="n"/>
-      <x:c r="I144" s="23" t="n"/>
+      <x:c r="A144" s="6"/>
+      <x:c r="B144" s="23"/>
+      <x:c r="C144" s="23"/>
+      <x:c r="D144" s="23"/>
+      <x:c r="E144" s="23"/>
+      <x:c r="F144" s="23"/>
+      <x:c r="G144" s="23"/>
+      <x:c r="H144" s="23"/>
+      <x:c r="I144" s="23"/>
     </x:row>
     <x:row r="145">
-      <x:c r="A145" s="6" t="n"/>
-      <x:c r="B145" s="23" t="n"/>
-      <x:c r="C145" s="23" t="n"/>
-      <x:c r="D145" s="23" t="n"/>
-      <x:c r="E145" s="23" t="n"/>
-      <x:c r="F145" s="23" t="n"/>
-      <x:c r="G145" s="23" t="n"/>
-      <x:c r="H145" s="23" t="n"/>
-      <x:c r="I145" s="23" t="n"/>
+      <x:c r="A145" s="6"/>
+      <x:c r="B145" s="23"/>
+      <x:c r="C145" s="23"/>
+      <x:c r="D145" s="23"/>
+      <x:c r="E145" s="23"/>
+      <x:c r="F145" s="23"/>
+      <x:c r="G145" s="23"/>
+      <x:c r="H145" s="23"/>
+      <x:c r="I145" s="23"/>
     </x:row>
     <x:row r="146">
-      <x:c r="A146" s="6" t="n"/>
-      <x:c r="B146" s="23" t="n"/>
-      <x:c r="C146" s="23" t="n"/>
-      <x:c r="D146" s="23" t="n"/>
-      <x:c r="E146" s="23" t="n"/>
-      <x:c r="F146" s="23" t="n"/>
-      <x:c r="G146" s="23" t="n"/>
-      <x:c r="H146" s="23" t="n"/>
-      <x:c r="I146" s="23" t="n"/>
+      <x:c r="A146" s="6"/>
+      <x:c r="B146" s="23"/>
+      <x:c r="C146" s="23"/>
+      <x:c r="D146" s="23"/>
+      <x:c r="E146" s="23"/>
+      <x:c r="F146" s="23"/>
+      <x:c r="G146" s="23"/>
+      <x:c r="H146" s="23"/>
+      <x:c r="I146" s="23"/>
     </x:row>
     <x:row r="147">
-      <x:c r="A147" s="6" t="n"/>
-      <x:c r="B147" s="23" t="n"/>
-      <x:c r="C147" s="23" t="n"/>
-      <x:c r="D147" s="23" t="n"/>
-      <x:c r="E147" s="23" t="n"/>
-      <x:c r="F147" s="23" t="n"/>
-      <x:c r="G147" s="23" t="n"/>
-      <x:c r="H147" s="23" t="n"/>
-      <x:c r="I147" s="23" t="n"/>
+      <x:c r="A147" s="6"/>
+      <x:c r="B147" s="23"/>
+      <x:c r="C147" s="23"/>
+      <x:c r="D147" s="23"/>
+      <x:c r="E147" s="23"/>
+      <x:c r="F147" s="23"/>
+      <x:c r="G147" s="23"/>
+      <x:c r="H147" s="23"/>
+      <x:c r="I147" s="23"/>
     </x:row>
     <x:row r="148">
-      <x:c r="A148" s="6" t="n"/>
-      <x:c r="B148" s="23" t="n"/>
-      <x:c r="C148" s="23" t="n"/>
-      <x:c r="D148" s="23" t="n"/>
-      <x:c r="E148" s="23" t="n"/>
-      <x:c r="F148" s="23" t="n"/>
-      <x:c r="G148" s="23" t="n"/>
-      <x:c r="H148" s="23" t="n"/>
-      <x:c r="I148" s="23" t="n"/>
+      <x:c r="A148" s="6"/>
+      <x:c r="B148" s="23"/>
+      <x:c r="C148" s="23"/>
+      <x:c r="D148" s="23"/>
+      <x:c r="E148" s="23"/>
+      <x:c r="F148" s="23"/>
+      <x:c r="G148" s="23"/>
+      <x:c r="H148" s="23"/>
+      <x:c r="I148" s="23"/>
     </x:row>
     <x:row r="149">
-      <x:c r="A149" s="6" t="n"/>
-      <x:c r="B149" s="23" t="n"/>
-      <x:c r="C149" s="23" t="n"/>
-      <x:c r="D149" s="23" t="n"/>
-      <x:c r="E149" s="23" t="n"/>
-      <x:c r="F149" s="23" t="n"/>
-      <x:c r="G149" s="23" t="n"/>
-      <x:c r="H149" s="23" t="n"/>
-      <x:c r="I149" s="23" t="n"/>
+      <x:c r="A149" s="6"/>
+      <x:c r="B149" s="23"/>
+      <x:c r="C149" s="23"/>
+      <x:c r="D149" s="23"/>
+      <x:c r="E149" s="23"/>
+      <x:c r="F149" s="23"/>
+      <x:c r="G149" s="23"/>
+      <x:c r="H149" s="23"/>
+      <x:c r="I149" s="23"/>
     </x:row>
     <x:row r="150">
-      <x:c r="A150" s="6" t="n"/>
-      <x:c r="B150" s="23" t="n"/>
-      <x:c r="C150" s="23" t="n"/>
-      <x:c r="D150" s="23" t="n"/>
-      <x:c r="E150" s="23" t="n"/>
-      <x:c r="F150" s="23" t="n"/>
-      <x:c r="G150" s="23" t="n"/>
-      <x:c r="H150" s="23" t="n"/>
-      <x:c r="I150" s="23" t="n"/>
+      <x:c r="A150" s="6"/>
+      <x:c r="B150" s="23"/>
+      <x:c r="C150" s="23"/>
+      <x:c r="D150" s="23"/>
+      <x:c r="E150" s="23"/>
+      <x:c r="F150" s="23"/>
+      <x:c r="G150" s="23"/>
+      <x:c r="H150" s="23"/>
+      <x:c r="I150" s="23"/>
     </x:row>
     <x:row r="151">
-      <x:c r="A151" s="6" t="n"/>
-      <x:c r="B151" s="23" t="n"/>
-      <x:c r="C151" s="23" t="n"/>
-      <x:c r="D151" s="23" t="n"/>
-      <x:c r="E151" s="23" t="n"/>
-      <x:c r="F151" s="23" t="n"/>
-      <x:c r="G151" s="23" t="n"/>
-      <x:c r="H151" s="23" t="n"/>
-      <x:c r="I151" s="23" t="n"/>
+      <x:c r="A151" s="6"/>
+      <x:c r="B151" s="23"/>
+      <x:c r="C151" s="23"/>
+      <x:c r="D151" s="23"/>
+      <x:c r="E151" s="23"/>
+      <x:c r="F151" s="23"/>
+      <x:c r="G151" s="23"/>
+      <x:c r="H151" s="23"/>
+      <x:c r="I151" s="23"/>
     </x:row>
     <x:row r="152">
-      <x:c r="A152" s="6" t="n"/>
-      <x:c r="B152" s="23" t="n"/>
-      <x:c r="C152" s="23" t="n"/>
-      <x:c r="D152" s="23" t="n"/>
-      <x:c r="E152" s="23" t="n"/>
-      <x:c r="F152" s="23" t="n"/>
-      <x:c r="G152" s="23" t="n"/>
-      <x:c r="H152" s="23" t="n"/>
-      <x:c r="I152" s="23" t="n"/>
+      <x:c r="A152" s="6"/>
+      <x:c r="B152" s="23"/>
+      <x:c r="C152" s="23"/>
+      <x:c r="D152" s="23"/>
+      <x:c r="E152" s="23"/>
+      <x:c r="F152" s="23"/>
+      <x:c r="G152" s="23"/>
+      <x:c r="H152" s="23"/>
+      <x:c r="I152" s="23"/>
     </x:row>
     <x:row r="153">
-      <x:c r="A153" s="6" t="n"/>
-      <x:c r="B153" s="23" t="n"/>
-      <x:c r="C153" s="23" t="n"/>
-      <x:c r="D153" s="23" t="n"/>
-      <x:c r="E153" s="23" t="n"/>
-      <x:c r="F153" s="23" t="n"/>
-      <x:c r="G153" s="23" t="n"/>
-      <x:c r="H153" s="23" t="n"/>
-      <x:c r="I153" s="23" t="n"/>
+      <x:c r="A153" s="6"/>
+      <x:c r="B153" s="23"/>
+      <x:c r="C153" s="23"/>
+      <x:c r="D153" s="23"/>
+      <x:c r="E153" s="23"/>
+      <x:c r="F153" s="23"/>
+      <x:c r="G153" s="23"/>
+      <x:c r="H153" s="23"/>
+      <x:c r="I153" s="23"/>
     </x:row>
     <x:row r="154">
-      <x:c r="A154" s="6" t="n"/>
-      <x:c r="B154" s="23" t="n"/>
-      <x:c r="C154" s="23" t="n"/>
-      <x:c r="D154" s="23" t="n"/>
-      <x:c r="E154" s="23" t="n"/>
-      <x:c r="F154" s="23" t="n"/>
-      <x:c r="G154" s="23" t="n"/>
-      <x:c r="H154" s="23" t="n"/>
-      <x:c r="I154" s="23" t="n"/>
+      <x:c r="A154" s="6"/>
+      <x:c r="B154" s="23"/>
+      <x:c r="C154" s="23"/>
+      <x:c r="D154" s="23"/>
+      <x:c r="E154" s="23"/>
+      <x:c r="F154" s="23"/>
+      <x:c r="G154" s="23"/>
+      <x:c r="H154" s="23"/>
+      <x:c r="I154" s="23"/>
     </x:row>
     <x:row r="155">
-      <x:c r="A155" s="6" t="n"/>
-      <x:c r="B155" s="23" t="n"/>
-      <x:c r="C155" s="23" t="n"/>
-      <x:c r="D155" s="23" t="n"/>
-      <x:c r="E155" s="23" t="n"/>
-      <x:c r="F155" s="23" t="n"/>
-      <x:c r="G155" s="23" t="n"/>
-      <x:c r="H155" s="23" t="n"/>
-      <x:c r="I155" s="23" t="n"/>
+      <x:c r="A155" s="6"/>
+      <x:c r="B155" s="23"/>
+      <x:c r="C155" s="23"/>
+      <x:c r="D155" s="23"/>
+      <x:c r="E155" s="23"/>
+      <x:c r="F155" s="23"/>
+      <x:c r="G155" s="23"/>
+      <x:c r="H155" s="23"/>
+      <x:c r="I155" s="23"/>
     </x:row>
     <x:row r="156">
-      <x:c r="A156" s="6" t="n"/>
-      <x:c r="B156" s="23" t="n"/>
-      <x:c r="C156" s="23" t="n"/>
-      <x:c r="D156" s="23" t="n"/>
-      <x:c r="E156" s="23" t="n"/>
-      <x:c r="F156" s="23" t="n"/>
-      <x:c r="G156" s="23" t="n"/>
-      <x:c r="H156" s="23" t="n"/>
-      <x:c r="I156" s="23" t="n"/>
+      <x:c r="A156" s="6"/>
+      <x:c r="B156" s="23"/>
+      <x:c r="C156" s="23"/>
+      <x:c r="D156" s="23"/>
+      <x:c r="E156" s="23"/>
+      <x:c r="F156" s="23"/>
+      <x:c r="G156" s="23"/>
+      <x:c r="H156" s="23"/>
+      <x:c r="I156" s="23"/>
     </x:row>
     <x:row r="157">
-      <x:c r="A157" s="6" t="n"/>
-      <x:c r="B157" s="23" t="n"/>
-      <x:c r="C157" s="23" t="n"/>
-      <x:c r="D157" s="23" t="n"/>
-      <x:c r="E157" s="23" t="n"/>
-      <x:c r="F157" s="23" t="n"/>
-      <x:c r="G157" s="23" t="n"/>
-      <x:c r="H157" s="23" t="n"/>
-      <x:c r="I157" s="23" t="n"/>
+      <x:c r="A157" s="6"/>
+      <x:c r="B157" s="23"/>
+      <x:c r="C157" s="23"/>
+      <x:c r="D157" s="23"/>
+      <x:c r="E157" s="23"/>
+      <x:c r="F157" s="23"/>
+      <x:c r="G157" s="23"/>
+      <x:c r="H157" s="23"/>
+      <x:c r="I157" s="23"/>
     </x:row>
     <x:row r="158">
-      <x:c r="A158" s="6" t="n"/>
-      <x:c r="B158" s="23" t="n"/>
-      <x:c r="C158" s="23" t="n"/>
-      <x:c r="D158" s="23" t="n"/>
-      <x:c r="E158" s="23" t="n"/>
-      <x:c r="F158" s="23" t="n"/>
-      <x:c r="G158" s="23" t="n"/>
-      <x:c r="H158" s="23" t="n"/>
-      <x:c r="I158" s="23" t="n"/>
+      <x:c r="A158" s="6"/>
+      <x:c r="B158" s="23"/>
+      <x:c r="C158" s="23"/>
+      <x:c r="D158" s="23"/>
+      <x:c r="E158" s="23"/>
+      <x:c r="F158" s="23"/>
+      <x:c r="G158" s="23"/>
+      <x:c r="H158" s="23"/>
+      <x:c r="I158" s="23"/>
     </x:row>
     <x:row r="159">
-      <x:c r="A159" s="6" t="n"/>
-      <x:c r="B159" s="23" t="n"/>
-      <x:c r="C159" s="23" t="n"/>
-      <x:c r="D159" s="23" t="n"/>
-      <x:c r="E159" s="23" t="n"/>
-      <x:c r="F159" s="23" t="n"/>
-      <x:c r="G159" s="23" t="n"/>
-      <x:c r="H159" s="23" t="n"/>
-      <x:c r="I159" s="23" t="n"/>
+      <x:c r="A159" s="6"/>
+      <x:c r="B159" s="23"/>
+      <x:c r="C159" s="23"/>
+      <x:c r="D159" s="23"/>
+      <x:c r="E159" s="23"/>
+      <x:c r="F159" s="23"/>
+      <x:c r="G159" s="23"/>
+      <x:c r="H159" s="23"/>
+      <x:c r="I159" s="23"/>
     </x:row>
     <x:row r="160">
-      <x:c r="A160" s="6" t="n"/>
-      <x:c r="B160" s="23" t="n"/>
-      <x:c r="C160" s="23" t="n"/>
-      <x:c r="D160" s="23" t="n"/>
-      <x:c r="E160" s="23" t="n"/>
-      <x:c r="F160" s="23" t="n"/>
-      <x:c r="G160" s="23" t="n"/>
-      <x:c r="H160" s="23" t="n"/>
-      <x:c r="I160" s="23" t="n"/>
+      <x:c r="A160" s="6"/>
+      <x:c r="B160" s="23"/>
+      <x:c r="C160" s="23"/>
+      <x:c r="D160" s="23"/>
+      <x:c r="E160" s="23"/>
+      <x:c r="F160" s="23"/>
+      <x:c r="G160" s="23"/>
+      <x:c r="H160" s="23"/>
+      <x:c r="I160" s="23"/>
     </x:row>
     <x:row r="161">
-      <x:c r="A161" s="6" t="n"/>
-      <x:c r="B161" s="23" t="n"/>
-      <x:c r="C161" s="23" t="n"/>
-      <x:c r="D161" s="23" t="n"/>
-      <x:c r="E161" s="23" t="n"/>
-      <x:c r="F161" s="23" t="n"/>
-      <x:c r="G161" s="23" t="n"/>
-      <x:c r="H161" s="23" t="n"/>
-      <x:c r="I161" s="23" t="n"/>
+      <x:c r="A161" s="6"/>
+      <x:c r="B161" s="23"/>
+      <x:c r="C161" s="23"/>
+      <x:c r="D161" s="23"/>
+      <x:c r="E161" s="23"/>
+      <x:c r="F161" s="23"/>
+      <x:c r="G161" s="23"/>
+      <x:c r="H161" s="23"/>
+      <x:c r="I161" s="23"/>
     </x:row>
     <x:row r="162">
-      <x:c r="A162" s="6" t="n"/>
-      <x:c r="B162" s="23" t="n"/>
-      <x:c r="C162" s="23" t="n"/>
-      <x:c r="D162" s="23" t="n"/>
-      <x:c r="E162" s="23" t="n"/>
-      <x:c r="F162" s="23" t="n"/>
-      <x:c r="G162" s="23" t="n"/>
-      <x:c r="H162" s="23" t="n"/>
-      <x:c r="I162" s="23" t="n"/>
+      <x:c r="A162" s="6"/>
+      <x:c r="B162" s="23"/>
+      <x:c r="C162" s="23"/>
+      <x:c r="D162" s="23"/>
+      <x:c r="E162" s="23"/>
+      <x:c r="F162" s="23"/>
+      <x:c r="G162" s="23"/>
+      <x:c r="H162" s="23"/>
+      <x:c r="I162" s="23"/>
     </x:row>
     <x:row r="163">
-      <x:c r="A163" s="6" t="n"/>
-      <x:c r="B163" s="23" t="n"/>
-      <x:c r="C163" s="23" t="n"/>
-      <x:c r="D163" s="23" t="n"/>
-      <x:c r="E163" s="23" t="n"/>
-      <x:c r="F163" s="23" t="n"/>
-      <x:c r="G163" s="23" t="n"/>
-      <x:c r="H163" s="23" t="n"/>
-      <x:c r="I163" s="23" t="n"/>
+      <x:c r="A163" s="6"/>
+      <x:c r="B163" s="23"/>
+      <x:c r="C163" s="23"/>
+      <x:c r="D163" s="23"/>
+      <x:c r="E163" s="23"/>
+      <x:c r="F163" s="23"/>
+      <x:c r="G163" s="23"/>
+      <x:c r="H163" s="23"/>
+      <x:c r="I163" s="23"/>
     </x:row>
     <x:row r="164">
-      <x:c r="A164" s="6" t="n"/>
-      <x:c r="B164" s="23" t="n"/>
-      <x:c r="C164" s="23" t="n"/>
-      <x:c r="D164" s="23" t="n"/>
-      <x:c r="E164" s="23" t="n"/>
-      <x:c r="F164" s="23" t="n"/>
-      <x:c r="G164" s="23" t="n"/>
-      <x:c r="H164" s="23" t="n"/>
-      <x:c r="I164" s="23" t="n"/>
+      <x:c r="A164" s="6"/>
+      <x:c r="B164" s="23"/>
+      <x:c r="C164" s="23"/>
+      <x:c r="D164" s="23"/>
+      <x:c r="E164" s="23"/>
+      <x:c r="F164" s="23"/>
+      <x:c r="G164" s="23"/>
+      <x:c r="H164" s="23"/>
+      <x:c r="I164" s="23"/>
     </x:row>
     <x:row r="165">
-      <x:c r="A165" s="6" t="n"/>
-      <x:c r="B165" s="23" t="n"/>
-      <x:c r="C165" s="23" t="n"/>
-      <x:c r="D165" s="23" t="n"/>
-      <x:c r="E165" s="23" t="n"/>
-      <x:c r="F165" s="23" t="n"/>
-      <x:c r="G165" s="23" t="n"/>
-      <x:c r="H165" s="23" t="n"/>
-      <x:c r="I165" s="23" t="n"/>
+      <x:c r="A165" s="6"/>
+      <x:c r="B165" s="23"/>
+      <x:c r="C165" s="23"/>
+      <x:c r="D165" s="23"/>
+      <x:c r="E165" s="23"/>
+      <x:c r="F165" s="23"/>
+      <x:c r="G165" s="23"/>
+      <x:c r="H165" s="23"/>
+      <x:c r="I165" s="23"/>
     </x:row>
     <x:row r="166">
-      <x:c r="A166" s="6" t="n"/>
-      <x:c r="B166" s="23" t="n"/>
-      <x:c r="C166" s="23" t="n"/>
-      <x:c r="D166" s="23" t="n"/>
-      <x:c r="E166" s="23" t="n"/>
-      <x:c r="F166" s="23" t="n"/>
-      <x:c r="G166" s="23" t="n"/>
-      <x:c r="H166" s="23" t="n"/>
-      <x:c r="I166" s="23" t="n"/>
+      <x:c r="A166" s="6"/>
+      <x:c r="B166" s="23"/>
+      <x:c r="C166" s="23"/>
+      <x:c r="D166" s="23"/>
+      <x:c r="E166" s="23"/>
+      <x:c r="F166" s="23"/>
+      <x:c r="G166" s="23"/>
+      <x:c r="H166" s="23"/>
+      <x:c r="I166" s="23"/>
     </x:row>
     <x:row r="167">
-      <x:c r="A167" s="6" t="n"/>
-      <x:c r="B167" s="23" t="n"/>
-      <x:c r="C167" s="23" t="n"/>
-      <x:c r="D167" s="23" t="n"/>
-      <x:c r="E167" s="23" t="n"/>
-      <x:c r="F167" s="23" t="n"/>
-      <x:c r="G167" s="23" t="n"/>
-      <x:c r="H167" s="23" t="n"/>
-      <x:c r="I167" s="23" t="n"/>
+      <x:c r="A167" s="6"/>
+      <x:c r="B167" s="23"/>
+      <x:c r="C167" s="23"/>
+      <x:c r="D167" s="23"/>
+      <x:c r="E167" s="23"/>
+      <x:c r="F167" s="23"/>
+      <x:c r="G167" s="23"/>
+      <x:c r="H167" s="23"/>
+      <x:c r="I167" s="23"/>
     </x:row>
     <x:row r="168">
-      <x:c r="A168" s="6" t="n"/>
-      <x:c r="B168" s="23" t="n"/>
-      <x:c r="C168" s="23" t="n"/>
-      <x:c r="D168" s="23" t="n"/>
-      <x:c r="E168" s="23" t="n"/>
-      <x:c r="F168" s="23" t="n"/>
-      <x:c r="G168" s="23" t="n"/>
-      <x:c r="H168" s="23" t="n"/>
-      <x:c r="I168" s="23" t="n"/>
+      <x:c r="A168" s="6"/>
+      <x:c r="B168" s="23"/>
+      <x:c r="C168" s="23"/>
+      <x:c r="D168" s="23"/>
+      <x:c r="E168" s="23"/>
+      <x:c r="F168" s="23"/>
+      <x:c r="G168" s="23"/>
+      <x:c r="H168" s="23"/>
+      <x:c r="I168" s="23"/>
     </x:row>
     <x:row r="169">
-      <x:c r="A169" s="6" t="n"/>
-      <x:c r="B169" s="23" t="n"/>
-      <x:c r="C169" s="23" t="n"/>
-      <x:c r="D169" s="23" t="n"/>
-      <x:c r="E169" s="23" t="n"/>
-      <x:c r="F169" s="23" t="n"/>
-      <x:c r="G169" s="23" t="n"/>
-      <x:c r="H169" s="23" t="n"/>
-      <x:c r="I169" s="23" t="n"/>
+      <x:c r="A169" s="6"/>
+      <x:c r="B169" s="23"/>
+      <x:c r="C169" s="23"/>
+      <x:c r="D169" s="23"/>
+      <x:c r="E169" s="23"/>
+      <x:c r="F169" s="23"/>
+      <x:c r="G169" s="23"/>
+      <x:c r="H169" s="23"/>
+      <x:c r="I169" s="23"/>
     </x:row>
     <x:row r="170">
-      <x:c r="A170" s="6" t="n"/>
-      <x:c r="B170" s="23" t="n"/>
-      <x:c r="C170" s="23" t="n"/>
-      <x:c r="D170" s="23" t="n"/>
-      <x:c r="E170" s="23" t="n"/>
-      <x:c r="F170" s="23" t="n"/>
-      <x:c r="G170" s="23" t="n"/>
-      <x:c r="H170" s="23" t="n"/>
-      <x:c r="I170" s="23" t="n"/>
+      <x:c r="A170" s="6"/>
+      <x:c r="B170" s="23"/>
+      <x:c r="C170" s="23"/>
+      <x:c r="D170" s="23"/>
+      <x:c r="E170" s="23"/>
+      <x:c r="F170" s="23"/>
+      <x:c r="G170" s="23"/>
+      <x:c r="H170" s="23"/>
+      <x:c r="I170" s="23"/>
     </x:row>
     <x:row r="171">
-      <x:c r="A171" s="6" t="n"/>
-      <x:c r="B171" s="23" t="n"/>
-      <x:c r="C171" s="23" t="n"/>
-      <x:c r="D171" s="23" t="n"/>
-      <x:c r="E171" s="23" t="n"/>
-      <x:c r="F171" s="23" t="n"/>
-      <x:c r="G171" s="23" t="n"/>
-      <x:c r="H171" s="23" t="n"/>
-      <x:c r="I171" s="23" t="n"/>
+      <x:c r="A171" s="6"/>
+      <x:c r="B171" s="23"/>
+      <x:c r="C171" s="23"/>
+      <x:c r="D171" s="23"/>
+      <x:c r="E171" s="23"/>
+      <x:c r="F171" s="23"/>
+      <x:c r="G171" s="23"/>
+      <x:c r="H171" s="23"/>
+      <x:c r="I171" s="23"/>
     </x:row>
     <x:row r="172">
-      <x:c r="A172" s="6" t="n"/>
-      <x:c r="B172" s="23" t="n"/>
-      <x:c r="C172" s="23" t="n"/>
-      <x:c r="D172" s="23" t="n"/>
-      <x:c r="E172" s="23" t="n"/>
-      <x:c r="F172" s="23" t="n"/>
-      <x:c r="G172" s="23" t="n"/>
-      <x:c r="H172" s="23" t="n"/>
-      <x:c r="I172" s="23" t="n"/>
+      <x:c r="A172" s="6"/>
+      <x:c r="B172" s="23"/>
+      <x:c r="C172" s="23"/>
+      <x:c r="D172" s="23"/>
+      <x:c r="E172" s="23"/>
+      <x:c r="F172" s="23"/>
+      <x:c r="G172" s="23"/>
+      <x:c r="H172" s="23"/>
+      <x:c r="I172" s="23"/>
     </x:row>
     <x:row r="173">
-      <x:c r="A173" s="6" t="n"/>
-      <x:c r="B173" s="23" t="n"/>
-      <x:c r="C173" s="23" t="n"/>
-      <x:c r="D173" s="23" t="n"/>
-      <x:c r="E173" s="23" t="n"/>
-      <x:c r="F173" s="23" t="n"/>
-      <x:c r="G173" s="23" t="n"/>
-      <x:c r="H173" s="23" t="n"/>
-      <x:c r="I173" s="23" t="n"/>
+      <x:c r="A173" s="6"/>
+      <x:c r="B173" s="23"/>
+      <x:c r="C173" s="23"/>
+      <x:c r="D173" s="23"/>
+      <x:c r="E173" s="23"/>
+      <x:c r="F173" s="23"/>
+      <x:c r="G173" s="23"/>
+      <x:c r="H173" s="23"/>
+      <x:c r="I173" s="23"/>
     </x:row>
     <x:row r="174">
-      <x:c r="A174" s="6" t="n"/>
-      <x:c r="B174" s="23" t="n"/>
-      <x:c r="C174" s="23" t="n"/>
-      <x:c r="D174" s="23" t="n"/>
-      <x:c r="E174" s="23" t="n"/>
-      <x:c r="F174" s="23" t="n"/>
-      <x:c r="G174" s="23" t="n"/>
-      <x:c r="H174" s="23" t="n"/>
-      <x:c r="I174" s="23" t="n"/>
+      <x:c r="A174" s="6"/>
+      <x:c r="B174" s="23"/>
+      <x:c r="C174" s="23"/>
+      <x:c r="D174" s="23"/>
+      <x:c r="E174" s="23"/>
+      <x:c r="F174" s="23"/>
+      <x:c r="G174" s="23"/>
+      <x:c r="H174" s="23"/>
+      <x:c r="I174" s="23"/>
     </x:row>
     <x:row r="175">
-      <x:c r="A175" s="6" t="n"/>
-      <x:c r="B175" s="23" t="n"/>
-      <x:c r="C175" s="23" t="n"/>
-      <x:c r="D175" s="23" t="n"/>
-      <x:c r="E175" s="23" t="n"/>
-      <x:c r="F175" s="23" t="n"/>
-      <x:c r="G175" s="23" t="n"/>
-      <x:c r="H175" s="23" t="n"/>
-      <x:c r="I175" s="23" t="n"/>
+      <x:c r="A175" s="6"/>
+      <x:c r="B175" s="23"/>
+      <x:c r="C175" s="23"/>
+      <x:c r="D175" s="23"/>
+      <x:c r="E175" s="23"/>
+      <x:c r="F175" s="23"/>
+      <x:c r="G175" s="23"/>
+      <x:c r="H175" s="23"/>
+      <x:c r="I175" s="23"/>
     </x:row>
     <x:row r="176">
-      <x:c r="A176" s="6" t="n"/>
-      <x:c r="B176" s="23" t="n"/>
-      <x:c r="C176" s="23" t="n"/>
-      <x:c r="D176" s="23" t="n"/>
-      <x:c r="E176" s="23" t="n"/>
-      <x:c r="F176" s="23" t="n"/>
-      <x:c r="G176" s="23" t="n"/>
-      <x:c r="H176" s="23" t="n"/>
-      <x:c r="I176" s="23" t="n"/>
+      <x:c r="A176" s="6"/>
+      <x:c r="B176" s="23"/>
+      <x:c r="C176" s="23"/>
+      <x:c r="D176" s="23"/>
+      <x:c r="E176" s="23"/>
+      <x:c r="F176" s="23"/>
+      <x:c r="G176" s="23"/>
+      <x:c r="H176" s="23"/>
+      <x:c r="I176" s="23"/>
     </x:row>
     <x:row r="177">
-      <x:c r="A177" s="6" t="n"/>
-      <x:c r="B177" s="23" t="n"/>
-      <x:c r="C177" s="23" t="n"/>
-      <x:c r="D177" s="23" t="n"/>
-      <x:c r="E177" s="23" t="n"/>
-      <x:c r="F177" s="23" t="n"/>
-      <x:c r="G177" s="23" t="n"/>
-      <x:c r="H177" s="23" t="n"/>
-      <x:c r="I177" s="23" t="n"/>
+      <x:c r="A177" s="6"/>
+      <x:c r="B177" s="23"/>
+      <x:c r="C177" s="23"/>
+      <x:c r="D177" s="23"/>
+      <x:c r="E177" s="23"/>
+      <x:c r="F177" s="23"/>
+      <x:c r="G177" s="23"/>
+      <x:c r="H177" s="23"/>
+      <x:c r="I177" s="23"/>
     </x:row>
     <x:row r="178">
-      <x:c r="A178" s="6" t="n"/>
-      <x:c r="B178" s="23" t="n"/>
-      <x:c r="C178" s="23" t="n"/>
-      <x:c r="D178" s="23" t="n"/>
-      <x:c r="E178" s="23" t="n"/>
-      <x:c r="F178" s="23" t="n"/>
-      <x:c r="G178" s="23" t="n"/>
-      <x:c r="H178" s="23" t="n"/>
-      <x:c r="I178" s="23" t="n"/>
+      <x:c r="A178" s="6"/>
+      <x:c r="B178" s="23"/>
+      <x:c r="C178" s="23"/>
+      <x:c r="D178" s="23"/>
+      <x:c r="E178" s="23"/>
+      <x:c r="F178" s="23"/>
+      <x:c r="G178" s="23"/>
+      <x:c r="H178" s="23"/>
+      <x:c r="I178" s="23"/>
     </x:row>
     <x:row r="179">
-      <x:c r="A179" s="6" t="n"/>
-      <x:c r="B179" s="23" t="n"/>
-      <x:c r="C179" s="23" t="n"/>
-      <x:c r="D179" s="23" t="n"/>
-      <x:c r="E179" s="23" t="n"/>
-      <x:c r="F179" s="23" t="n"/>
-      <x:c r="G179" s="23" t="n"/>
-      <x:c r="H179" s="23" t="n"/>
-      <x:c r="I179" s="23" t="n"/>
+      <x:c r="A179" s="6"/>
+      <x:c r="B179" s="23"/>
+      <x:c r="C179" s="23"/>
+      <x:c r="D179" s="23"/>
+      <x:c r="E179" s="23"/>
+      <x:c r="F179" s="23"/>
+      <x:c r="G179" s="23"/>
+      <x:c r="H179" s="23"/>
+      <x:c r="I179" s="23"/>
     </x:row>
     <x:row r="180">
-      <x:c r="A180" s="6" t="n"/>
-      <x:c r="B180" s="23" t="n"/>
-      <x:c r="C180" s="23" t="n"/>
-      <x:c r="D180" s="23" t="n"/>
-      <x:c r="E180" s="23" t="n"/>
-      <x:c r="F180" s="23" t="n"/>
-      <x:c r="G180" s="23" t="n"/>
-      <x:c r="H180" s="23" t="n"/>
-      <x:c r="I180" s="23" t="n"/>
+      <x:c r="A180" s="6"/>
+      <x:c r="B180" s="23"/>
+      <x:c r="C180" s="23"/>
+      <x:c r="D180" s="23"/>
+      <x:c r="E180" s="23"/>
+      <x:c r="F180" s="23"/>
+      <x:c r="G180" s="23"/>
+      <x:c r="H180" s="23"/>
+      <x:c r="I180" s="23"/>
     </x:row>
     <x:row r="181">
-      <x:c r="A181" s="6" t="n"/>
-      <x:c r="B181" s="23" t="n"/>
-      <x:c r="C181" s="23" t="n"/>
-      <x:c r="D181" s="23" t="n"/>
-      <x:c r="E181" s="23" t="n"/>
-      <x:c r="F181" s="23" t="n"/>
-      <x:c r="G181" s="23" t="n"/>
-      <x:c r="H181" s="23" t="n"/>
-      <x:c r="I181" s="23" t="n"/>
+      <x:c r="A181" s="6"/>
+      <x:c r="B181" s="23"/>
+      <x:c r="C181" s="23"/>
+      <x:c r="D181" s="23"/>
+      <x:c r="E181" s="23"/>
+      <x:c r="F181" s="23"/>
+      <x:c r="G181" s="23"/>
+      <x:c r="H181" s="23"/>
+      <x:c r="I181" s="23"/>
     </x:row>
     <x:row r="182">
-      <x:c r="A182" s="6" t="n"/>
-      <x:c r="B182" s="23" t="n"/>
-      <x:c r="C182" s="23" t="n"/>
-      <x:c r="D182" s="23" t="n"/>
-      <x:c r="E182" s="23" t="n"/>
-      <x:c r="F182" s="23" t="n"/>
-      <x:c r="G182" s="23" t="n"/>
-      <x:c r="H182" s="23" t="n"/>
-      <x:c r="I182" s="23" t="n"/>
+      <x:c r="A182" s="6"/>
+      <x:c r="B182" s="23"/>
+      <x:c r="C182" s="23"/>
+      <x:c r="D182" s="23"/>
+      <x:c r="E182" s="23"/>
+      <x:c r="F182" s="23"/>
+      <x:c r="G182" s="23"/>
+      <x:c r="H182" s="23"/>
+      <x:c r="I182" s="23"/>
     </x:row>
     <x:row r="183">
-      <x:c r="A183" s="6" t="n"/>
-      <x:c r="B183" s="23" t="n"/>
-      <x:c r="C183" s="23" t="n"/>
-      <x:c r="D183" s="23" t="n"/>
-      <x:c r="E183" s="23" t="n"/>
-      <x:c r="F183" s="23" t="n"/>
-      <x:c r="G183" s="23" t="n"/>
-      <x:c r="H183" s="23" t="n"/>
-      <x:c r="I183" s="23" t="n"/>
+      <x:c r="A183" s="6"/>
+      <x:c r="B183" s="23"/>
+      <x:c r="C183" s="23"/>
+      <x:c r="D183" s="23"/>
+      <x:c r="E183" s="23"/>
+      <x:c r="F183" s="23"/>
+      <x:c r="G183" s="23"/>
+      <x:c r="H183" s="23"/>
+      <x:c r="I183" s="23"/>
     </x:row>
     <x:row r="184">
-      <x:c r="A184" s="6" t="n"/>
-      <x:c r="B184" s="23" t="n"/>
-      <x:c r="C184" s="23" t="n"/>
-      <x:c r="D184" s="23" t="n"/>
-      <x:c r="E184" s="23" t="n"/>
-      <x:c r="F184" s="23" t="n"/>
-      <x:c r="G184" s="23" t="n"/>
-      <x:c r="H184" s="23" t="n"/>
-      <x:c r="I184" s="23" t="n"/>
+      <x:c r="A184" s="6"/>
+      <x:c r="B184" s="23"/>
+      <x:c r="C184" s="23"/>
+      <x:c r="D184" s="23"/>
+      <x:c r="E184" s="23"/>
+      <x:c r="F184" s="23"/>
+      <x:c r="G184" s="23"/>
+      <x:c r="H184" s="23"/>
+      <x:c r="I184" s="23"/>
     </x:row>
     <x:row r="185">
-      <x:c r="A185" s="6" t="n"/>
-      <x:c r="B185" s="23" t="n"/>
-      <x:c r="C185" s="23" t="n"/>
-      <x:c r="D185" s="23" t="n"/>
-      <x:c r="E185" s="23" t="n"/>
-      <x:c r="F185" s="23" t="n"/>
-      <x:c r="G185" s="23" t="n"/>
-      <x:c r="H185" s="23" t="n"/>
-      <x:c r="I185" s="23" t="n"/>
+      <x:c r="A185" s="6"/>
+      <x:c r="B185" s="23"/>
+      <x:c r="C185" s="23"/>
+      <x:c r="D185" s="23"/>
+      <x:c r="E185" s="23"/>
+      <x:c r="F185" s="23"/>
+      <x:c r="G185" s="23"/>
+      <x:c r="H185" s="23"/>
+      <x:c r="I185" s="23"/>
     </x:row>
     <x:row r="186">
-      <x:c r="A186" s="6" t="n"/>
-      <x:c r="B186" s="23" t="n"/>
-      <x:c r="C186" s="23" t="n"/>
-      <x:c r="D186" s="23" t="n"/>
-      <x:c r="E186" s="23" t="n"/>
-      <x:c r="F186" s="23" t="n"/>
-      <x:c r="G186" s="23" t="n"/>
-      <x:c r="H186" s="23" t="n"/>
-      <x:c r="I186" s="23" t="n"/>
+      <x:c r="A186" s="6"/>
+      <x:c r="B186" s="23"/>
+      <x:c r="C186" s="23"/>
+      <x:c r="D186" s="23"/>
+      <x:c r="E186" s="23"/>
+      <x:c r="F186" s="23"/>
+      <x:c r="G186" s="23"/>
+      <x:c r="H186" s="23"/>
+      <x:c r="I186" s="23"/>
     </x:row>
     <x:row r="187">
-      <x:c r="A187" s="6" t="n"/>
-      <x:c r="B187" s="23" t="n"/>
-      <x:c r="C187" s="23" t="n"/>
-      <x:c r="D187" s="23" t="n"/>
-      <x:c r="E187" s="23" t="n"/>
-      <x:c r="F187" s="23" t="n"/>
-      <x:c r="G187" s="23" t="n"/>
-      <x:c r="H187" s="23" t="n"/>
-      <x:c r="I187" s="23" t="n"/>
+      <x:c r="A187" s="6"/>
+      <x:c r="B187" s="23"/>
+      <x:c r="C187" s="23"/>
+      <x:c r="D187" s="23"/>
+      <x:c r="E187" s="23"/>
+      <x:c r="F187" s="23"/>
+      <x:c r="G187" s="23"/>
+      <x:c r="H187" s="23"/>
+      <x:c r="I187" s="23"/>
     </x:row>
     <x:row r="188">
-      <x:c r="A188" s="6" t="n"/>
-      <x:c r="B188" s="23" t="n"/>
-      <x:c r="C188" s="23" t="n"/>
-      <x:c r="D188" s="23" t="n"/>
-      <x:c r="E188" s="23" t="n"/>
-      <x:c r="F188" s="23" t="n"/>
-      <x:c r="G188" s="23" t="n"/>
-      <x:c r="H188" s="23" t="n"/>
-      <x:c r="I188" s="23" t="n"/>
+      <x:c r="A188" s="6"/>
+      <x:c r="B188" s="23"/>
+      <x:c r="C188" s="23"/>
+      <x:c r="D188" s="23"/>
+      <x:c r="E188" s="23"/>
+      <x:c r="F188" s="23"/>
+      <x:c r="G188" s="23"/>
+      <x:c r="H188" s="23"/>
+      <x:c r="I188" s="23"/>
     </x:row>
     <x:row r="189">
-      <x:c r="A189" s="6" t="n"/>
-      <x:c r="B189" s="23" t="n"/>
-      <x:c r="C189" s="23" t="n"/>
-      <x:c r="D189" s="23" t="n"/>
-      <x:c r="E189" s="23" t="n"/>
-      <x:c r="F189" s="23" t="n"/>
-      <x:c r="G189" s="23" t="n"/>
-      <x:c r="H189" s="23" t="n"/>
-      <x:c r="I189" s="23" t="n"/>
+      <x:c r="A189" s="6"/>
+      <x:c r="B189" s="23"/>
+      <x:c r="C189" s="23"/>
+      <x:c r="D189" s="23"/>
+      <x:c r="E189" s="23"/>
+      <x:c r="F189" s="23"/>
+      <x:c r="G189" s="23"/>
+      <x:c r="H189" s="23"/>
+      <x:c r="I189" s="23"/>
     </x:row>
     <x:row r="190">
-      <x:c r="A190" s="6" t="n"/>
-      <x:c r="B190" s="23" t="n"/>
-      <x:c r="C190" s="23" t="n"/>
-      <x:c r="D190" s="23" t="n"/>
-      <x:c r="E190" s="23" t="n"/>
-      <x:c r="F190" s="23" t="n"/>
-      <x:c r="G190" s="23" t="n"/>
-      <x:c r="H190" s="23" t="n"/>
-      <x:c r="I190" s="23" t="n"/>
+      <x:c r="A190" s="6"/>
+      <x:c r="B190" s="23"/>
+      <x:c r="C190" s="23"/>
+      <x:c r="D190" s="23"/>
+      <x:c r="E190" s="23"/>
+      <x:c r="F190" s="23"/>
+      <x:c r="G190" s="23"/>
+      <x:c r="H190" s="23"/>
+      <x:c r="I190" s="23"/>
     </x:row>
     <x:row r="191">
-      <x:c r="A191" s="6" t="n"/>
-      <x:c r="B191" s="23" t="n"/>
-      <x:c r="C191" s="23" t="n"/>
-      <x:c r="D191" s="23" t="n"/>
-      <x:c r="E191" s="23" t="n"/>
-      <x:c r="F191" s="23" t="n"/>
-      <x:c r="G191" s="23" t="n"/>
-      <x:c r="H191" s="23" t="n"/>
-      <x:c r="I191" s="23" t="n"/>
+      <x:c r="A191" s="6"/>
+      <x:c r="B191" s="23"/>
+      <x:c r="C191" s="23"/>
+      <x:c r="D191" s="23"/>
+      <x:c r="E191" s="23"/>
+      <x:c r="F191" s="23"/>
+      <x:c r="G191" s="23"/>
+      <x:c r="H191" s="23"/>
+      <x:c r="I191" s="23"/>
     </x:row>
     <x:row r="192">
-      <x:c r="A192" s="6" t="n"/>
-      <x:c r="B192" s="23" t="n"/>
-      <x:c r="C192" s="23" t="n"/>
-      <x:c r="D192" s="23" t="n"/>
-      <x:c r="E192" s="23" t="n"/>
-      <x:c r="F192" s="23" t="n"/>
-      <x:c r="G192" s="23" t="n"/>
-      <x:c r="H192" s="23" t="n"/>
-      <x:c r="I192" s="23" t="n"/>
+      <x:c r="A192" s="6"/>
+      <x:c r="B192" s="23"/>
+      <x:c r="C192" s="23"/>
+      <x:c r="D192" s="23"/>
+      <x:c r="E192" s="23"/>
+      <x:c r="F192" s="23"/>
+      <x:c r="G192" s="23"/>
+      <x:c r="H192" s="23"/>
+      <x:c r="I192" s="23"/>
     </x:row>
     <x:row r="193">
-      <x:c r="A193" s="6" t="n"/>
-      <x:c r="B193" s="23" t="n"/>
-      <x:c r="C193" s="23" t="n"/>
-      <x:c r="D193" s="23" t="n"/>
-      <x:c r="E193" s="23" t="n"/>
-      <x:c r="F193" s="23" t="n"/>
-      <x:c r="G193" s="23" t="n"/>
-      <x:c r="H193" s="23" t="n"/>
-      <x:c r="I193" s="23" t="n"/>
+      <x:c r="A193" s="6"/>
+      <x:c r="B193" s="23"/>
+      <x:c r="C193" s="23"/>
+      <x:c r="D193" s="23"/>
+      <x:c r="E193" s="23"/>
+      <x:c r="F193" s="23"/>
+      <x:c r="G193" s="23"/>
+      <x:c r="H193" s="23"/>
+      <x:c r="I193" s="23"/>
     </x:row>
     <x:row r="194">
-      <x:c r="A194" s="6" t="n"/>
-      <x:c r="B194" s="23" t="n"/>
-      <x:c r="C194" s="23" t="n"/>
-      <x:c r="D194" s="23" t="n"/>
-      <x:c r="E194" s="23" t="n"/>
-      <x:c r="F194" s="23" t="n"/>
-      <x:c r="G194" s="23" t="n"/>
-      <x:c r="H194" s="23" t="n"/>
-      <x:c r="I194" s="23" t="n"/>
+      <x:c r="A194" s="6"/>
+      <x:c r="B194" s="23"/>
+      <x:c r="C194" s="23"/>
+      <x:c r="D194" s="23"/>
+      <x:c r="E194" s="23"/>
+      <x:c r="F194" s="23"/>
+      <x:c r="G194" s="23"/>
+      <x:c r="H194" s="23"/>
+      <x:c r="I194" s="23"/>
     </x:row>
     <x:row r="195">
-      <x:c r="A195" s="6" t="n"/>
-      <x:c r="B195" s="23" t="n"/>
-      <x:c r="C195" s="23" t="n"/>
-      <x:c r="D195" s="23" t="n"/>
-      <x:c r="E195" s="23" t="n"/>
-      <x:c r="F195" s="23" t="n"/>
-      <x:c r="G195" s="23" t="n"/>
-      <x:c r="H195" s="23" t="n"/>
-      <x:c r="I195" s="23" t="n"/>
+      <x:c r="A195" s="6"/>
+      <x:c r="B195" s="23"/>
+      <x:c r="C195" s="23"/>
+      <x:c r="D195" s="23"/>
+      <x:c r="E195" s="23"/>
+      <x:c r="F195" s="23"/>
+      <x:c r="G195" s="23"/>
+      <x:c r="H195" s="23"/>
+      <x:c r="I195" s="23"/>
     </x:row>
     <x:row r="196">
-      <x:c r="A196" s="6" t="n"/>
-      <x:c r="B196" s="23" t="n"/>
-      <x:c r="C196" s="23" t="n"/>
-      <x:c r="D196" s="23" t="n"/>
-      <x:c r="E196" s="23" t="n"/>
-      <x:c r="F196" s="23" t="n"/>
-      <x:c r="G196" s="23" t="n"/>
-      <x:c r="H196" s="23" t="n"/>
-      <x:c r="I196" s="23" t="n"/>
+      <x:c r="A196" s="6"/>
+      <x:c r="B196" s="23"/>
+      <x:c r="C196" s="23"/>
+      <x:c r="D196" s="23"/>
+      <x:c r="E196" s="23"/>
+      <x:c r="F196" s="23"/>
+      <x:c r="G196" s="23"/>
+      <x:c r="H196" s="23"/>
+      <x:c r="I196" s="23"/>
     </x:row>
     <x:row r="197">
-      <x:c r="A197" s="6" t="n"/>
-      <x:c r="B197" s="23" t="n"/>
-      <x:c r="C197" s="23" t="n"/>
-      <x:c r="D197" s="23" t="n"/>
-      <x:c r="E197" s="23" t="n"/>
-      <x:c r="F197" s="23" t="n"/>
-      <x:c r="G197" s="23" t="n"/>
-      <x:c r="H197" s="23" t="n"/>
-      <x:c r="I197" s="23" t="n"/>
+      <x:c r="A197" s="6"/>
+      <x:c r="B197" s="23"/>
+      <x:c r="C197" s="23"/>
+      <x:c r="D197" s="23"/>
+      <x:c r="E197" s="23"/>
+      <x:c r="F197" s="23"/>
+      <x:c r="G197" s="23"/>
+      <x:c r="H197" s="23"/>
+      <x:c r="I197" s="23"/>
     </x:row>
     <x:row r="198">
-      <x:c r="A198" s="6" t="n"/>
-      <x:c r="B198" s="23" t="n"/>
-      <x:c r="C198" s="23" t="n"/>
-      <x:c r="D198" s="23" t="n"/>
-      <x:c r="E198" s="23" t="n"/>
-      <x:c r="F198" s="23" t="n"/>
-      <x:c r="G198" s="23" t="n"/>
-      <x:c r="H198" s="23" t="n"/>
-      <x:c r="I198" s="23" t="n"/>
+      <x:c r="A198" s="6"/>
+      <x:c r="B198" s="23"/>
+      <x:c r="C198" s="23"/>
+      <x:c r="D198" s="23"/>
+      <x:c r="E198" s="23"/>
+      <x:c r="F198" s="23"/>
+      <x:c r="G198" s="23"/>
+      <x:c r="H198" s="23"/>
+      <x:c r="I198" s="23"/>
     </x:row>
     <x:row r="199">
-      <x:c r="A199" s="6" t="n"/>
-      <x:c r="B199" s="23" t="n"/>
-      <x:c r="C199" s="23" t="n"/>
-      <x:c r="D199" s="23" t="n"/>
-      <x:c r="E199" s="23" t="n"/>
-      <x:c r="F199" s="23" t="n"/>
-      <x:c r="G199" s="23" t="n"/>
-      <x:c r="H199" s="23" t="n"/>
-      <x:c r="I199" s="23" t="n"/>
+      <x:c r="A199" s="6"/>
+      <x:c r="B199" s="23"/>
+      <x:c r="C199" s="23"/>
+      <x:c r="D199" s="23"/>
+      <x:c r="E199" s="23"/>
+      <x:c r="F199" s="23"/>
+      <x:c r="G199" s="23"/>
+      <x:c r="H199" s="23"/>
+      <x:c r="I199" s="23"/>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" s="6" t="n"/>
-      <x:c r="B200" s="23" t="n"/>
-      <x:c r="C200" s="23" t="n"/>
-      <x:c r="D200" s="23" t="n"/>
-      <x:c r="E200" s="23" t="n"/>
-      <x:c r="F200" s="23" t="n"/>
-      <x:c r="G200" s="23" t="n"/>
-      <x:c r="H200" s="23" t="n"/>
-      <x:c r="I200" s="23" t="n"/>
+      <x:c r="A200" s="6"/>
+      <x:c r="B200" s="23"/>
+      <x:c r="C200" s="23"/>
+      <x:c r="D200" s="23"/>
+      <x:c r="E200" s="23"/>
+      <x:c r="F200" s="23"/>
+      <x:c r="G200" s="23"/>
+      <x:c r="H200" s="23"/>
+      <x:c r="I200" s="23"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="6" t="n"/>
@@ -33892,7 +33911,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34526460b02e45f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf15bae8d5744c45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34795,7 +34814,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c004669031b4127"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red21f29ab9b04356"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35674,7 +35693,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra698a6dc924044fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf826fd164e7c4025"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36097,7 +36116,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a80dc7d8054105"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34917b05dbd84409"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona notícia da Seleção Sub-20 sobre Vitorinha
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R466c76ffa7a345e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R684fd1ca9c4b45bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Refb9a20472dd4465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rc83268b0fdb141e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R56f0255bd705412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R5e52aa2429cc4bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rc235af7f8ca84129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5ba24e109cd24200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rb0f0ef9923194f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R1fd332f9318e4b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R031fddd5a6cb4ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Re6a68e7f6ace4a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R4f28c0e102844981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R749c2f1418874b16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R0247607662f84d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R47d9eb3c2de042ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R2f206fbf24134adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R29a973dc711e48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R33a16952c3214714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R06994de3a59b440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra2df49d3c58d4434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R08bec0dac4604b3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R22afb290f73c459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R1a9fac54a9b347e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R91d5f506431c4d9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R2c1e0fa065974db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rd3f79bd7a94942c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R52bb1238a7b949ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R5de1d53d318749bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R3efb10921a444b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rb19caff6658c4bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd299d5bd24204e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R05a55a010faf45b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rfe0885fd7e844514"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R5ad65d8624fc4d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R2d28768e1674482b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R11a99a24ce114481"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc340ae99db644d1d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfacd497295f14338"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf6db28bad3742a0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48f61a83e8014d67"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1be855c8fd74079"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf196b58698df4559"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raee4c951aa1d4c7a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25a689e36e0e4229"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R882805184a2f4cf2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,8 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I47"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2964,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4de84697034dc7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R789075bd60a34361"/>
 </x:worksheet>
 </file>
 
@@ -5253,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe7a25df30bc4122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R049aecf2d9354320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7561,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reac15c6d5bdb42e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad991c93fbe24b1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8193,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ddc1fc14c514d97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c51f93b33c424b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12383,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14db8528a18a4046"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71d0c0773a354197"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445df68e09244239"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc948fa3e1354f9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12676,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6423d04ce334ae5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c5cd59cca54f0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25227,7 +25227,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1210e3efed544d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566d100334f341aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27127,7 +27127,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72c7b655527a4d04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda0bfcfbd4434b3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27539,7 +27539,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06f369a6ef3d456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27c8588b46af4647"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27606,28 +27606,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
@@ -27635,28 +27635,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27664,19 +27664,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27685,7 +27685,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27693,57 +27693,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27751,28 +27751,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -27780,28 +27780,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -27809,19 +27809,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27830,7 +27830,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -27838,57 +27838,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -27896,28 +27896,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -27925,28 +27925,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -27954,19 +27954,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -27975,7 +27975,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -27983,57 +27983,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28041,28 +28041,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28070,19 +28070,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28091,7 +28091,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28099,19 +28099,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28120,7 +28120,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28128,19 +28128,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28149,7 +28149,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28157,48 +28157,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28207,7 +28207,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28215,19 +28215,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28236,56 +28236,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28294,36 +28294,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28331,19 +28331,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28352,7 +28352,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28360,28 +28360,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H28" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28389,28 +28389,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28418,48 +28418,48 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28468,7 +28468,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28476,28 +28476,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28505,48 +28505,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28555,36 +28555,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28592,28 +28592,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28621,57 +28621,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28679,115 +28679,115 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -28795,19 +28795,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28816,7 +28816,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -28824,98 +28824,116 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I46" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B47" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G47" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H47" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I46" s="23" t="str">
+      <x:c r="I47" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="6"/>
-      <x:c r="B47" s="23"/>
-      <x:c r="C47" s="23"/>
-      <x:c r="D47" s="23"/>
-      <x:c r="E47" s="23"/>
-      <x:c r="F47" s="23"/>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="23"/>
-      <x:c r="I47" s="23"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="6"/>
@@ -33911,7 +33929,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf15bae8d5744c45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68e2f2e462084bf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34814,7 +34832,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red21f29ab9b04356"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9679bcca8e44d6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35693,7 +35711,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf826fd164e7c4025"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ba69489f654799"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36116,7 +36134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34917b05dbd84409"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00026a9a24964abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona licitação de infraestrutura da Arena Pernambuco
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R33a16952c3214714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R06994de3a59b440a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra2df49d3c58d4434"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R08bec0dac4604b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R22afb290f73c459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R1a9fac54a9b347e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R91d5f506431c4d9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R2c1e0fa065974db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rd3f79bd7a94942c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R52bb1238a7b949ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R5de1d53d318749bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R3efb10921a444b10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rb19caff6658c4bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd299d5bd24204e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R05a55a010faf45b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rfe0885fd7e844514"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R5ad65d8624fc4d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R2d28768e1674482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R422fc88a52854293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R784da7d537f746ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R2452193d9b104700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R64891f3b6ba34beb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R5cf294f0d9214031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Rc28a8d761649466e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Red027fdb97464bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R7b05c81b0d6e490a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R09f5edd6541248ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R19f42c766ecc4cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R9d9be9a0027e46a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R3530b7900c504a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rf985c67f276e4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R5fc7cb95f5ab48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rc33cb935b2b043f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rbf71632a69df462d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Ra4405eed9a6f4318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Red9f8c48200a4d34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc340ae99db644d1d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R426f4e1da4d5409e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf6db28bad3742a0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6f1ad0946dc4bda"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1be855c8fd74079"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4c2c6c4e8214a72"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raee4c951aa1d4c7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd375873565b64fb4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R882805184a2f4cf2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67cc8e46540b4676"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,8 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I47"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I48"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2964,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R789075bd60a34361"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442979ac10c14003"/>
 </x:worksheet>
 </file>
 
@@ -5253,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R049aecf2d9354320"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c20a519e9ca4182"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7561,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad991c93fbe24b1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898c7ffa801d4ed1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8193,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c51f93b33c424b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b50550b576a4c44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12383,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71d0c0773a354197"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47da859ba36f40af"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc948fa3e1354f9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03a9f0815c594eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12676,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c5cd59cca54f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46f2a3c7053a40fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25227,7 +25227,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566d100334f341aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R922cb1284c6c471b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27127,7 +27127,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda0bfcfbd4434b3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c4a43d28f1456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27539,7 +27539,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27c8588b46af4647"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbece27af079a4a72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27603,22 +27603,22 @@
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="150.75" customHeight="1">
       <x:c r="A2" s="31" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27627,7 +27627,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
@@ -27635,28 +27635,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27664,28 +27664,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27693,19 +27693,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27714,7 +27714,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27722,57 +27722,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -27780,28 +27780,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -27809,28 +27809,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -27838,19 +27838,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27859,7 +27859,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -27867,57 +27867,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -27925,28 +27925,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -27954,28 +27954,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -27983,19 +27983,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28004,7 +28004,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28012,57 +28012,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28070,28 +28070,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28099,19 +28099,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28120,7 +28120,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28128,19 +28128,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28149,7 +28149,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28157,19 +28157,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28178,7 +28178,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28186,48 +28186,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28236,7 +28236,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28244,19 +28244,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28265,56 +28265,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28323,36 +28323,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28360,19 +28360,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28381,7 +28381,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28389,28 +28389,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28418,28 +28418,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28447,48 +28447,48 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28497,7 +28497,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28505,28 +28505,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28534,48 +28534,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28584,36 +28584,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28621,28 +28621,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28650,57 +28650,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -28708,115 +28708,115 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -28824,19 +28824,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28845,7 +28845,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -28853,98 +28853,116 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I47" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B48" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C48" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D48" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E48" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F48" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G48" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H48" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I47" s="23" t="str">
+      <x:c r="I48" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="6"/>
-      <x:c r="B48" s="23"/>
-      <x:c r="C48" s="23"/>
-      <x:c r="D48" s="23"/>
-      <x:c r="E48" s="23"/>
-      <x:c r="F48" s="23"/>
-      <x:c r="G48" s="23"/>
-      <x:c r="H48" s="23"/>
-      <x:c r="I48" s="23"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="6"/>
@@ -33929,7 +33947,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68e2f2e462084bf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39e62a19b44a4d63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34832,7 +34850,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9679bcca8e44d6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d4a0f3d563041c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35711,7 +35729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ba69489f654799"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f5b5d41b9f4df2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36134,7 +36152,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00026a9a24964abf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e96fa6101fd4c53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona desdobramento do workshop para Porto Alegre
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R422fc88a52854293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R784da7d537f746ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R2452193d9b104700"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R64891f3b6ba34beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R5cf294f0d9214031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Rc28a8d761649466e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Red027fdb97464bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R7b05c81b0d6e490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R09f5edd6541248ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R19f42c766ecc4cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R9d9be9a0027e46a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R3530b7900c504a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rf985c67f276e4b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R5fc7cb95f5ab48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rc33cb935b2b043f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rbf71632a69df462d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Ra4405eed9a6f4318"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Red9f8c48200a4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R4b5aa9f42a404f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rcb0e992682d64a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R8e7203cabeb54352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rd36f718a16674644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R22df86a36df34555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R7a44fc90bf204874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R205e83ea20944409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rb68521a05c75455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R50a92b27fd9c423f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R24419c1f37344c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R2f4e03f406bb46c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rbf15cc5b13a6489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R97ca5e1d01dd47cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R640c94d87e63415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rf0f1f7941f6a4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R691bbbcb91b24392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R3d83ef259ca84d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R32ea9aa0419c462f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R426f4e1da4d5409e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9f18c818e2614866"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6f1ad0946dc4bda"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7113d5ce2dd94349"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4c2c6c4e8214a72"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e6cb47b5ba94025"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd375873565b64fb4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b9c2f17f24d41e4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67cc8e46540b4676"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4e7def3277a4241"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,8 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I48"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I49"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2964,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442979ac10c14003"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280fedfebec4007"/>
 </x:worksheet>
 </file>
 
@@ -5253,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c20a519e9ca4182"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fda3f70b8854c92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7561,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898c7ffa801d4ed1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbafacc3c55064fb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8193,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b50550b576a4c44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73bdc2ccd7b445dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12383,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47da859ba36f40af"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8686a1cf12e6419c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03a9f0815c594eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra36b5c8a553c4e7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12676,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46f2a3c7053a40fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra454aaf71b3b4359"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25227,7 +25227,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R922cb1284c6c471b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb336a315fb5141d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27127,7 +27127,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c4a43d28f1456f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8f941b3bc004fac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27539,7 +27539,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbece27af079a4a72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R276e2cc0cb334de2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27922,31 +27922,31 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
         <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -27954,28 +27954,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -27983,28 +27983,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28012,19 +28012,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28033,7 +28033,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28041,57 +28041,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28099,28 +28099,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28128,19 +28128,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28149,7 +28149,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28157,19 +28157,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28178,7 +28178,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28186,19 +28186,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28207,7 +28207,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28215,48 +28215,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28265,7 +28265,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28273,19 +28273,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28294,56 +28294,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28352,36 +28352,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H28" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28389,19 +28389,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28410,7 +28410,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28418,28 +28418,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28447,28 +28447,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28476,48 +28476,48 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28526,7 +28526,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28534,28 +28534,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28563,48 +28563,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28613,36 +28613,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28650,28 +28650,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28679,57 +28679,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -28737,115 +28737,115 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -28853,19 +28853,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28874,7 +28874,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -28882,98 +28882,116 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I48" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B49" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C49" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D49" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E49" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F49" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G49" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H49" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I48" s="23" t="str">
+      <x:c r="I49" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="6"/>
-      <x:c r="B49" s="23"/>
-      <x:c r="C49" s="23"/>
-      <x:c r="D49" s="23"/>
-      <x:c r="E49" s="23"/>
-      <x:c r="F49" s="23"/>
-      <x:c r="G49" s="23"/>
-      <x:c r="H49" s="23"/>
-      <x:c r="I49" s="23"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="6"/>
@@ -33947,7 +33965,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39e62a19b44a4d63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1fe54999234fb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34850,7 +34868,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d4a0f3d563041c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1d9b2499de4170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35729,7 +35747,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f5b5d41b9f4df2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27919c11276b4812"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36152,7 +36170,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e96fa6101fd4c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R429624e07a714744"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona iniciativa de legado do Sesc RJ
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R4b5aa9f42a404f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rcb0e992682d64a92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R8e7203cabeb54352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rd36f718a16674644"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R22df86a36df34555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R7a44fc90bf204874"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R205e83ea20944409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rb68521a05c75455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R50a92b27fd9c423f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R24419c1f37344c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R2f4e03f406bb46c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rbf15cc5b13a6489d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R97ca5e1d01dd47cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R640c94d87e63415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rf0f1f7941f6a4917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R691bbbcb91b24392"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R3d83ef259ca84d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R32ea9aa0419c462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R9f59f917a7ae4f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R94ce25a44a484789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra7653faececa4f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R8234ec856190452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rcce12723b8994846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R7ed10c04f5374ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R82349b1acb43411c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rae6499f742fd44f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R4d447be74d124f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R886400e58e1a41bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R8678266995a740d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R5d7c166313404f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R585abe31d51f4777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rff6607b50e05440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rb6d48e8941fc44ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Ra8a66bf09da743be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rb533308b67ee4d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R9e6d7aa270a949ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9f18c818e2614866"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R357bd8c49ac242a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7113d5ce2dd94349"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R97c44043c16c4b7c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e6cb47b5ba94025"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b630ddbd34c453f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b9c2f17f24d41e4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a2ebc6478c24d80"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4e7def3277a4241"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfeff37e56134594"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,8 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I49"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I50"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2964,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280fedfebec4007"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761e11be19f84e0a"/>
 </x:worksheet>
 </file>
 
@@ -5253,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fda3f70b8854c92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f763ca9ea954b19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7561,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbafacc3c55064fb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ad4b5ccada489c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8193,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73bdc2ccd7b445dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdb3bc2aa4a4cb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12383,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8686a1cf12e6419c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9def725010284156"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra36b5c8a553c4e7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red56c1a37d9b4eac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12676,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra454aaf71b3b4359"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53c5acfe7404452"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13959,7 +13959,7 @@
       <x:c r="B2" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C2" s="29" t="n">
+      <x:c r="C2" s="32" t="n">
         <x:v>45859.5</x:v>
       </x:c>
       <x:c r="D2" s="23" t="str">
@@ -13983,8 +13983,12 @@
       <x:c r="J2" s="23" t="str">
         <x:v>Parque Jornalista Eduardo Couri (Barragem Santa Lúcia)</x:v>
       </x:c>
-      <x:c r="K2" s="8"/>
-      <x:c r="L2" s="8"/>
+      <x:c r="K2" s="8" t="n">
+        <x:v>-19.9167</x:v>
+      </x:c>
+      <x:c r="L2" s="8" t="n">
+        <x:v>-43.9345</x:v>
+      </x:c>
       <x:c r="M2" s="23" t="str">
         <x:v>https://agencia.petrobras.com.br/w/regionais/caravana-do-futebol-feminino-petrobras-chega-a-belo-horizonte-com-programacao-gratuita</x:v>
       </x:c>
@@ -14005,7 +14009,7 @@
       <x:c r="B3" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C3" s="29" t="n">
+      <x:c r="C3" s="32" t="n">
         <x:v>45887.5</x:v>
       </x:c>
       <x:c r="D3" s="23" t="str">
@@ -14029,8 +14033,12 @@
       <x:c r="J3" s="23" t="str">
         <x:v>Mercado Livre Arena Pacaembu</x:v>
       </x:c>
-      <x:c r="K3" s="8"/>
-      <x:c r="L3" s="8"/>
+      <x:c r="K3" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L3" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M3" s="23" t="str">
         <x:v>https://prefeitura.sp.gov.br/web/cultura/w/caravana-do-futebol-feminino-chega-na-cidade-com-apoio-da-prefeitura-de-s%C3%A3o-paulo</x:v>
       </x:c>
@@ -14051,7 +14059,7 @@
       <x:c r="B4" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C4" s="29" t="n">
+      <x:c r="C4" s="32" t="n">
         <x:v>45936.5</x:v>
       </x:c>
       <x:c r="D4" s="23" t="str">
@@ -14075,8 +14083,12 @@
       <x:c r="J4" s="23" t="str">
         <x:v>Avenida Borges de Medeiros, 2651–2729, Praia de Belas</x:v>
       </x:c>
-      <x:c r="K4" s="8"/>
-      <x:c r="L4" s="8"/>
+      <x:c r="K4" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L4" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M4" s="23" t="str">
         <x:v>https://agencia.petrobras.com.br/w/caravana-do-futebol-feminino-petrobras-chega-em-porto-alegre-com-programa%C3%A7%C3%A3o-gratuita</x:v>
       </x:c>
@@ -14097,7 +14109,7 @@
       <x:c r="B5" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C5" s="29" t="n">
+      <x:c r="C5" s="32" t="n">
         <x:v>45975.5</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
@@ -14121,8 +14133,12 @@
       <x:c r="J5" s="23" t="str">
         <x:v>Parque Costa Azul</x:v>
       </x:c>
-      <x:c r="K5" s="8"/>
-      <x:c r="L5" s="8"/>
+      <x:c r="K5" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L5" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M5" s="23" t="str">
         <x:v>https://agencia.petrobras.com.br/w/caravana-do-futebol-feminino-petrobras-chega-em-salvador-com-programa%C3%A7%C3%A3o-gratuita</x:v>
       </x:c>
@@ -14143,7 +14159,7 @@
       <x:c r="B6" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C6" s="29" t="n">
+      <x:c r="C6" s="32" t="n">
         <x:v>46047.5</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
@@ -14165,8 +14181,12 @@
       <x:c r="J6" s="23" t="str">
         <x:v>Avenida Atlântica, Copacabana</x:v>
       </x:c>
-      <x:c r="K6" s="8"/>
-      <x:c r="L6" s="8"/>
+      <x:c r="K6" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L6" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M6" s="23" t="str">
         <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/copa-mundo-feminina-brasil-marca-emblema-oficial</x:v>
       </x:c>
@@ -14187,7 +14207,7 @@
       <x:c r="B7" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C7" s="29" t="n">
+      <x:c r="C7" s="32" t="n">
         <x:v>46084.5</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
@@ -14209,8 +14229,12 @@
       <x:c r="J7" s="23" t="str">
         <x:v>Vila Olímpica Apolinho</x:v>
       </x:c>
-      <x:c r="K7" s="8"/>
-      <x:c r="L7" s="8"/>
+      <x:c r="K7" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L7" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M7" s="23" t="str">
         <x:v>https://esportes.prefeitura.rio/noticias/prefeitura-lanca-o-projeto-rio-capital-do-futebol-feminino/</x:v>
       </x:c>
@@ -14231,7 +14255,7 @@
       <x:c r="B8" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C8" s="29" t="n">
+      <x:c r="C8" s="32" t="n">
         <x:v>46088.5</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
@@ -14253,8 +14277,12 @@
       <x:c r="J8" s="23" t="str">
         <x:v>Estádio Beira-Rio, campos do Sesc, Vila Ventura e Ulbra</x:v>
       </x:c>
-      <x:c r="K8" s="8"/>
-      <x:c r="L8" s="8"/>
+      <x:c r="K8" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L8" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M8" s="23" t="str">
         <x:v>https://prefeitura.poa.br/secopa2027/noticias/copa-feminina-prefeitura-acompanha-vistoria-da-fifa-em-centros-de-treinamento</x:v>
       </x:c>
@@ -14275,7 +14303,7 @@
       <x:c r="B9" s="9" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C9" s="30" t="n">
+      <x:c r="C9" s="31" t="n">
         <x:v>46089.5</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
@@ -14297,8 +14325,12 @@
       <x:c r="J9" s="9" t="str">
         <x:v>Quadra 20, Trecho 3 da Orla do Guaíba</x:v>
       </x:c>
-      <x:c r="K9" s="12"/>
-      <x:c r="L9" s="12"/>
+      <x:c r="K9" s="12" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L9" s="12" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M9" s="9" t="str">
         <x:v>https://www.prefeitura.poa.br/secopa2027/noticias/gre-nal-feminino-pelo-dia-da-mulher-sera-no-trecho-3-da-orla-neste-domingo</x:v>
       </x:c>
@@ -14319,7 +14351,7 @@
       <x:c r="B10" s="9" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C10" s="30" t="n">
+      <x:c r="C10" s="31" t="n">
         <x:v>46091.5</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
@@ -14341,8 +14373,12 @@
       <x:c r="J10" s="9" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K10" s="12"/>
-      <x:c r="L10" s="12"/>
+      <x:c r="K10" s="12" t="n">
+        <x:v>-15.7939</x:v>
+      </x:c>
+      <x:c r="L10" s="12" t="n">
+        <x:v>-47.8828</x:v>
+      </x:c>
       <x:c r="M10" s="9" t="str">
         <x:v>https://www.gov.br/esporte/pt-br/noticias-e-conteudos/esporte/com-coordenacao-do-mesp-o-gecopa-comeca-a-tracar-primeiras-estrategias-e-desafios-para-a-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
@@ -14363,7 +14399,7 @@
       <x:c r="B11" s="9" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C11" s="30" t="n">
+      <x:c r="C11" s="31" t="n">
         <x:v>46109.5</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
@@ -14385,8 +14421,12 @@
       <x:c r="J11" s="9" t="str">
         <x:v>Areninha do José Walter e Areninha Sargento Hermínio</x:v>
       </x:c>
-      <x:c r="K11" s="12"/>
-      <x:c r="L11" s="12"/>
+      <x:c r="K11" s="12" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L11" s="12" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M11" s="9" t="str">
         <x:v>https://www.fortaleza.ce.gov.br/noticias/copa-feminina-guerreiras-do-sol-coloca-protagonismo-feminino-em-campo-nos-bairros-de-fortaleza</x:v>
       </x:c>
@@ -14407,7 +14447,7 @@
       <x:c r="B12" s="9" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C12" s="30" t="n">
+      <x:c r="C12" s="31" t="n">
         <x:v>46126.5</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
@@ -14451,7 +14491,7 @@
       <x:c r="B13" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C13" s="29" t="n">
+      <x:c r="C13" s="32" t="n">
         <x:v>46127.5</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
@@ -14473,8 +14513,12 @@
       <x:c r="J13" s="23" t="str">
         <x:v>Teatro Túlio Piva</x:v>
       </x:c>
-      <x:c r="K13" s="8"/>
-      <x:c r="L13" s="8"/>
+      <x:c r="K13" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L13" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M13" s="23" t="str">
         <x:v>https://prefeitura.poa.br/secopa2027/noticias/premio-elas-no-campo-sera-entregue-nesta-quarta-feira-na-capital</x:v>
       </x:c>
@@ -14495,7 +14539,7 @@
       <x:c r="B14" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C14" s="29" t="n">
+      <x:c r="C14" s="32" t="n">
         <x:v>46135.5</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
@@ -14517,8 +14561,12 @@
       <x:c r="J14" s="23" t="str">
         <x:v>SmartLab do Centro Administrativo Municipal</x:v>
       </x:c>
-      <x:c r="K14" s="8"/>
-      <x:c r="L14" s="8"/>
+      <x:c r="K14" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L14" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M14" s="23" t="str">
         <x:v>https://prefeitura.poa.br/secopa2027/noticias/copa-feminina-prefeitura-recebe-representantes-do-governo-federal-e-da-fifa</x:v>
       </x:c>
@@ -14539,7 +14587,7 @@
       <x:c r="B15" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C15" s="29" t="n">
+      <x:c r="C15" s="32" t="n">
         <x:v>46136.5</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
@@ -14561,8 +14609,12 @@
       <x:c r="J15" s="23" t="str">
         <x:v>Estádio Beira-Rio</x:v>
       </x:c>
-      <x:c r="K15" s="8"/>
-      <x:c r="L15" s="8"/>
+      <x:c r="K15" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L15" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M15" s="23" t="str">
         <x:v>https://www.gov.br/esporte/pt-br/noticias-e-conteudos/esporte/ministerio-do-esporte-inicia-visitas-tecnicas-aos-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
@@ -14583,7 +14635,7 @@
       <x:c r="B16" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C16" s="29" t="n">
+      <x:c r="C16" s="32" t="n">
         <x:v>46140.5</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
@@ -14627,7 +14679,7 @@
       <x:c r="B17" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C17" s="29" t="n">
+      <x:c r="C17" s="32" t="n">
         <x:v>46141.5</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
@@ -14649,8 +14701,12 @@
       <x:c r="J17" s="23" t="str">
         <x:v>Arena de Pernambuco e Bairro do Recife</x:v>
       </x:c>
-      <x:c r="K17" s="8"/>
-      <x:c r="L17" s="8"/>
+      <x:c r="K17" s="8" t="n">
+        <x:v>-8.0476</x:v>
+      </x:c>
+      <x:c r="L17" s="8" t="n">
+        <x:v>-34.877</x:v>
+      </x:c>
       <x:c r="M17" s="23" t="str">
         <x:v>https://www2.recife.pe.gov.br/noticias/29/04/2026/recife-apresenta-planejamento-para-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
@@ -14671,7 +14727,7 @@
       <x:c r="B18" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C18" s="29" t="n">
+      <x:c r="C18" s="32" t="n">
         <x:v>46147.5</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
@@ -14693,8 +14749,12 @@
       <x:c r="J18" s="23" t="str">
         <x:v>Arena Itaquera e Museu do Futebol</x:v>
       </x:c>
-      <x:c r="K18" s="8"/>
-      <x:c r="L18" s="8"/>
+      <x:c r="K18" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L18" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M18" s="23" t="str">
         <x:v>https://www.gov.br/esporte/pt-br/noticias-e-conteudos/esporte/arena-itaquera-recebe-ministerio-do-esporte-em-preparacao-para-a-copa-do-mundo-feminina-de-2027</x:v>
       </x:c>
@@ -14715,7 +14775,7 @@
       <x:c r="B19" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C19" s="29" t="n">
+      <x:c r="C19" s="32" t="n">
         <x:v>46149.5</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
@@ -14737,8 +14797,12 @@
       <x:c r="J19" s="23" t="str">
         <x:v>Centro de Operações e Resiliência do Rio</x:v>
       </x:c>
-      <x:c r="K19" s="8"/>
-      <x:c r="L19" s="8"/>
+      <x:c r="K19" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L19" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M19" s="23" t="str">
         <x:v>https://prefeitura.rio/casa-civil/prefeitura-do-rio-recebe-visita-tecnica-de-delegacoes-da-fifa-e-do-governo-federal/</x:v>
       </x:c>
@@ -14759,7 +14823,7 @@
       <x:c r="B20" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C20" s="29" t="n">
+      <x:c r="C20" s="32" t="n">
         <x:v>46150.5</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
@@ -14781,8 +14845,12 @@
       <x:c r="J20" s="23" t="str">
         <x:v>Centro de Eventos do Ceará</x:v>
       </x:c>
-      <x:c r="K20" s="8"/>
-      <x:c r="L20" s="8"/>
+      <x:c r="K20" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L20" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M20" s="23" t="str">
         <x:v>https://prefeitura.pbh.gov.br/noticias/belo-horizonte-tera-destaque-na-programacao-do-salao-nacional-do-turismo</x:v>
       </x:c>
@@ -14803,7 +14871,7 @@
       <x:c r="B21" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C21" s="29" t="n">
+      <x:c r="C21" s="32" t="n">
         <x:v>46153.5</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
@@ -14825,8 +14893,12 @@
       <x:c r="J21" s="23" t="str">
         <x:v>Mineirão</x:v>
       </x:c>
-      <x:c r="K21" s="8"/>
-      <x:c r="L21" s="8"/>
+      <x:c r="K21" s="8" t="n">
+        <x:v>-19.9167</x:v>
+      </x:c>
+      <x:c r="L21" s="8" t="n">
+        <x:v>-43.9345</x:v>
+      </x:c>
       <x:c r="M21" s="23" t="str">
         <x:v>https://prefeitura.pbh.gov.br/noticias/pbh-recebe-comitiva-da-fifa-e-ministerio-dos-esportes-como-preparacao-para-copa-feminina</x:v>
       </x:c>
@@ -14847,7 +14919,7 @@
       <x:c r="B22" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C22" s="29" t="n">
+      <x:c r="C22" s="32" t="n">
         <x:v>46155.5</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
@@ -14869,8 +14941,12 @@
       <x:c r="J22" s="23" t="str">
         <x:v>Espaço SmartLab do Centro Administrativo Municipal</x:v>
       </x:c>
-      <x:c r="K22" s="8"/>
-      <x:c r="L22" s="8"/>
+      <x:c r="K22" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L22" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M22" s="23" t="str">
         <x:v>https://prefeitura.poa.br/secopa2027/noticias/consulta-publica-debate-o-legado-da-copa-do-mundo-de-futebol-feminino-em-porto</x:v>
       </x:c>
@@ -14891,7 +14967,7 @@
       <x:c r="B23" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C23" s="29" t="n">
+      <x:c r="C23" s="32" t="n">
         <x:v>46155.5</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
@@ -14913,8 +14989,12 @@
       <x:c r="J23" s="23" t="str">
         <x:v>Arena Fonte Nova</x:v>
       </x:c>
-      <x:c r="K23" s="8"/>
-      <x:c r="L23" s="8"/>
+      <x:c r="K23" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L23" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M23" s="23" t="str">
         <x:v>https://salvador.ba.gov.br/prefeitura-apresenta-estrategias-para-copa-do-mundo-feminina-em-salvador-durante-encontro-com-a-fifa/</x:v>
       </x:c>
@@ -14935,7 +15015,7 @@
       <x:c r="B24" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C24" s="29" t="n">
+      <x:c r="C24" s="32" t="n">
         <x:v>46155.5</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
@@ -14957,8 +15037,12 @@
       <x:c r="J24" s="23" t="str">
         <x:v>Paço Municipal</x:v>
       </x:c>
-      <x:c r="K24" s="8"/>
-      <x:c r="L24" s="8"/>
+      <x:c r="K24" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L24" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M24" s="23" t="str">
         <x:v>https://www.fortaleza.ce.gov.br/noticias/prefeitura-de-fortaleza-recebe-representantes-da-fifa-para-planejamento-da-copa-do-mundo-feminina-de-2027</x:v>
       </x:c>
@@ -14979,7 +15063,7 @@
       <x:c r="B25" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C25" s="29" t="n">
+      <x:c r="C25" s="32" t="n">
         <x:v>46160.5</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
@@ -15001,8 +15085,12 @@
       <x:c r="J25" s="23" t="str">
         <x:v>Arena Castelão</x:v>
       </x:c>
-      <x:c r="K25" s="8"/>
-      <x:c r="L25" s="8"/>
+      <x:c r="K25" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L25" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M25" s="23" t="str">
         <x:v>https://mpce.mp.br/mp-do-ceara-acompanha-visita-tecnica-de-comitiva-do-ministerio-do-esporte-a-arena-castelao-em-preparacao-para-os-jogos-da-copa-do-mundo-feminina-2027/</x:v>
       </x:c>
@@ -15023,7 +15111,7 @@
       <x:c r="B26" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C26" s="29" t="n">
+      <x:c r="C26" s="32" t="n">
         <x:v>46160.5</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
@@ -15045,8 +15133,12 @@
       <x:c r="J26" s="23" t="str">
         <x:v>Paço Municipal, Arena Castelão e Aterro da Praia de Iracema</x:v>
       </x:c>
-      <x:c r="K26" s="8"/>
-      <x:c r="L26" s="8"/>
+      <x:c r="K26" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L26" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M26" s="23" t="str">
         <x:v>https://www.fortaleza.ce.gov.br/noticias/fortaleza-recebe-comitivas-da-fifa-governo-federal-e-governo-do-estado-para-alinhamento-da-copa-do-mundo-feminina-de-2027</x:v>
       </x:c>
@@ -15067,7 +15159,7 @@
       <x:c r="B27" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C27" s="29" t="n">
+      <x:c r="C27" s="32" t="n">
         <x:v>46162.5</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
@@ -15089,8 +15181,12 @@
       <x:c r="J27" s="23" t="str">
         <x:v>Ministério do Esporte e Estádio Nacional Mané Garrincha</x:v>
       </x:c>
-      <x:c r="K27" s="8"/>
-      <x:c r="L27" s="8"/>
+      <x:c r="K27" s="8" t="n">
+        <x:v>-15.7939</x:v>
+      </x:c>
+      <x:c r="L27" s="8" t="n">
+        <x:v>-47.8828</x:v>
+      </x:c>
       <x:c r="M27" s="23" t="str">
         <x:v>https://www.gov.br/esporte/pt-br/noticias-e-conteudos/esporte/ultima-cidade-a-receber-visita-tecnica-brasilia-avanca-no-planejamento-para-a-copa-do-mundo-de-futebol-feminino-2027</x:v>
       </x:c>
@@ -15111,7 +15207,7 @@
       <x:c r="B28" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C28" s="29" t="n">
+      <x:c r="C28" s="32" t="n">
         <x:v>46167.5</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
@@ -15133,8 +15229,12 @@
       <x:c r="J28" s="23" t="str">
         <x:v>Praça das Artes</x:v>
       </x:c>
-      <x:c r="K28" s="8"/>
-      <x:c r="L28" s="8"/>
+      <x:c r="K28" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L28" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M28" s="23" t="str">
         <x:v>https://prefeitura.sp.gov.br/web/turismo/w/prefeitura-de-s%C3%A3o-paulo-promove-encontro-sobre-futebol-feminino-e-copa-do-mundo</x:v>
       </x:c>
@@ -15155,7 +15255,7 @@
       <x:c r="B29" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C29" s="29" t="n">
+      <x:c r="C29" s="32" t="n">
         <x:v>46175.5</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
@@ -15199,7 +15299,7 @@
       <x:c r="B30" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C30" s="29" t="n">
+      <x:c r="C30" s="32" t="n">
         <x:v>46176.5</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
@@ -15221,8 +15321,12 @@
       <x:c r="J30" s="23" t="str">
         <x:v>Centro de Convenções de João Pessoa</x:v>
       </x:c>
-      <x:c r="K30" s="8"/>
-      <x:c r="L30" s="8"/>
+      <x:c r="K30" s="8" t="n">
+        <x:v>-7.115</x:v>
+      </x:c>
+      <x:c r="L30" s="8" t="n">
+        <x:v>-34.8641</x:v>
+      </x:c>
       <x:c r="M30" s="23" t="str">
         <x:v>https://brasil61.com/n/copa-feminina-de-2027-e-vista-como-oportunidade-para-ampliar-direitos-e-abrir-espacos-para-mulheres-mtur260027</x:v>
       </x:c>
@@ -15243,7 +15347,7 @@
       <x:c r="B31" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C31" s="29" t="n">
+      <x:c r="C31" s="32" t="n">
         <x:v>46182.5</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
@@ -15265,8 +15369,12 @@
       <x:c r="J31" s="23" t="str">
         <x:v>Arena Castelão</x:v>
       </x:c>
-      <x:c r="K31" s="8"/>
-      <x:c r="L31" s="8"/>
+      <x:c r="K31" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L31" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M31" s="23" t="str">
         <x:v>https://www.fortaleza.ce.gov.br/noticias/fortaleza-recebe-amistoso-entre-brasil-e-estados-unidos-e-registra-maior-publico-do-futebol-feminino-no-nordeste</x:v>
       </x:c>
@@ -15287,7 +15395,7 @@
       <x:c r="B32" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C32" s="29" t="n">
+      <x:c r="C32" s="32" t="n">
         <x:v>46183.5</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
@@ -15331,7 +15439,7 @@
       <x:c r="B33" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C33" s="29" t="n">
+      <x:c r="C33" s="32" t="n">
         <x:v>46185.5</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
@@ -15353,8 +15461,12 @@
       <x:c r="J33" s="23" t="str">
         <x:v>Rua Barão Rodrigues Mendes — Rua do Frevo</x:v>
       </x:c>
-      <x:c r="K33" s="8"/>
-      <x:c r="L33" s="8"/>
+      <x:c r="K33" s="8" t="n">
+        <x:v>-8.0476</x:v>
+      </x:c>
+      <x:c r="L33" s="8" t="n">
+        <x:v>-34.877</x:v>
+      </x:c>
       <x:c r="M33" s="23" t="str">
         <x:v>https://www2.recife.pe.gov.br/noticias/10/06/2026/recentro-promove-acao-na-rua-do-frevo-unindo-copa-do-mundo-e-o-periodo-junino</x:v>
       </x:c>
@@ -15375,7 +15487,7 @@
       <x:c r="B34" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C34" s="29" t="n">
+      <x:c r="C34" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
@@ -15397,8 +15509,12 @@
       <x:c r="J34" s="23" t="str">
         <x:v>Diversos espaços públicos, museus de Grêmio e Internacional e escolas municipais</x:v>
       </x:c>
-      <x:c r="K34" s="8"/>
-      <x:c r="L34" s="8"/>
+      <x:c r="K34" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L34" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M34" s="23" t="str">
         <x:v>https://www.prefeitura.poa.br/secopa2027/noticias/porto-alegre-entra-na-contagem-regressiva-de-um-ano-para-copa-do-mundo-feminina</x:v>
       </x:c>
@@ -15419,7 +15535,7 @@
       <x:c r="B35" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C35" s="29" t="n">
+      <x:c r="C35" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
@@ -15441,8 +15557,12 @@
       <x:c r="J35" s="23" t="str">
         <x:v>Cristo Redentor</x:v>
       </x:c>
-      <x:c r="K35" s="8"/>
-      <x:c r="L35" s="8"/>
+      <x:c r="K35" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L35" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M35" s="23" t="str">
         <x:v>https://blog.paineirascorcovado.com.br/2026/06/25/copa-do-mundo-feminina-2027-cristo-redentor/</x:v>
       </x:c>
@@ -15463,7 +15583,7 @@
       <x:c r="B36" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C36" s="29" t="n">
+      <x:c r="C36" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
@@ -15485,8 +15605,12 @@
       <x:c r="J36" s="23" t="str">
         <x:v>Monumento à Cidade do Salvador, Arcos da Montanha, Bambuzal do Aeroporto, estações do BRT, Casa do Olodum e sede da Prefeitura</x:v>
       </x:c>
-      <x:c r="K36" s="8"/>
-      <x:c r="L36" s="8"/>
+      <x:c r="K36" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L36" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M36" s="23" t="str">
         <x:v>https://salvador.ba.gov.br/salvador-celebra-marco-de-um-ano-para-a-copa-do-mundo-feminina-com-iluminacao-especial-em-monumentos-da-cidade/</x:v>
       </x:c>
@@ -15507,7 +15631,7 @@
       <x:c r="B37" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C37" s="29" t="n">
+      <x:c r="C37" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
@@ -15529,8 +15653,12 @@
       <x:c r="J37" s="23" t="str">
         <x:v>Paço Municipal, Ponte dos Ingleses e Arena Castelão</x:v>
       </x:c>
-      <x:c r="K37" s="8"/>
-      <x:c r="L37" s="8"/>
+      <x:c r="K37" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L37" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M37" s="23" t="str">
         <x:v>https://www.fortaleza.ce.gov.br/noticias/fortaleza-inicia-contagem-regressiva-de-um-ano-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027</x:v>
       </x:c>
@@ -15551,7 +15679,7 @@
       <x:c r="B38" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C38" s="29" t="n">
+      <x:c r="C38" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
@@ -15573,8 +15701,12 @@
       <x:c r="J38" s="23" t="str">
         <x:v>Boulevard da Rio Branco, pontes, monumentos e polos do São João</x:v>
       </x:c>
-      <x:c r="K38" s="8"/>
-      <x:c r="L38" s="8"/>
+      <x:c r="K38" s="8" t="n">
+        <x:v>-8.0476</x:v>
+      </x:c>
+      <x:c r="L38" s="8" t="n">
+        <x:v>-34.877</x:v>
+      </x:c>
       <x:c r="M38" s="23" t="str">
         <x:v>https://www2.recife.pe.gov.br/noticias/23/06/2026/recife-comeca-contagem-regressiva-para-copa-do-mundo-feminina-da-fifatm</x:v>
       </x:c>
@@ -15595,7 +15727,7 @@
       <x:c r="B39" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C39" s="29" t="n">
+      <x:c r="C39" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
@@ -15617,8 +15749,12 @@
       <x:c r="J39" s="23" t="str">
         <x:v>Estádio Nacional Mané Garrincha, Parque da Cidade e Rodoviária do Plano Piloto</x:v>
       </x:c>
-      <x:c r="K39" s="8"/>
-      <x:c r="L39" s="8"/>
+      <x:c r="K39" s="8" t="n">
+        <x:v>-15.7939</x:v>
+      </x:c>
+      <x:c r="L39" s="8" t="n">
+        <x:v>-47.8828</x:v>
+      </x:c>
       <x:c r="M39" s="23" t="str">
         <x:v>https://agenciabrasil.ebc.com.br/esportes/noticia/2026-06/brasilia-inicia-contagem-regressiva-de-1-ano-da-copa-do-mundo-feminina</x:v>
       </x:c>
@@ -15639,7 +15775,7 @@
       <x:c r="B40" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C40" s="29" t="n">
+      <x:c r="C40" s="32" t="n">
         <x:v>46197.5</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
@@ -15661,8 +15797,12 @@
       <x:c r="J40" s="23" t="str">
         <x:v>Fan Fest de Copacabana</x:v>
       </x:c>
-      <x:c r="K40" s="8"/>
-      <x:c r="L40" s="8"/>
+      <x:c r="K40" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L40" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M40" s="23" t="str">
         <x:v>https://prefeitura.rio/cidade/pioneiras-da-selecao-feminina-de-futebol-promovem-o-mundial-com-acao-em-copacabana/</x:v>
       </x:c>
@@ -15683,7 +15823,7 @@
       <x:c r="B41" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C41" s="29" t="n">
+      <x:c r="C41" s="32" t="n">
         <x:v>46199.5</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
@@ -15727,7 +15867,7 @@
       <x:c r="B42" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C42" s="29" t="n">
+      <x:c r="C42" s="32" t="n">
         <x:v>46199.5</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
@@ -15749,8 +15889,12 @@
       <x:c r="J42" s="23" t="str">
         <x:v>Online</x:v>
       </x:c>
-      <x:c r="K42" s="8"/>
-      <x:c r="L42" s="8"/>
+      <x:c r="K42" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L42" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M42" s="23" t="str">
         <x:v>https://prefeitura.sp.gov.br/web/turismo/l/48770028</x:v>
       </x:c>
@@ -15771,7 +15915,7 @@
       <x:c r="B43" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C43" s="29" t="n">
+      <x:c r="C43" s="32" t="n">
         <x:v>46205.5</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
@@ -15815,7 +15959,7 @@
       <x:c r="B44" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C44" s="29" t="n">
+      <x:c r="C44" s="32" t="n">
         <x:v>46211.5</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
@@ -15837,8 +15981,12 @@
       <x:c r="J44" s="23" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K44" s="8"/>
-      <x:c r="L44" s="8"/>
+      <x:c r="K44" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L44" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M44" s="23" t="str">
         <x:v>https://agenciadenoticias.salvador.ba.gov.br/index.php/pt-br/releases-2/geral/30922-governanca-integrada-marca-reuniao-da-prefeitura-para-planejamento-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
@@ -15859,7 +16007,7 @@
       <x:c r="B45" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C45" s="29" t="n">
+      <x:c r="C45" s="32" t="n">
         <x:v>46219.5</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
@@ -15903,7 +16051,7 @@
       <x:c r="B46" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C46" s="29" t="n">
+      <x:c r="C46" s="32" t="n">
         <x:v>46230.5</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
@@ -15947,7 +16095,7 @@
       <x:c r="B47" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C47" s="29" t="n">
+      <x:c r="C47" s="32" t="n">
         <x:v>46232.5</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
@@ -15969,8 +16117,12 @@
       <x:c r="J47" s="23" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K47" s="8"/>
-      <x:c r="L47" s="8"/>
+      <x:c r="K47" s="8" t="n">
+        <x:v>-3.7319</x:v>
+      </x:c>
+      <x:c r="L47" s="8" t="n">
+        <x:v>-38.5267</x:v>
+      </x:c>
       <x:c r="M47" s="23" t="str">
         <x:v>https://mpce.mp.br/mp-do-ceara-e-representante-da-fifa-se-reunem-para-alinhar-parceria-para-a-copa-do-mundo-feminina-de-2027/</x:v>
       </x:c>
@@ -15991,7 +16143,7 @@
       <x:c r="B48" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C48" s="29" t="n">
+      <x:c r="C48" s="32" t="n">
         <x:v>46235.5</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
@@ -16013,8 +16165,12 @@
       <x:c r="J48" s="23" t="str">
         <x:v>Casa Mãe Paulistana para Mães e Cuidadores de Pessoas com Deficiência</x:v>
       </x:c>
-      <x:c r="K48" s="8"/>
-      <x:c r="L48" s="8"/>
+      <x:c r="K48" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L48" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M48" s="23" t="str">
         <x:v>https://prefeitura.sp.gov.br/web/pessoa_com_deficiencia/w/copa-do-mundo-2026-prefeitura-de-s%C3%A3o-paulo-promove-a%C3%A7%C3%B5es-inclusivas-para-pessoas-com-defici%C3%AAncia-e-seus-familiares</x:v>
       </x:c>
@@ -16035,7 +16191,7 @@
       <x:c r="B49" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C49" s="29" t="n">
+      <x:c r="C49" s="32" t="n">
         <x:v>46237.5</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
@@ -16057,8 +16213,12 @@
       <x:c r="J49" s="23" t="str">
         <x:v>Museu do Futebol</x:v>
       </x:c>
-      <x:c r="K49" s="8"/>
-      <x:c r="L49" s="8"/>
+      <x:c r="K49" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L49" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M49" s="23" t="str">
         <x:v>https://www.sympla.com.br/evento/forum-sustentabilidade-em-campo/3498582</x:v>
       </x:c>
@@ -16079,7 +16239,7 @@
       <x:c r="B50" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C50" s="29" t="n">
+      <x:c r="C50" s="32" t="n">
         <x:v>46238.5</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
@@ -16127,7 +16287,7 @@
       <x:c r="B51" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C51" s="29" t="n">
+      <x:c r="C51" s="32" t="n">
         <x:v>46238.5</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
@@ -16149,8 +16309,12 @@
       <x:c r="J51" s="23" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K51" s="8"/>
-      <x:c r="L51" s="8"/>
+      <x:c r="K51" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L51" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M51" s="23" t="str">
         <x:v>https://secult.salvador.ba.gov.br/prefeitura-se-reune-com-clubes-federacao-atletas-e-entidades-para-debater-legado-social-da-copa-do-mundo-feminina-da-fifa-2027/</x:v>
       </x:c>
@@ -16171,7 +16335,7 @@
       <x:c r="B52" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C52" s="29" t="n">
+      <x:c r="C52" s="32" t="n">
         <x:v>46238.5</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
@@ -16193,8 +16357,12 @@
       <x:c r="J52" s="23" t="str">
         <x:v>Rio Innovation Week</x:v>
       </x:c>
-      <x:c r="K52" s="8"/>
-      <x:c r="L52" s="8"/>
+      <x:c r="K52" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L52" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M52" s="23" t="str">
         <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/04/diretor-da-copa-2027-revela-que-730-mil-pessoas-ja-mostraram-interesse-em-comprar-ingressos-a-gente-vai-encher-estadio.ghtml</x:v>
       </x:c>
@@ -16215,7 +16383,7 @@
       <x:c r="B53" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C53" s="29" t="n">
+      <x:c r="C53" s="32" t="n">
         <x:v>46241.5</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
@@ -16263,7 +16431,7 @@
       <x:c r="B54" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C54" s="29" t="n">
+      <x:c r="C54" s="32" t="n">
         <x:v>46243.5</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
@@ -16313,7 +16481,7 @@
       <x:c r="B55" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C55" s="29" t="n">
+      <x:c r="C55" s="32" t="n">
         <x:v>46245.5</x:v>
       </x:c>
       <x:c r="D55" s="23" t="str">
@@ -16335,8 +16503,12 @@
       <x:c r="J55" s="23" t="str">
         <x:v>Teatro Nacional Cláudio Santoro</x:v>
       </x:c>
-      <x:c r="K55" s="8"/>
-      <x:c r="L55" s="8"/>
+      <x:c r="K55" s="8" t="n">
+        <x:v>-15.7939</x:v>
+      </x:c>
+      <x:c r="L55" s="8" t="n">
+        <x:v>-47.8828</x:v>
+      </x:c>
       <x:c r="M55" s="23" t="str">
         <x:v>https://elasemacao.com/</x:v>
       </x:c>
@@ -16357,7 +16529,7 @@
       <x:c r="B56" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C56" s="29" t="n">
+      <x:c r="C56" s="32" t="n">
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="D56" s="23" t="str">
@@ -16379,8 +16551,12 @@
       <x:c r="J56" s="23" t="str">
         <x:v>Sede da FGF e Esefid/UFRGS</x:v>
       </x:c>
-      <x:c r="K56" s="8"/>
-      <x:c r="L56" s="8"/>
+      <x:c r="K56" s="8" t="n">
+        <x:v>-30.0346</x:v>
+      </x:c>
+      <x:c r="L56" s="8" t="n">
+        <x:v>-51.2177</x:v>
+      </x:c>
       <x:c r="M56" s="23" t="str">
         <x:v>https://prefeitura.poa.br/secopa2027/noticias/seminario-mulheres-em-campo-ocorre-nesta-sexta-feira</x:v>
       </x:c>
@@ -16401,7 +16577,7 @@
       <x:c r="B57" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C57" s="29" t="n">
+      <x:c r="C57" s="32" t="n">
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="D57" s="23" t="str">
@@ -16449,7 +16625,7 @@
       <x:c r="B58" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C58" s="29" t="n">
+      <x:c r="C58" s="32" t="n">
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="D58" s="23" t="str">
@@ -16471,8 +16647,12 @@
       <x:c r="J58" s="23" t="str">
         <x:v>Sede da FIFA, Zurique / transmissão online</x:v>
       </x:c>
-      <x:c r="K58" s="8"/>
-      <x:c r="L58" s="8"/>
+      <x:c r="K58" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L58" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M58" s="23" t="str">
         <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
@@ -16493,7 +16673,7 @@
       <x:c r="B59" s="23" t="str">
         <x:v>Realizado</x:v>
       </x:c>
-      <x:c r="C59" s="29" t="n">
+      <x:c r="C59" s="32" t="n">
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="D59" s="23" t="str">
@@ -16541,7 +16721,7 @@
       <x:c r="B60" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C60" s="29" t="n">
+      <x:c r="C60" s="32" t="n">
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="D60" s="23" t="str">
@@ -16589,7 +16769,7 @@
       <x:c r="B61" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C61" s="29" t="n">
+      <x:c r="C61" s="32" t="n">
         <x:v>46264.5</x:v>
       </x:c>
       <x:c r="D61" s="23" t="str">
@@ -16611,8 +16791,12 @@
       <x:c r="J61" s="23" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K61" s="8"/>
-      <x:c r="L61" s="8"/>
+      <x:c r="K61" s="8" t="n">
+        <x:v>-12.9777</x:v>
+      </x:c>
+      <x:c r="L61" s="8" t="n">
+        <x:v>-38.5016</x:v>
+      </x:c>
       <x:c r="M61" s="23" t="str">
         <x:v>https://comunicacao.salvador.ba.gov.br/prefeitura-lanca-copa-salvador-interbairros-2026-com-40-times-e-participacao-inedita-de-equipes-femininas/</x:v>
       </x:c>
@@ -16633,7 +16817,7 @@
       <x:c r="B62" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C62" s="29" t="n">
+      <x:c r="C62" s="32" t="n">
         <x:v>46270.5</x:v>
       </x:c>
       <x:c r="D62" s="23" t="str">
@@ -16677,7 +16861,7 @@
       <x:c r="B63" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C63" s="29" t="n">
+      <x:c r="C63" s="32" t="n">
         <x:v>46273.5</x:v>
       </x:c>
       <x:c r="D63" s="23" t="str">
@@ -16721,7 +16905,7 @@
       <x:c r="B64" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C64" s="29" t="n">
+      <x:c r="C64" s="32" t="n">
         <x:v>46279.5</x:v>
       </x:c>
       <x:c r="D64" s="23" t="str">
@@ -16769,7 +16953,7 @@
       <x:c r="B65" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C65" s="29" t="n">
+      <x:c r="C65" s="32" t="n">
         <x:v>46284.5</x:v>
       </x:c>
       <x:c r="D65" s="23" t="str">
@@ -16791,8 +16975,12 @@
       <x:c r="J65" s="23" t="str">
         <x:v>Praça Tiradentes — ponto de encontro em frente ao VLT</x:v>
       </x:c>
-      <x:c r="K65" s="8"/>
-      <x:c r="L65" s="8"/>
+      <x:c r="K65" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L65" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M65" s="23" t="str">
         <x:v>https://www.sympla.com.br/evento/historia-do-futebol-feminino-no-rio/3546698</x:v>
       </x:c>
@@ -16813,7 +17001,7 @@
       <x:c r="B66" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C66" s="29" t="n">
+      <x:c r="C66" s="32" t="n">
         <x:v>46287.5</x:v>
       </x:c>
       <x:c r="D66" s="23" t="str">
@@ -16835,8 +17023,12 @@
       <x:c r="J66" s="23" t="str">
         <x:v>Granja Comary</x:v>
       </x:c>
-      <x:c r="K66" s="8"/>
-      <x:c r="L66" s="8"/>
+      <x:c r="K66" s="8" t="n">
+        <x:v>-22.4167</x:v>
+      </x:c>
+      <x:c r="L66" s="8" t="n">
+        <x:v>-42.9782</x:v>
+      </x:c>
       <x:c r="M66" s="23" t="str">
         <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
       </x:c>
@@ -16857,7 +17049,7 @@
       <x:c r="B67" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C67" s="29" t="n">
+      <x:c r="C67" s="32" t="n">
         <x:v>46298.5</x:v>
       </x:c>
       <x:c r="D67" s="23" t="str">
@@ -16879,8 +17071,12 @@
       <x:c r="J67" s="23" t="str">
         <x:v>Pro Magno Centro de Eventos</x:v>
       </x:c>
-      <x:c r="K67" s="8"/>
-      <x:c r="L67" s="8"/>
+      <x:c r="K67" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L67" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M67" s="23" t="str">
         <x:v>https://cobexpo.soudaliga.com.br/reserva?date=2026-10-03&amp;id=22500&amp;nextInternalLocale=pt-BR</x:v>
       </x:c>
@@ -16901,7 +17097,7 @@
       <x:c r="B68" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C68" s="29" t="n">
+      <x:c r="C68" s="32" t="n">
         <x:v>46300.5</x:v>
       </x:c>
       <x:c r="D68" s="23" t="str">
@@ -16945,7 +17141,7 @@
       <x:c r="B69" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C69" s="29" t="n">
+      <x:c r="C69" s="32" t="n">
         <x:v>46300.5</x:v>
       </x:c>
       <x:c r="D69" s="23" t="str">
@@ -16989,7 +17185,7 @@
       <x:c r="B70" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C70" s="29" t="n">
+      <x:c r="C70" s="32" t="n">
         <x:v>46312.5</x:v>
       </x:c>
       <x:c r="D70" s="23" t="str">
@@ -17033,7 +17229,7 @@
       <x:c r="B71" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C71" s="29" t="n">
+      <x:c r="C71" s="32" t="n">
         <x:v>46340.5</x:v>
       </x:c>
       <x:c r="D71" s="23" t="str">
@@ -17077,7 +17273,7 @@
       <x:c r="B72" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C72" s="29" t="n">
+      <x:c r="C72" s="32" t="n">
         <x:v>46341.5</x:v>
       </x:c>
       <x:c r="D72" s="23" t="str">
@@ -17101,8 +17297,12 @@
       <x:c r="J72" s="23" t="str">
         <x:v>Local a definir</x:v>
       </x:c>
-      <x:c r="K72" s="8"/>
-      <x:c r="L72" s="8"/>
+      <x:c r="K72" s="8" t="n">
+        <x:v>-23.5505</x:v>
+      </x:c>
+      <x:c r="L72" s="8" t="n">
+        <x:v>-46.6333</x:v>
+      </x:c>
       <x:c r="M72" s="23" t="str">
         <x:v>https://www.ebc.com.br/premiotvbrasilpetrobrasparaelas/</x:v>
       </x:c>
@@ -17123,7 +17323,7 @@
       <x:c r="B73" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C73" s="29" t="n">
+      <x:c r="C73" s="32" t="n">
         <x:v>46350.5</x:v>
       </x:c>
       <x:c r="D73" s="23" t="str">
@@ -17167,7 +17367,7 @@
       <x:c r="B74" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C74" s="29" t="n">
+      <x:c r="C74" s="32" t="n">
         <x:v>46350.5</x:v>
       </x:c>
       <x:c r="D74" s="23" t="str">
@@ -17211,7 +17411,7 @@
       <x:c r="B75" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C75" s="29" t="n">
+      <x:c r="C75" s="32" t="n">
         <x:v>46357.5</x:v>
       </x:c>
       <x:c r="D75" s="23" t="str">
@@ -17255,7 +17455,7 @@
       <x:c r="B76" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C76" s="29" t="n">
+      <x:c r="C76" s="32" t="n">
         <x:v>46362.5</x:v>
       </x:c>
       <x:c r="D76" s="23" t="str">
@@ -17299,7 +17499,7 @@
       <x:c r="B77" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C77" s="29" t="n">
+      <x:c r="C77" s="32" t="n">
         <x:v>46367.5</x:v>
       </x:c>
       <x:c r="D77" s="23" t="str">
@@ -17321,8 +17521,12 @@
       <x:c r="J77" s="23" t="str">
         <x:v>Museu de Arte Moderna do Rio de Janeiro (MAM Rio)</x:v>
       </x:c>
-      <x:c r="K77" s="8"/>
-      <x:c r="L77" s="8"/>
+      <x:c r="K77" s="8" t="n">
+        <x:v>-22.9068</x:v>
+      </x:c>
+      <x:c r="L77" s="8" t="n">
+        <x:v>-43.1729</x:v>
+      </x:c>
       <x:c r="M77" s="23" t="str">
         <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/sorteio-grupos-copa-mundo-feminina-2027-data-local</x:v>
       </x:c>
@@ -17343,7 +17547,7 @@
       <x:c r="B78" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C78" s="29" t="n">
+      <x:c r="C78" s="32" t="n">
         <x:v>46444.5</x:v>
       </x:c>
       <x:c r="D78" s="23" t="str">
@@ -17387,7 +17591,7 @@
       <x:c r="B79" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C79" s="6" t="n">
+      <x:c r="C79" s="32" t="n">
         <x:v>46478.5</x:v>
       </x:c>
       <x:c r="D79" s="23" t="str">
@@ -17431,7 +17635,7 @@
       <x:c r="B80" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C80" s="6" t="n">
+      <x:c r="C80" s="32" t="n">
         <x:v>46482.5</x:v>
       </x:c>
       <x:c r="D80" s="23" t="str">
@@ -17475,7 +17679,7 @@
       <x:c r="B81" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C81" s="6" t="n">
+      <x:c r="C81" s="32" t="n">
         <x:v>46508.5</x:v>
       </x:c>
       <x:c r="D81" s="23" t="str">
@@ -17523,7 +17727,7 @@
       <x:c r="B82" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C82" s="6" t="n">
+      <x:c r="C82" s="32" t="n">
         <x:v>46548.5</x:v>
       </x:c>
       <x:c r="D82" s="23" t="str">
@@ -17571,7 +17775,7 @@
       <x:c r="B83" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C83" s="6" t="n">
+      <x:c r="C83" s="32" t="n">
         <x:v>46562.5</x:v>
       </x:c>
       <x:c r="D83" s="23" t="str">
@@ -17619,7 +17823,7 @@
       <x:c r="B84" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C84" s="6" t="n">
+      <x:c r="C84" s="32" t="n">
         <x:v>46567.5</x:v>
       </x:c>
       <x:c r="D84" s="23" t="str">
@@ -17667,7 +17871,7 @@
       <x:c r="B85" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C85" s="6" t="n">
+      <x:c r="C85" s="32" t="n">
         <x:v>46572.5</x:v>
       </x:c>
       <x:c r="D85" s="23" t="str">
@@ -17715,7 +17919,7 @@
       <x:c r="B86" s="23" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="C86" s="6" t="n">
+      <x:c r="C86" s="32" t="n">
         <x:v>46593.5</x:v>
       </x:c>
       <x:c r="D86" s="23" t="str">
@@ -25227,7 +25431,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb336a315fb5141d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R688bbb8965a64817"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27127,7 +27331,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8f941b3bc004fac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f68e7d2ddb64dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27539,7 +27743,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R276e2cc0cb334de2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3ce8d3db0a04f0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28792,22 +28996,22 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28816,65 +29020,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -28882,19 +29086,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28903,7 +29107,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -28911,98 +29115,116 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I49" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B50" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C50" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D50" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E50" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F50" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G50" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H50" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I49" s="23" t="str">
+      <x:c r="I50" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="6"/>
-      <x:c r="B50" s="23"/>
-      <x:c r="C50" s="23"/>
-      <x:c r="D50" s="23"/>
-      <x:c r="E50" s="23"/>
-      <x:c r="F50" s="23"/>
-      <x:c r="G50" s="23"/>
-      <x:c r="H50" s="23"/>
-      <x:c r="I50" s="23"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="6"/>
@@ -33965,7 +34187,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1fe54999234fb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc8d3998c7314bce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34868,7 +35090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1d9b2499de4170"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R674efaa89eb44052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35747,7 +35969,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27919c11276b4812"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf17dad092a3435f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36170,7 +36392,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R429624e07a714744"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1567f1d39a074ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Registra lei federal de incentivos para a Copa 2027
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R9f59f917a7ae4f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R94ce25a44a484789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra7653faececa4f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R8234ec856190452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rcce12723b8994846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R7ed10c04f5374ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R82349b1acb43411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rae6499f742fd44f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R4d447be74d124f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R886400e58e1a41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R8678266995a740d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R5d7c166313404f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R585abe31d51f4777"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rff6607b50e05440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rb6d48e8941fc44ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Ra8a66bf09da743be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rb533308b67ee4d07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R9e6d7aa270a949ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R2cab5dfd23754f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R85075fb254f34e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra8f4c50aecbc45ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Reff91232f81a43fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R4afcbd51d35741c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R51c512d25e764497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R2f06728f434f4188"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R60056d2be9fe4c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R45dfb465813943d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rdcd9ce3f24bd4b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Ra0252cfe2b5f4dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R346326940cb24a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R271d1403db894c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R88695e06611a410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rf416b4fcf7e8476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rb278c3fcad874ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rd177a393f3154bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R11de46526e364991"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R357bd8c49ac242a2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R604a7a5c35c24be7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R97c44043c16c4b7c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08cc29fe6477486f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b630ddbd34c453f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1309e7e495c46f5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a2ebc6478c24d80"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00db17bb80864332"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfeff37e56134594"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e4e84cf14a74626"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1387,8 +1387,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I50"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I51"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2964,7 +2964,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761e11be19f84e0a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e85aa5eb10a419c"/>
 </x:worksheet>
 </file>
 
@@ -5253,7 +5253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f763ca9ea954b19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e8e5867bb0b42b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7561,7 +7561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ad4b5ccada489c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7e058aaf3647e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8193,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdb3bc2aa4a4cb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ef18f283d7444a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12383,9 +12383,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9def725010284156"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a80fc0b727b4da9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red56c1a37d9b4eac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5229c9297fb4eb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12676,7 +12676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53c5acfe7404452"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dc6752812dc4585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25431,7 +25431,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R688bbb8965a64817"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc81867437e414d40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27331,7 +27331,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f68e7d2ddb64dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d76da1710634002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27743,7 +27743,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3ce8d3db0a04f0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d69d5455694900"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27836,31 +27836,31 @@
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
       <x:c r="A3" s="31" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27868,28 +27868,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27897,28 +27897,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27926,19 +27926,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27947,7 +27947,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27955,57 +27955,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -28013,28 +28013,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28042,28 +28042,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -28071,19 +28071,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28092,7 +28092,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28100,28 +28100,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -28129,57 +28129,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
         <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28187,28 +28187,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28216,28 +28216,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28245,19 +28245,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28266,7 +28266,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28274,57 +28274,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28332,28 +28332,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28361,19 +28361,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28382,7 +28382,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28390,19 +28390,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28411,7 +28411,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28419,19 +28419,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28440,7 +28440,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28448,48 +28448,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28498,7 +28498,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28506,19 +28506,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28527,56 +28527,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28585,36 +28585,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28622,19 +28622,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28643,7 +28643,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28651,28 +28651,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28680,28 +28680,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28709,48 +28709,48 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28759,7 +28759,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28767,28 +28767,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28796,48 +28796,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28846,36 +28846,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28883,28 +28883,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -28912,57 +28912,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -28970,28 +28970,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -28999,48 +28999,48 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29049,65 +29049,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -29115,19 +29115,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29136,7 +29136,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -29144,98 +29144,116 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H50" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I50" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B51" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C51" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G51" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H51" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I50" s="23" t="str">
+      <x:c r="I51" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="6"/>
-      <x:c r="B51" s="23"/>
-      <x:c r="C51" s="23"/>
-      <x:c r="D51" s="23"/>
-      <x:c r="E51" s="23"/>
-      <x:c r="F51" s="23"/>
-      <x:c r="G51" s="23"/>
-      <x:c r="H51" s="23"/>
-      <x:c r="I51" s="23"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="6"/>
@@ -34187,7 +34205,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc8d3998c7314bce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdebdd6c8313468c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35090,7 +35108,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R674efaa89eb44052"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6b4b4c82eaa4e58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35969,7 +35987,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf17dad092a3435f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe93abce8efa4173"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36392,7 +36410,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1567f1d39a074ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97e2ec6009354271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona balanço dos 300 dias para a Copa Feminina
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rf803a815c21f4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rf8dd54894e84428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Rafb67a7b3ca54f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rbdb6fc4ee555476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R05c1287c3cea4ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R10b0f999a33b4d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R77d9b10451264f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Raadba24883aa46ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rcd60d85838b94962"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R929f1e80a9a24599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R7749612eea75480f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rc6a98e1b29284682"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R76fb9868c1424370"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R69f57993cd964143"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Rbdf630231bc74df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rfa3201a120644844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rf51e9125e0cf4fca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R595a2b0d72db45d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rec8bcce443e5450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R39b0de9a7e124948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R16b6314b888c445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rcdce99ff67744661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rf679b4c7b91b44dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R0f039ad4d5784c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Ra89a959cdd36488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rf161b87c1f39474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R725b73f9c28148a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R54dddcacdc1248ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rae137334d62b4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Ra68f7af1f0454e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R33689d4bebf94e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R54b36db585754054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R3efbfa255411482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rb1e867a590cc4e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rf705367522f54ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Ra213048fe6f3401b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3094a9e263ea4e56"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78ab5cd438aa49c8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67a4ec60fd434c57"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e766663772540f9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5b5cf16fac5148c9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R974e33877e384246"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1fe2743846549f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfda08c2eef6d460f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5787647a1084790"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2327bfabc12443df"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1273,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="EventosTable" displayName="EventosTable" ref="A1:P87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="EventosTable" displayName="EventosTable" ref="A1:P87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:P87"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="ID"/>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I52"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I53"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2965,7 +2965,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ffb46e841b4981"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf8c14bc90494af1"/>
 </x:worksheet>
 </file>
 
@@ -5254,7 +5254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd69a51dec44a41ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf611bfed0a704b7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7562,7 +7562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2cc4ead476498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48bd2afa1fc94a6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8194,7 +8194,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0fbceb7b36e4efc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1168f8d59cea4b26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12384,9 +12384,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92d05abac08040c2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5cab28c69264be7"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c32e7f849f44ad2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40481260b186446a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12677,7 +12677,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11f41e16f26f4422"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5110d7c703244add"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25464,7 +25464,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75a0bda415b2455b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cb704ffb534c2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27366,7 +27366,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b04894f91db4f8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d95e66ac3b4cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27778,7 +27778,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62fd43897c774292"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a7d3b67fc9402d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27900,31 +27900,31 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
       <x:c r="A4" s="31" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27932,28 +27932,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27961,19 +27961,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27982,7 +27982,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27990,28 +27990,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -28019,57 +28019,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28077,28 +28077,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -28106,19 +28106,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28127,7 +28127,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28135,19 +28135,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28156,7 +28156,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -28164,10 +28164,10 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28176,7 +28176,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28185,7 +28185,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -28193,19 +28193,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28214,7 +28214,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28222,57 +28222,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28280,28 +28280,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28309,19 +28309,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28330,7 +28330,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28338,28 +28338,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28367,57 +28367,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28425,28 +28425,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28454,19 +28454,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28475,7 +28475,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28483,19 +28483,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28504,7 +28504,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28512,19 +28512,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28533,7 +28533,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28541,48 +28541,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28591,7 +28591,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28599,19 +28599,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28620,56 +28620,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28678,27 +28678,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28707,7 +28707,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28715,28 +28715,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28744,28 +28744,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28773,28 +28773,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28802,19 +28802,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28823,36 +28823,36 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28860,28 +28860,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28889,48 +28889,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28939,27 +28939,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28968,7 +28968,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -28976,28 +28976,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -29005,57 +29005,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -29063,28 +29063,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -29092,48 +29092,48 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29142,65 +29142,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -29208,28 +29208,28 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -29237,19 +29237,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29258,77 +29258,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H51" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H52" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I52" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B53" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C53" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D53" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E53" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F53" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G53" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H53" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I52" s="23" t="str">
+      <x:c r="I53" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="6"/>
-      <x:c r="B53" s="23"/>
-      <x:c r="C53" s="23"/>
-      <x:c r="D53" s="23"/>
-      <x:c r="E53" s="23"/>
-      <x:c r="F53" s="23"/>
-      <x:c r="G53" s="23"/>
-      <x:c r="H53" s="23"/>
-      <x:c r="I53" s="23"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="6"/>
@@ -34258,7 +34276,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b0a7b539e2e4d76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eabc698a9b74f5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35161,7 +35179,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4faf086b94f45e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff7b8fb3adc405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36040,7 +36058,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R280d2da1e74b4fef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53af5a93753047aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36463,7 +36481,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85cedcdc26bd4f2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7503714b68d4a1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona perfil de Dulce na preparação da Seleção Sub-20
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rec8bcce443e5450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R39b0de9a7e124948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R16b6314b888c445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rcdce99ff67744661"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Rf679b4c7b91b44dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R0f039ad4d5784c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Ra89a959cdd36488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rf161b87c1f39474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R725b73f9c28148a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R54dddcacdc1248ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rae137334d62b4b4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Ra68f7af1f0454e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R33689d4bebf94e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R54b36db585754054"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R3efbfa255411482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Rb1e867a590cc4e2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rf705367522f54ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Ra213048fe6f3401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Ra561df00130145fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R29ed48603e1a45a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R857c05633d5342d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R78078d43dd5741bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Ra6722923958e409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R41436bf19cd24e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R19b46ece652f4d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5600c36b7a814c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R0efbb85324854636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rd81135fcc87445a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R1a151bd1be604181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Re93cdb4950e74016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Red0861c15f304d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Ree5a773d36a5410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R298bd89532994ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R74e27c9a4b8341c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R539343f9b68d45dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rcc9231434de145ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78ab5cd438aa49c8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R07478ee323434772"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e766663772540f9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf226723e322b4720"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R974e33877e384246"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7aa1f17236e746fd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfda08c2eef6d460f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb34c6dc6f152463b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2327bfabc12443df"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6044e42006244e5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1273,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="EventosTable" displayName="EventosTable" ref="A1:P87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="EventosTable" displayName="EventosTable" ref="A1:P87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:P87"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="ID"/>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I53"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I54"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2965,7 +2965,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf8c14bc90494af1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc9076d4c8a4ef7"/>
 </x:worksheet>
 </file>
 
@@ -5254,7 +5254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf611bfed0a704b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5af58a790c9c4975"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7562,7 +7562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48bd2afa1fc94a6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf6b712641674406"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8194,7 +8194,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1168f8d59cea4b26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d9820ddcd04f6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12384,9 +12384,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5cab28c69264be7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R129aaaf22eda4c47"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40481260b186446a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3730911242c94f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12677,7 +12677,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5110d7c703244add"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc99a3b580ab842ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25464,7 +25464,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cb704ffb534c2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51b647b5460b47e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27366,7 +27366,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d95e66ac3b4cfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8bb353882a04cdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27778,7 +27778,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a7d3b67fc9402d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1209689d39a0481c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27845,19 +27845,19 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
+        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Empetur</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27866,7 +27866,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
+        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
@@ -27874,28 +27874,28 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Tributação / legislação federal / organização</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Presidência da República</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27903,57 +27903,57 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
       <x:c r="A5" s="31" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27961,28 +27961,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27990,19 +27990,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28011,7 +28011,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -28019,28 +28019,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -28048,57 +28048,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -28106,28 +28106,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28135,19 +28135,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28156,7 +28156,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -28164,19 +28164,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28185,7 +28185,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -28193,10 +28193,10 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28205,7 +28205,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28214,7 +28214,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28222,19 +28222,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28243,7 +28243,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28251,57 +28251,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28309,28 +28309,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28338,19 +28338,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28359,7 +28359,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28367,28 +28367,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28396,57 +28396,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28454,28 +28454,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28483,19 +28483,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28504,7 +28504,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28512,19 +28512,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28533,7 +28533,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28541,19 +28541,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28562,7 +28562,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28570,48 +28570,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28620,7 +28620,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28628,19 +28628,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28649,56 +28649,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28707,27 +28707,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28736,7 +28736,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28744,28 +28744,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28773,28 +28773,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28802,28 +28802,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28831,19 +28831,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28852,36 +28852,36 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28889,28 +28889,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28918,48 +28918,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28968,27 +28968,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28997,7 +28997,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -29005,28 +29005,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -29034,57 +29034,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -29092,28 +29092,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -29121,48 +29121,48 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29171,65 +29171,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -29237,28 +29237,28 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H50" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -29266,19 +29266,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29287,77 +29287,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H52" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I52" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C53" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G53" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H53" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I53" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="32" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B54" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C54" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D54" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E54" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F54" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G54" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H54" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I53" s="23" t="str">
+      <x:c r="I54" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="6"/>
-      <x:c r="B54" s="23"/>
-      <x:c r="C54" s="23"/>
-      <x:c r="D54" s="23"/>
-      <x:c r="E54" s="23"/>
-      <x:c r="F54" s="23"/>
-      <x:c r="G54" s="23"/>
-      <x:c r="H54" s="23"/>
-      <x:c r="I54" s="23"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="6"/>
@@ -34276,7 +34294,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eabc698a9b74f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5227dcb0e014aa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35179,7 +35197,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff7b8fb3adc405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bacbfa5c0eb4d84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36058,7 +36076,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53af5a93753047aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03a800b2731c4bfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36481,7 +36499,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7503714b68d4a1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205abe9956c94dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona avanços de Fortaleza para a Copa 2027
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Ra561df00130145fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R29ed48603e1a45a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R857c05633d5342d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R78078d43dd5741bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Ra6722923958e409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R41436bf19cd24e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R19b46ece652f4d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5600c36b7a814c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R0efbb85324854636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rd81135fcc87445a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R1a151bd1be604181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Re93cdb4950e74016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Red0861c15f304d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Ree5a773d36a5410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R298bd89532994ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R74e27c9a4b8341c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R539343f9b68d45dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rcc9231434de145ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R0470068755134e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R24b199b1289d41b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra2a7d9c381694f66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R1e50c19276784b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Re8bc9922cd684891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R34e4f96a7ee44a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rd419204885144828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R30efb1053fc74c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R7895cf8115ae4b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rcb3a0bf45c9842f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R64f908e4bd2b4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rbd16a178cb624b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R7f61ee8ed0df434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R7c4c75c2013b4047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R9e06b6b82f9d48d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R33743f529cf043c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R68927c7bccbc49d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Ra19be7de4b824881"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R07478ee323434772"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R58840a5aa1194ed7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf226723e322b4720"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba7cc2dae60d4cdf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7aa1f17236e746fd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a66bb20b1574687"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb34c6dc6f152463b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1ead43a09ef4be5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6044e42006244e5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R969b42c2923d4527"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I54"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I55"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -1716,35 +1716,27 @@
       <x:c r="N4" s="9" t="n"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TOTAL DE EVENTOS
-85</x:t>
-        </x:is>
+      <x:c r="A5" s="22" t="str">
+        <x:v>TOTAL DE EVENTOS
+86</x:v>
       </x:c>
       <x:c r="B5" s="23" t="n"/>
       <x:c r="C5" s="23" t="n"/>
-      <x:c r="D5" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EVENTOS FUTUROS
-26</x:t>
-        </x:is>
+      <x:c r="D5" s="22" t="str">
+        <x:v>EVENTOS FUTUROS
+27</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n"/>
       <x:c r="F5" s="23" t="n"/>
-      <x:c r="G5" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PÚBLICO ESTIMADO
-127.244</x:t>
-        </x:is>
+      <x:c r="G5" s="22" t="str">
+        <x:v>PÚBLICO ESTIMADO
+127.244</x:v>
       </x:c>
       <x:c r="H5" s="23" t="n"/>
       <x:c r="I5" s="23" t="n"/>
-      <x:c r="J5" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PATROCINADORES
-5</x:t>
-        </x:is>
+      <x:c r="J5" s="22" t="str">
+        <x:v>PATROCINADORES
+5</x:v>
       </x:c>
       <x:c r="K5" s="23" t="n"/>
       <x:c r="L5" s="23" t="n"/>
@@ -1796,11 +1788,9 @@
       <x:c r="N8" s="9" t="n"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CIDADES MONITORADAS
-15</x:t>
-        </x:is>
+      <x:c r="A9" s="22" t="str">
+        <x:v>CIDADES MONITORADAS
+14</x:v>
       </x:c>
       <x:c r="B9" s="23" t="n"/>
       <x:c r="C9" s="23" t="n"/>
@@ -2965,7 +2955,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc9076d4c8a4ef7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff3d142e257410d"/>
 </x:worksheet>
 </file>
 
@@ -5254,7 +5244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5af58a790c9c4975"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ec510692ded47e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7562,7 +7552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf6b712641674406"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9d9c116cf0740e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8194,7 +8184,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d9820ddcd04f6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa9f154a0db4da8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12384,9 +12374,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R129aaaf22eda4c47"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb850e07d5564b14"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3730911242c94f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcd91b6e40c4030"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12677,7 +12667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc99a3b580ab842ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09320f78cc384abc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25464,7 +25454,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51b647b5460b47e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f971076bf9e4266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27366,7 +27356,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8bb353882a04cdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ec9b729d62428f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27778,7 +27768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1209689d39a0481c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26b0e37d0aca48e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27845,28 +27835,28 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
+        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
+        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Diário do Nordeste</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
+        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
@@ -27874,19 +27864,19 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
+        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Empetur</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27895,7 +27885,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
+        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27903,28 +27893,28 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Tributação / legislação federal / organização</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Presidência da República</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27932,57 +27922,57 @@
         <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262.5</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27990,28 +27980,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -28019,19 +28009,19 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28040,7 +28030,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -28048,28 +28038,28 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28077,57 +28067,57 @@
         <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261.5</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28135,28 +28125,28 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -28164,19 +28154,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28185,7 +28175,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -28193,19 +28183,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28214,7 +28204,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28222,10 +28212,10 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28234,7 +28224,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28243,7 +28233,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28251,19 +28241,19 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28272,7 +28262,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28280,57 +28270,57 @@
         <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H17" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28338,28 +28328,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28367,19 +28357,19 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28388,7 +28378,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28396,28 +28386,28 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28425,57 +28415,57 @@
         <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259.5</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28483,28 +28473,28 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28512,19 +28502,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28533,7 +28523,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28541,19 +28531,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28562,7 +28552,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28570,19 +28560,19 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28591,7 +28581,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28599,48 +28589,48 @@
         <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H28" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258.5</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28649,7 +28639,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28657,19 +28647,19 @@
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28678,56 +28668,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257.5</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256.5</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28736,27 +28726,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255.5</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28765,7 +28755,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -28773,28 +28763,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -28802,28 +28792,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28831,28 +28821,28 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28860,19 +28850,19 @@
         <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28881,36 +28871,36 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254.5</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28918,28 +28908,28 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -28947,48 +28937,48 @@
         <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253.5</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28997,27 +28987,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252.5</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29026,7 +29016,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -29034,28 +29024,28 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -29063,57 +29053,57 @@
         <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251.5</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -29121,28 +29111,28 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -29150,48 +29140,48 @@
         <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248.5</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29200,65 +29190,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247.5</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H50" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -29266,28 +29256,28 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H51" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -29295,19 +29285,19 @@
         <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29316,77 +29306,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I52" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239.5</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C53" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G53" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H53" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I53" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238.5</x:v>
       </x:c>
       <x:c r="B54" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C54" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F54" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G54" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H54" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I54" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="6" t="n">
+        <x:v>46199.5</x:v>
+      </x:c>
+      <x:c r="B55" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C55" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D55" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E55" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F55" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G55" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H55" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I54" s="23" t="str">
+      <x:c r="I55" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="6"/>
-      <x:c r="B55" s="23"/>
-      <x:c r="C55" s="23"/>
-      <x:c r="D55" s="23"/>
-      <x:c r="E55" s="23"/>
-      <x:c r="F55" s="23"/>
-      <x:c r="G55" s="23"/>
-      <x:c r="H55" s="23"/>
-      <x:c r="I55" s="23"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="6"/>
@@ -34294,7 +34302,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5227dcb0e014aa7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb75bd9773834c0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35197,7 +35205,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bacbfa5c0eb4d84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50d3432d4ac74a3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36076,7 +36084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03a800b2731c4bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61425d1a2e284549"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36499,7 +36507,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205abe9956c94dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d91d83181eb4d97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona entrevista de Bianca na Seleção Sub-20
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R0470068755134e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R24b199b1289d41b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="Ra2a7d9c381694f66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R1e50c19276784b23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Re8bc9922cd684891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R34e4f96a7ee44a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Rd419204885144828"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R30efb1053fc74c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R7895cf8115ae4b99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rcb3a0bf45c9842f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R64f908e4bd2b4a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Rbd16a178cb624b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R7f61ee8ed0df434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R7c4c75c2013b4047"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R9e06b6b82f9d48d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R33743f529cf043c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R68927c7bccbc49d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Ra19be7de4b824881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R5f0c290e65cb4341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rf37d8579c5e943b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R1c37684da6604066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R803875726cf643f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R1fa523a168ce4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Re366327ccb004139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R2743b249870c4e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rd8ed5e36f7fd47ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R367acee4be6348ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R8dbff407ac73450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R3c97498b47a744ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R447a89f640224f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R1b2a1fa537484491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd151ace8adc146c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R9e1be32659294e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Redf9ee36f285426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rffd0ad6363f84040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R6f3d77fc62114737"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R58840a5aa1194ed7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R426d1e35d90d4de2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba7cc2dae60d4cdf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12499fd7342b4317"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a66bb20b1574687"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R816548c8a22f4be6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1ead43a09ef4be5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3cd43069557849ef"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R969b42c2923d4527"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf7398ce3b9e64150"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I55"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I56"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2955,7 +2955,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff3d142e257410d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e157392685140fe"/>
 </x:worksheet>
 </file>
 
@@ -5244,7 +5244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ec510692ded47e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bfa1a594b7846ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7552,7 +7552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9d9c116cf0740e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92bcd742b7d84620"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8184,7 +8184,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa9f154a0db4da8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ba2d203a904c69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12374,9 +12374,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb850e07d5564b14"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3c34b16c92c4066"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcd91b6e40c4030"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4366338a7854ae9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12667,7 +12667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09320f78cc384abc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95e006f6a97b4122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25454,7 +25454,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f971076bf9e4266"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R214b886d8861473e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27356,7 +27356,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ec9b729d62428f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc573877b3ef04d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27768,7 +27768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26b0e37d0aca48e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19a5174265cf40a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27832,80 +27832,80 @@
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="150.75" customHeight="1">
       <x:c r="A2" s="31" t="n">
-        <x:v>46262.5</x:v>
+        <x:v>46263</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
+        <x:v>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Polônia</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Diário do Nordeste</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
+        <x:v>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
       <x:c r="A3" s="31" t="n">
-        <x:v>46262.5</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
+        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
+        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Diário do Nordeste</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
+        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
       <x:c r="A4" s="31" t="n">
-        <x:v>46262.5</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
+        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Empetur</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27914,143 +27914,143 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
+        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
       <x:c r="A5" s="31" t="n">
-        <x:v>46262.5</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Tributação / legislação federal / organização</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Presidência da República</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="32" t="n">
-        <x:v>46262.5</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28059,143 +28059,143 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32" t="n">
-        <x:v>46261.5</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28204,27 +28204,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28233,18 +28233,18 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28253,7 +28253,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28262,27 +28262,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28291,114 +28291,114 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28407,143 +28407,143 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="n">
-        <x:v>46259.5</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28552,27 +28552,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28581,27 +28581,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28610,56 +28610,56 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32" t="n">
-        <x:v>46258.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H29" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28668,27 +28668,27 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46257.5</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28697,56 +28697,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="n">
-        <x:v>46256.5</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H32" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="n">
-        <x:v>46255.5</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28755,27 +28755,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28784,114 +28784,114 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H35" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32" t="n">
-        <x:v>46254.5</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28900,114 +28900,114 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46253.5</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32" t="n">
-        <x:v>46252.5</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29016,27 +29016,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46252</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29045,172 +29045,172 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H44" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46251.5</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46248.5</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32" t="n">
-        <x:v>46247.5</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29219,114 +29219,114 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46247</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H50" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46246</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H51" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H52" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I52" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="n">
-        <x:v>46239.5</x:v>
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C53" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G53" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29335,77 +29335,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I53" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="32" t="n">
-        <x:v>46238.5</x:v>
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="B54" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C54" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F54" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G54" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H54" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I54" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="6" t="n">
-        <x:v>46199.5</x:v>
+        <x:v>46238</x:v>
       </x:c>
       <x:c r="B55" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C55" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D55" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E55" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F55" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G55" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H55" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I55" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="6" t="n">
+        <x:v>46199</x:v>
+      </x:c>
+      <x:c r="B56" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C56" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F56" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G56" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H56" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I55" s="23" t="str">
+      <x:c r="I56" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="6"/>
-      <x:c r="B56" s="23"/>
-      <x:c r="C56" s="23"/>
-      <x:c r="D56" s="23"/>
-      <x:c r="E56" s="23"/>
-      <x:c r="F56" s="23"/>
-      <x:c r="G56" s="23"/>
-      <x:c r="H56" s="23"/>
-      <x:c r="I56" s="23"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="6"/>
@@ -34302,7 +34320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb75bd9773834c0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R419af19b387b439c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35205,7 +35223,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50d3432d4ac74a3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R816a99d7e608471c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36084,7 +36102,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61425d1a2e284549"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266e7bcebc07476d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36507,7 +36525,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d91d83181eb4d97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98a5797863a34e27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza notícia sobre integração da Seleção Sub-20
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R5f0c290e65cb4341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="Rf37d8579c5e943b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R1c37684da6604066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R803875726cf643f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R1fa523a168ce4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="Re366327ccb004139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R2743b249870c4e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rd8ed5e36f7fd47ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R367acee4be6348ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R8dbff407ac73450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R3c97498b47a744ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R447a89f640224f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R1b2a1fa537484491"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rd151ace8adc146c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R9e1be32659294e52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="Redf9ee36f285426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Rffd0ad6363f84040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R6f3d77fc62114737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rc6e1ef22c1c3484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R5f59188134c34e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R3a801689f4e0418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R48ef44ea6b71465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R0194f633d70e41d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R547a2f3ac5fa4788"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R72b0e7dc74df42bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5e7f0d7b4e7148be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R62967ecf7fc3483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R59c90b772f1c4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rf3e34bdd74e24cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R21eea333e95b454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R54b6c6bde4c34b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R50df33ea169e449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R8ef01748f5c74337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R09eee21bd64d499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Ra2f48b247eca40d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rbe32da9cc9d246b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R426d1e35d90d4de2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd54761a42e9464d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12499fd7342b4317"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ae6e3433a17408c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R816548c8a22f4be6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ad25a970c5d4382"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3cd43069557849ef"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6cbce24257764e09"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf7398ce3b9e64150"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c823d6e89a34987"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I56"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I57"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2955,7 +2955,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e157392685140fe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3436a005474247"/>
 </x:worksheet>
 </file>
 
@@ -5244,7 +5244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bfa1a594b7846ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R019b9245d3d9453f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7552,7 +7552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92bcd742b7d84620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra261ac29adba40d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8184,7 +8184,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ba2d203a904c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce70b7a8eed4695"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12374,9 +12374,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3c34b16c92c4066"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R450c1e16161b4c89"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4366338a7854ae9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1de33d472e4f03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12667,7 +12667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95e006f6a97b4122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da8882dcdfe494d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25454,7 +25454,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R214b886d8861473e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d881ffec45a40ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25510,8 +25510,8 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="23" t="str" cm="1">
-        <x:f t="array" ref="A2:A28">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
-        <x:v>EVT-0064</x:v>
+        <x:f t="array" ref="A2:A26">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
+        <x:v>EVT-0082</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="23"/>
@@ -25523,7 +25523,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="23" t="str">
-        <x:v>EVT-0091</x:v>
+        <x:v>EVT-0083</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="23"/>
@@ -25535,7 +25535,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="23" t="str">
-        <x:v>EVT-0082</x:v>
+        <x:v>EVT-0022</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="23"/>
@@ -25547,7 +25547,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="23" t="str">
-        <x:v>EVT-0083</x:v>
+        <x:v>EVT-0062</x:v>
       </x:c>
       <x:c r="B5" s="6"/>
       <x:c r="C5" s="23"/>
@@ -25559,7 +25559,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="23" t="str">
-        <x:v>EVT-0022</x:v>
+        <x:v>EVT-0084</x:v>
       </x:c>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="23"/>
@@ -25571,7 +25571,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="23" t="str">
-        <x:v>EVT-0062</x:v>
+        <x:v>EVT-0074</x:v>
       </x:c>
       <x:c r="B7" s="6"/>
       <x:c r="C7" s="23"/>
@@ -25583,7 +25583,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
-        <x:v>EVT-0084</x:v>
+        <x:v>EVT-0006</x:v>
       </x:c>
       <x:c r="B8" s="6"/>
       <x:c r="C8" s="23"/>
@@ -25595,7 +25595,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="23" t="str">
-        <x:v>EVT-0074</x:v>
+        <x:v>EVT-0085</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n"/>
       <x:c r="C9" s="23" t="n"/>
@@ -25607,7 +25607,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="23" t="str">
-        <x:v>EVT-0006</x:v>
+        <x:v>EVT-0086</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n"/>
       <x:c r="C10" s="23" t="n"/>
@@ -25619,7 +25619,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="23" t="str">
-        <x:v>EVT-0085</x:v>
+        <x:v>EVT-0087</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n"/>
       <x:c r="C11" s="23" t="n"/>
@@ -25631,7 +25631,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="23" t="str">
-        <x:v>EVT-0086</x:v>
+        <x:v>EVT-0055</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n"/>
       <x:c r="C12" s="23" t="n"/>
@@ -25643,7 +25643,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="23" t="str">
-        <x:v>EVT-0087</x:v>
+        <x:v>EVT-0007</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n"/>
       <x:c r="C13" s="23" t="n"/>
@@ -25655,7 +25655,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="23" t="str">
-        <x:v>EVT-0055</x:v>
+        <x:v>EVT-0088</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n"/>
       <x:c r="C14" s="23" t="n"/>
@@ -25667,7 +25667,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="23" t="str">
-        <x:v>EVT-0007</x:v>
+        <x:v>EVT-0011</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n"/>
       <x:c r="C15" s="23" t="n"/>
@@ -25679,7 +25679,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="23" t="str">
-        <x:v>EVT-0088</x:v>
+        <x:v>EVT-0089</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n"/>
       <x:c r="C16" s="23" t="n"/>
@@ -25691,61 +25691,61 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="23" t="str">
-        <x:v>EVT-0011</x:v>
+        <x:v>EVT-0010</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="23" t="str">
-        <x:v>EVT-0089</x:v>
+        <x:v>EVT-0008</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="23" t="str">
-        <x:v>EVT-0010</x:v>
+        <x:v>EVT-0090</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="23" t="str">
-        <x:v>EVT-0008</x:v>
+        <x:v>EVT-0009</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="23" t="str">
-        <x:v>EVT-0090</x:v>
+        <x:v>EVT-0012</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="23" t="str">
-        <x:v>EVT-0009</x:v>
+        <x:v>EVT-0077</x:v>
       </x:c>
       <x:c r="B22" s="6" t="n"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="23" t="str">
-        <x:v>EVT-0012</x:v>
+        <x:v>EVT-0017</x:v>
       </x:c>
       <x:c r="B23" s="6" t="n"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="23" t="str">
-        <x:v>EVT-0077</x:v>
+        <x:v>EVT-0018</x:v>
       </x:c>
       <x:c r="B24" s="6" t="n"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="23" t="str">
-        <x:v>EVT-0017</x:v>
+        <x:v>EVT-0019</x:v>
       </x:c>
       <x:c r="B25" s="6" t="n"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="23" t="str">
-        <x:v>EVT-0018</x:v>
+        <x:v>EVT-0020</x:v>
       </x:c>
       <x:c r="B26" s="6" t="n"/>
     </x:row>
@@ -27356,7 +27356,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc573877b3ef04d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa7e2d438a60474f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27768,7 +27768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19a5174265cf40a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e4c86486394c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27832,13 +27832,13 @@
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="150.75" customHeight="1">
       <x:c r="A2" s="31" t="n">
-        <x:v>46263</x:v>
+        <x:v>46264.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</x:v>
+        <x:v>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>Polônia</x:v>
@@ -27847,7 +27847,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27856,36 +27856,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</x:v>
+        <x:v>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
       <x:c r="A3" s="31" t="n">
-        <x:v>46262</x:v>
+        <x:v>46263</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
+        <x:v>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Polônia</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Diário do Nordeste</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
+        <x:v>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
@@ -27893,28 +27893,28 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
+        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
+        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Diário do Nordeste</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
+        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27922,19 +27922,19 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
+        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Empetur</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27943,7 +27943,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
+        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27951,28 +27951,28 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Tributação / legislação federal / organização</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Presidência da República</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27980,57 +27980,57 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="32" t="n">
-        <x:v>46261</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -28038,28 +28038,28 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28067,19 +28067,19 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28088,7 +28088,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -28096,28 +28096,28 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28125,57 +28125,57 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="n">
-        <x:v>46260</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -28183,28 +28183,28 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28212,19 +28212,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28233,7 +28233,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28241,19 +28241,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28262,7 +28262,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28270,10 +28270,10 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28282,7 +28282,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28291,7 +28291,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28299,19 +28299,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E18" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28320,7 +28320,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28328,57 +28328,57 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32" t="n">
-        <x:v>46259</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28386,28 +28386,28 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28415,19 +28415,19 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28436,7 +28436,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28444,28 +28444,28 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H23" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28473,57 +28473,57 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="n">
-        <x:v>46258</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -28531,28 +28531,28 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28560,19 +28560,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28581,7 +28581,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28589,19 +28589,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28610,7 +28610,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28618,19 +28618,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28639,7 +28639,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28647,48 +28647,48 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H30" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32" t="n">
-        <x:v>46257</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28697,7 +28697,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -28705,19 +28705,19 @@
         <x:v>46257</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28726,56 +28726,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32" t="n">
-        <x:v>46256</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H33" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46255</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28784,27 +28784,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="n">
-        <x:v>46254</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28813,7 +28813,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -28821,28 +28821,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H36" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28850,28 +28850,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28879,28 +28879,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28908,19 +28908,19 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28929,36 +28929,36 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32" t="n">
-        <x:v>46253</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H40" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -28966,28 +28966,28 @@
         <x:v>46253</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -28995,48 +28995,48 @@
         <x:v>46253</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32" t="n">
-        <x:v>46252</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29045,27 +29045,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46251</x:v>
+        <x:v>46252</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29074,7 +29074,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -29082,28 +29082,28 @@
         <x:v>46251</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H45" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -29111,57 +29111,57 @@
         <x:v>46251</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -29169,28 +29169,28 @@
         <x:v>46248</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -29198,48 +29198,48 @@
         <x:v>46248</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32" t="n">
-        <x:v>46247</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29248,65 +29248,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="n">
-        <x:v>46246</x:v>
+        <x:v>46247</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H51" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="n">
-        <x:v>46239</x:v>
+        <x:v>46246</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H52" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I52" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -29314,28 +29314,28 @@
         <x:v>46239</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C53" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G53" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H53" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I53" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -29343,19 +29343,19 @@
         <x:v>46239</x:v>
       </x:c>
       <x:c r="B54" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C54" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F54" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G54" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29364,77 +29364,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I54" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="6" t="n">
-        <x:v>46238</x:v>
+      <x:c r="A55" s="32" t="n">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="B55" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C55" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D55" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E55" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F55" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G55" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H55" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I55" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="6" t="n">
-        <x:v>46199</x:v>
+      <x:c r="A56" s="32" t="n">
+        <x:v>46238</x:v>
       </x:c>
       <x:c r="B56" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C56" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D56" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E56" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F56" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G56" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H56" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I56" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="32" t="n">
+        <x:v>46199</x:v>
+      </x:c>
+      <x:c r="B57" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C57" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G57" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H57" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I56" s="23" t="str">
+      <x:c r="I57" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="6"/>
-      <x:c r="B57" s="23"/>
-      <x:c r="C57" s="23"/>
-      <x:c r="D57" s="23"/>
-      <x:c r="E57" s="23"/>
-      <x:c r="F57" s="23"/>
-      <x:c r="G57" s="23"/>
-      <x:c r="H57" s="23"/>
-      <x:c r="I57" s="23"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="6"/>
@@ -34320,7 +34338,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R419af19b387b439c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe989ea0c5434ed5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35223,7 +35241,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R816a99d7e608471c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8c78b12350426a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36102,7 +36120,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266e7bcebc07476d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef7a1f164264e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36525,7 +36543,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98a5797863a34e27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb85a636b46be499a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza preparação da Seleção Sub-20 na Polônia
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="Rc6e1ef22c1c3484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R5f59188134c34e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R3a801689f4e0418a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="R48ef44ea6b71465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="R0194f633d70e41d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R547a2f3ac5fa4788"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="R72b0e7dc74df42bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="R5e7f0d7b4e7148be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="R62967ecf7fc3483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="R59c90b772f1c4731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="Rf3e34bdd74e24cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="R21eea333e95b454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="R54b6c6bde4c34b4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="R50df33ea169e449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="R8ef01748f5c74337"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R09eee21bd64d499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="Ra2f48b247eca40d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="Rbe32da9cc9d246b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="1" r:id="R63da3fa205a240d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Eventos" sheetId="2" r:id="R75b4e61dfdba43c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Agenda" sheetId="3" r:id="R21f3cd94a78e4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Radar_IAC" sheetId="4" r:id="Rfc4820ee22c5432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Radar_INP" sheetId="5" r:id="Ra5e4cf7b65d04cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Noticias" sheetId="6" r:id="R7d4fc5ed2ec24ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Mapa_Base" sheetId="7" r:id="Reb2c6f85046c449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Patrocinadores" sheetId="8" r:id="Rba779cf9bc444adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Cidades" sheetId="9" r:id="Rd81aa8339b314d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Legado" sheetId="10" r:id="Rf8d55731525444d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Obras" sheetId="11" r:id="R679265925c404016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Voluntariado" sheetId="12" r:id="Refaa64e420ae4341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Midia" sheetId="13" r:id="Rc30caae53cef40a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Riscos" sheetId="14" r:id="Rff49624d3eae4ca0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Config" sheetId="15" r:id="Re1c43e9f04184b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Manual" sheetId="16" r:id="R3247ad12091042ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Base_Geografica_Brasil" sheetId="17" r:id="R358bfb358cc84849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_PowerBI_Guia" sheetId="18" r:id="R49bcf2efb0494dfa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,7 +1138,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd54761a42e9464d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e7ce9ac1d6146be"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,7 +1168,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ae6e3433a17408c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf27aff7f3b7e4200"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1198,7 +1198,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ad25a970c5d4382"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0f3ba743daf34735"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1228,7 +1228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6cbce24257764e09"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb023cc932e9b42d1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1263,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c823d6e89a34987"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ec4bbbb1c5b4abf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1388,8 +1388,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I57"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I58" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I58"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Título"/>
@@ -2955,7 +2955,7 @@
     <x:mergeCell ref="A5:C7"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3436a005474247"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4daf1581554006"/>
 </x:worksheet>
 </file>
 
@@ -5244,7 +5244,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R019b9245d3d9453f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R134d837fe7d34ab3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7552,7 +7552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra261ac29adba40d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b985a7e61644e3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8184,7 +8184,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce70b7a8eed4695"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb6f41253a724b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12374,9 +12374,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R450c1e16161b4c89"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf058f10a63f645d3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1de33d472e4f03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra27f7972b82a4fde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12667,7 +12667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da8882dcdfe494d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf683203f48114f54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25454,7 +25454,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d881ffec45a40ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99cc69c8d8c2480d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25510,8 +25510,8 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="23" t="str" cm="1">
-        <x:f t="array" ref="A2:A26">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
-        <x:v>EVT-0082</x:v>
+        <x:f t="array" ref="A2:A28">_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6,7,8},'02_Eventos'!A2:A495,'02_Eventos'!C2:C495,'02_Eventos'!E2:E495,'02_Eventos'!D2:D495,'02_Eventos'!F2:F495,'02_Eventos'!I2:I495,'02_Eventos'!H2:H495,'02_Eventos'!B2:B495),('02_Eventos'!C2:C495&gt;=TODAY())*('02_Eventos'!B2:B495&lt;&gt;"Cancelado"),"Sem eventos futuros")</x:f>
+        <x:v>EVT-0064</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="23"/>
@@ -25523,7 +25523,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="23" t="str">
-        <x:v>EVT-0083</x:v>
+        <x:v>EVT-0091</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="23"/>
@@ -25535,7 +25535,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="23" t="str">
-        <x:v>EVT-0022</x:v>
+        <x:v>EVT-0082</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="23"/>
@@ -25547,7 +25547,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="23" t="str">
-        <x:v>EVT-0062</x:v>
+        <x:v>EVT-0083</x:v>
       </x:c>
       <x:c r="B5" s="6"/>
       <x:c r="C5" s="23"/>
@@ -25559,7 +25559,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="23" t="str">
-        <x:v>EVT-0084</x:v>
+        <x:v>EVT-0022</x:v>
       </x:c>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="23"/>
@@ -25571,7 +25571,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="23" t="str">
-        <x:v>EVT-0074</x:v>
+        <x:v>EVT-0062</x:v>
       </x:c>
       <x:c r="B7" s="6"/>
       <x:c r="C7" s="23"/>
@@ -25583,7 +25583,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
-        <x:v>EVT-0006</x:v>
+        <x:v>EVT-0084</x:v>
       </x:c>
       <x:c r="B8" s="6"/>
       <x:c r="C8" s="23"/>
@@ -25595,7 +25595,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="23" t="str">
-        <x:v>EVT-0085</x:v>
+        <x:v>EVT-0074</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n"/>
       <x:c r="C9" s="23" t="n"/>
@@ -25607,7 +25607,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="23" t="str">
-        <x:v>EVT-0086</x:v>
+        <x:v>EVT-0006</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n"/>
       <x:c r="C10" s="23" t="n"/>
@@ -25619,7 +25619,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="23" t="str">
-        <x:v>EVT-0087</x:v>
+        <x:v>EVT-0085</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n"/>
       <x:c r="C11" s="23" t="n"/>
@@ -25631,7 +25631,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="23" t="str">
-        <x:v>EVT-0055</x:v>
+        <x:v>EVT-0086</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n"/>
       <x:c r="C12" s="23" t="n"/>
@@ -25643,7 +25643,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="23" t="str">
-        <x:v>EVT-0007</x:v>
+        <x:v>EVT-0087</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n"/>
       <x:c r="C13" s="23" t="n"/>
@@ -25655,7 +25655,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="23" t="str">
-        <x:v>EVT-0088</x:v>
+        <x:v>EVT-0055</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n"/>
       <x:c r="C14" s="23" t="n"/>
@@ -25667,7 +25667,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="23" t="str">
-        <x:v>EVT-0011</x:v>
+        <x:v>EVT-0007</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n"/>
       <x:c r="C15" s="23" t="n"/>
@@ -25679,7 +25679,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="23" t="str">
-        <x:v>EVT-0089</x:v>
+        <x:v>EVT-0088</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n"/>
       <x:c r="C16" s="23" t="n"/>
@@ -25691,61 +25691,61 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="23" t="str">
-        <x:v>EVT-0010</x:v>
+        <x:v>EVT-0011</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="23" t="str">
-        <x:v>EVT-0008</x:v>
+        <x:v>EVT-0089</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="23" t="str">
-        <x:v>EVT-0090</x:v>
+        <x:v>EVT-0010</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="23" t="str">
-        <x:v>EVT-0009</x:v>
+        <x:v>EVT-0008</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="23" t="str">
-        <x:v>EVT-0012</x:v>
+        <x:v>EVT-0090</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="23" t="str">
-        <x:v>EVT-0077</x:v>
+        <x:v>EVT-0009</x:v>
       </x:c>
       <x:c r="B22" s="6" t="n"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="23" t="str">
-        <x:v>EVT-0017</x:v>
+        <x:v>EVT-0012</x:v>
       </x:c>
       <x:c r="B23" s="6" t="n"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="23" t="str">
-        <x:v>EVT-0018</x:v>
+        <x:v>EVT-0077</x:v>
       </x:c>
       <x:c r="B24" s="6" t="n"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="23" t="str">
-        <x:v>EVT-0019</x:v>
+        <x:v>EVT-0017</x:v>
       </x:c>
       <x:c r="B25" s="6" t="n"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="23" t="str">
-        <x:v>EVT-0020</x:v>
+        <x:v>EVT-0018</x:v>
       </x:c>
       <x:c r="B26" s="6" t="n"/>
     </x:row>
@@ -27356,7 +27356,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa7e2d438a60474f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96a91f56515242e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27768,7 +27768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e4c86486394c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c986694b8854688"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27835,19 +27835,19 @@
         <x:v>46264.5</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</x:v>
+        <x:v>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Polônia</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27856,18 +27856,18 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="114" customHeight="1">
       <x:c r="A3" s="31" t="n">
-        <x:v>46263</x:v>
+        <x:v>46264.5</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</x:v>
+        <x:v>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>Polônia</x:v>
@@ -27876,7 +27876,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>Positivo</x:v>
@@ -27885,36 +27885,36 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</x:v>
+        <x:v>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="99.75" customHeight="1">
       <x:c r="A4" s="31" t="n">
-        <x:v>46262</x:v>
+        <x:v>46263</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
+        <x:v>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>Polônia</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Diário do Nordeste</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
+        <x:v>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="128.25" customHeight="1">
@@ -27922,28 +27922,28 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
+        <x:v>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
+        <x:v>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Diário do Nordeste</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
+        <x:v>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -27951,19 +27951,19 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
+        <x:v>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
-        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / transição de categoria</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>Empetur</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -27972,7 +27972,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
+        <x:v>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27980,28 +27980,28 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
+        <x:v>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
-        <x:v>Tributação / legislação federal / organização</x:v>
+        <x:v>Infraestrutura / Arena Pernambuco / contratação pública</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
-        <x:v>Presidência da República</x:v>
+        <x:v>Empetur</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
+        <x:v>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
+        <x:v>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -28009,57 +28009,57 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
+        <x:v>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
+        <x:v>Tributação / legislação federal / organização</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>Presidência da República</x:v>
       </x:c>
       <x:c r="F8" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
+        <x:v>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I8" s="23" t="str">
-        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
+        <x:v>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="32" t="n">
-        <x:v>46261</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
-        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
+        <x:v>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</x:v>
       </x:c>
       <x:c r="C9" s="23" t="str">
-        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
+        <x:v>Contagem regressiva / Porto Alegre / Fan Fest / legado</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Bahia Notícias</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
-        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I9" s="23" t="str">
-        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
+        <x:v>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28067,28 +28067,28 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
-        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
+        <x:v>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
-        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
+        <x:v>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>Bahia Notícias</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
+        <x:v>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</x:v>
       </x:c>
       <x:c r="G10" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I10" s="23" t="str">
-        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
+        <x:v>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -28096,19 +28096,19 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
-        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
+        <x:v>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Marketing / audiência digital / patrocínios / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
+        <x:v>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</x:v>
       </x:c>
       <x:c r="G11" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28117,7 +28117,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I11" s="23" t="str">
-        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
+        <x:v>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -28125,28 +28125,28 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
+        <x:v>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>Alerj</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
-        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</x:v>
       </x:c>
       <x:c r="G12" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I12" s="23" t="str">
-        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
+        <x:v>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -28154,57 +28154,57 @@
         <x:v>46261</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
-        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
+        <x:v>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
+        <x:v>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Cracóvia/POL</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Alerj</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
+        <x:v>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</x:v>
       </x:c>
       <x:c r="G13" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H13" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I13" s="23" t="str">
-        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
+        <x:v>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32" t="n">
-        <x:v>46260</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
-        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
+        <x:v>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
-        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</x:v>
       </x:c>
       <x:c r="D14" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Cracóvia/POL</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>Correio do Povo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
-        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</x:v>
       </x:c>
       <x:c r="G14" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I14" s="23" t="str">
-        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
+        <x:v>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -28212,28 +28212,28 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
-        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
+        <x:v>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
+        <x:v>Tour da Taça / ativações / EVT-0090</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Federação Gaúcha de Futebol</x:v>
+        <x:v>Correio do Povo</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
-        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
+        <x:v>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</x:v>
       </x:c>
       <x:c r="G15" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I15" s="23" t="str">
-        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
+        <x:v>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -28241,19 +28241,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
+        <x:v>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
-        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
+        <x:v>II Workshop de Cidades-Sede e Estádios / Porto Alegre</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>Folha de Pernambuco</x:v>
+        <x:v>Federação Gaúcha de Futebol</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
+        <x:v>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28262,7 +28262,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
-        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
+        <x:v>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -28270,19 +28270,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
+        <x:v>Recife integrará programa de voluntários da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Voluntariado / preparação das cidades-sede / Recife</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Bielsko-Biała/POL</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Folha de Pernambuco</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
+        <x:v>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</x:v>
       </x:c>
       <x:c r="G17" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28291,7 +28291,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I17" s="23" t="str">
-        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
+        <x:v>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -28299,10 +28299,10 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
+        <x:v>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D18" s="23" t="str">
         <x:v>Bielsko-Biała/POL</x:v>
@@ -28311,7 +28311,7 @@
         <x:v>CBF</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</x:v>
       </x:c>
       <x:c r="G18" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28320,7 +28320,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I18" s="23" t="str">
-        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
+        <x:v>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -28328,19 +28328,19 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
+        <x:v>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
-        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / preparação</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Bielsko-Biała/POL</x:v>
       </x:c>
       <x:c r="E19" s="23" t="str">
-        <x:v>Meio &amp; Mensagem</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</x:v>
       </x:c>
       <x:c r="G19" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28349,7 +28349,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
+        <x:v>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -28357,57 +28357,57 @@
         <x:v>46260</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
-        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
+        <x:v>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
+        <x:v>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Internacional</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>Folha de S.Paulo / AFP</x:v>
+        <x:v>Meio &amp; Mensagem</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
+        <x:v>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</x:v>
       </x:c>
       <x:c r="G20" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H20" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I20" s="23" t="str">
-        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
+        <x:v>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="n">
-        <x:v>46259</x:v>
+        <x:v>46260</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
+        <x:v>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
-        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina / governança FIFA</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Internacional</x:v>
       </x:c>
       <x:c r="E21" s="23" t="str">
-        <x:v>A TARDE</x:v>
+        <x:v>Folha de S.Paulo / AFP</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</x:v>
       </x:c>
       <x:c r="G21" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H21" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I21" s="23" t="str">
-        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
+        <x:v>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -28415,28 +28415,28 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
-        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
+        <x:v>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
-        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
+        <x:v>Cultura / turismo / alimentação / Salvador</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E22" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>A TARDE</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
+        <x:v>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</x:v>
       </x:c>
       <x:c r="G22" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H22" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I22" s="23" t="str">
-        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
+        <x:v>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -28444,19 +28444,19 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
-        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
+        <x:v>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C23" s="23" t="str">
-        <x:v>Calendário continental / clubes / organização</x:v>
+        <x:v>Sorteio / governança / premiação / EVT-0010</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>América do Sul / Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E23" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</x:v>
       </x:c>
       <x:c r="G23" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28465,7 +28465,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I23" s="23" t="str">
-        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
+        <x:v>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -28473,28 +28473,28 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
+        <x:v>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Negócios / audiência / patrocínios</x:v>
+        <x:v>Calendário continental / clubes / organização</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>América do Sul / Brasil</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>MKT Esportivo</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
+        <x:v>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I24" s="23" t="str">
-        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
+        <x:v>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -28502,57 +28502,57 @@
         <x:v>46259</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
-        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
+        <x:v>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</x:v>
       </x:c>
       <x:c r="C25" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
+        <x:v>Negócios / audiência / patrocínios</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Porto Alegre/RS</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E25" s="23" t="str">
-        <x:v>GZH</x:v>
+        <x:v>MKT Esportivo</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
+        <x:v>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</x:v>
       </x:c>
       <x:c r="G25" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H25" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I25" s="23" t="str">
-        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
+        <x:v>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="n">
-        <x:v>46258</x:v>
+        <x:v>46259</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
-        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
+        <x:v>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
-        <x:v>Calendário / estádios / EVT-0077</x:v>
+        <x:v>Seleção Brasileira / preparação / Porto Alegre</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Porto Alegre/RS</x:v>
       </x:c>
       <x:c r="E26" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>GZH</x:v>
       </x:c>
       <x:c r="F26" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
+        <x:v>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</x:v>
       </x:c>
       <x:c r="G26" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H26" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I26" s="23" t="str">
-        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
+        <x:v>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -28560,28 +28560,28 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
-        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
+        <x:v>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C27" s="23" t="str">
-        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
+        <x:v>Calendário / estádios / EVT-0077</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E27" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F27" s="23" t="str">
-        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G27" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H27" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I27" s="23" t="str">
-        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
+        <x:v>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -28589,19 +28589,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
-        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
+        <x:v>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
+        <x:v>II Workshop de Cidades-Sede / planejamento / EVT-0023</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E28" s="23" t="str">
-        <x:v>TV Brasil</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F28" s="23" t="str">
-        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
+        <x:v>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</x:v>
       </x:c>
       <x:c r="G28" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28610,7 +28610,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I28" s="23" t="str">
-        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
+        <x:v>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -28618,19 +28618,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B29" s="23" t="str">
-        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
+        <x:v>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</x:v>
       </x:c>
       <x:c r="C29" s="23" t="str">
-        <x:v>Turismo / hotelaria / economia local</x:v>
+        <x:v>Elas Jogam Summit / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Fortaleza/CE</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E29" s="23" t="str">
-        <x:v>TurisNews</x:v>
+        <x:v>TV Brasil</x:v>
       </x:c>
       <x:c r="F29" s="23" t="str">
-        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
+        <x:v>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</x:v>
       </x:c>
       <x:c r="G29" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28639,7 +28639,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I29" s="23" t="str">
-        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
+        <x:v>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -28647,19 +28647,19 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B30" s="23" t="str">
-        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
+        <x:v>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
-        <x:v>Sustentabilidade / Fortaleza</x:v>
+        <x:v>Turismo / hotelaria / economia local</x:v>
       </x:c>
       <x:c r="D30" s="23" t="str">
         <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E30" s="23" t="str">
-        <x:v>Agência Sebrae de Notícias</x:v>
+        <x:v>TurisNews</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
+        <x:v>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</x:v>
       </x:c>
       <x:c r="G30" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28668,7 +28668,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I30" s="23" t="str">
-        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
+        <x:v>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -28676,48 +28676,48 @@
         <x:v>46258</x:v>
       </x:c>
       <x:c r="B31" s="23" t="str">
-        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
+        <x:v>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</x:v>
       </x:c>
       <x:c r="C31" s="23" t="str">
-        <x:v>Sorteio / calendário / EVT-0010</x:v>
+        <x:v>Sustentabilidade / Fortaleza</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Fortaleza/CE</x:v>
       </x:c>
       <x:c r="E31" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Agência Sebrae de Notícias</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
+        <x:v>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</x:v>
       </x:c>
       <x:c r="G31" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H31" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
+        <x:v>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32" t="n">
-        <x:v>46257</x:v>
+        <x:v>46258</x:v>
       </x:c>
       <x:c r="B32" s="23" t="str">
-        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
+        <x:v>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
-        <x:v>Patrocínio / negócios</x:v>
+        <x:v>Sorteio / calendário / EVT-0010</x:v>
       </x:c>
       <x:c r="D32" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E32" s="23" t="str">
-        <x:v>Exame</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</x:v>
       </x:c>
       <x:c r="G32" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28726,7 +28726,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I32" s="23" t="str">
-        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
+        <x:v>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -28734,19 +28734,19 @@
         <x:v>46257</x:v>
       </x:c>
       <x:c r="B33" s="23" t="str">
-        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
+        <x:v>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C33" s="23" t="str">
-        <x:v>Tributação / organização / políticas públicas</x:v>
+        <x:v>Patrocínio / negócios</x:v>
       </x:c>
       <x:c r="D33" s="23" t="str">
-        <x:v>Rio de Janeiro/RJ</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E33" s="23" t="str">
-        <x:v>Governo do Estado do Rio de Janeiro</x:v>
+        <x:v>Exame</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
+        <x:v>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</x:v>
       </x:c>
       <x:c r="G33" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28755,56 +28755,56 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I33" s="23" t="str">
-        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
+        <x:v>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32" t="n">
-        <x:v>46256</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="B34" s="23" t="str">
-        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
+        <x:v>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
-        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
+        <x:v>Tributação / organização / políticas públicas</x:v>
       </x:c>
       <x:c r="D34" s="23" t="str">
-        <x:v>Salvador/BA</x:v>
+        <x:v>Rio de Janeiro/RJ</x:v>
       </x:c>
       <x:c r="E34" s="23" t="str">
-        <x:v>Correio</x:v>
+        <x:v>Governo do Estado do Rio de Janeiro</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
+        <x:v>https://www.rj.gov.br/radioroquettepinto/node/20221</x:v>
       </x:c>
       <x:c r="G34" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H34" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I34" s="23" t="str">
-        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
+        <x:v>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32" t="n">
-        <x:v>46255</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="B35" s="23" t="str">
-        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
+        <x:v>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</x:v>
       </x:c>
       <x:c r="C35" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Copa Salvador Interbairros / legado / EVT-0064</x:v>
       </x:c>
       <x:c r="D35" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Salvador/BA</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>Correio</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
+        <x:v>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</x:v>
       </x:c>
       <x:c r="G35" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28813,27 +28813,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I35" s="23" t="str">
-        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
+        <x:v>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32" t="n">
-        <x:v>46254</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="B36" s="23" t="str">
-        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
+        <x:v>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
-        <x:v>Seleção Brasileira / preparação</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D36" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E36" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</x:v>
       </x:c>
       <x:c r="G36" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -28842,7 +28842,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I36" s="23" t="str">
-        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
+        <x:v>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -28850,28 +28850,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B37" s="23" t="str">
-        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
+        <x:v>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</x:v>
       </x:c>
       <x:c r="C37" s="23" t="str">
-        <x:v>Ingressos / relacionamento</x:v>
+        <x:v>Seleção Brasileira / preparação</x:v>
       </x:c>
       <x:c r="D37" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</x:v>
       </x:c>
       <x:c r="G37" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H37" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I37" s="23" t="str">
-        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
+        <x:v>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -28879,28 +28879,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B38" s="23" t="str">
-        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
+        <x:v>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C38" s="23" t="str">
-        <x:v>Calendário / sedes</x:v>
+        <x:v>Ingressos / relacionamento</x:v>
       </x:c>
       <x:c r="D38" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E38" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</x:v>
       </x:c>
       <x:c r="G38" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H38" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I38" s="23" t="str">
-        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
+        <x:v>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -28908,28 +28908,28 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B39" s="23" t="str">
-        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
+        <x:v>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</x:v>
       </x:c>
       <x:c r="C39" s="23" t="str">
-        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
+        <x:v>Calendário / sedes</x:v>
       </x:c>
       <x:c r="D39" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E39" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F39" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
+        <x:v>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</x:v>
       </x:c>
       <x:c r="G39" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H39" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I39" s="23" t="str">
-        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
+        <x:v>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -28937,19 +28937,19 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="B40" s="23" t="str">
-        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
+        <x:v>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
-        <x:v>Repescagem / sorteio</x:v>
+        <x:v>Investimentos públicos / segurança / infraestrutura</x:v>
       </x:c>
       <x:c r="D40" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E40" s="23" t="str">
-        <x:v>FIFA</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
+        <x:v>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</x:v>
       </x:c>
       <x:c r="G40" s="23" t="str">
         <x:v>Neutro</x:v>
@@ -28958,36 +28958,36 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I40" s="23" t="str">
-        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
+        <x:v>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32" t="n">
-        <x:v>46253</x:v>
+        <x:v>46254</x:v>
       </x:c>
       <x:c r="B41" s="23" t="str">
-        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
+        <x:v>Sorteio define caminhos da fase preliminar da repescagem mundial</x:v>
       </x:c>
       <x:c r="C41" s="23" t="str">
-        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
+        <x:v>Repescagem / sorteio</x:v>
       </x:c>
       <x:c r="D41" s="23" t="str">
-        <x:v>Brasil / Polônia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E41" s="23" t="str">
         <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F41" s="23" t="str">
-        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
+        <x:v>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</x:v>
       </x:c>
       <x:c r="G41" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H41" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I41" s="23" t="str">
-        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
+        <x:v>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -28995,28 +28995,28 @@
         <x:v>46253</x:v>
       </x:c>
       <x:c r="B42" s="23" t="str">
-        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
+        <x:v>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-20 Feminina</x:v>
       </x:c>
       <x:c r="D42" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Brasil / Polônia</x:v>
       </x:c>
       <x:c r="E42" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>FIFA</x:v>
       </x:c>
       <x:c r="F42" s="23" t="str">
-        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
+        <x:v>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</x:v>
       </x:c>
       <x:c r="G42" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H42" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I42" s="23" t="str">
-        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
+        <x:v>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -29024,48 +29024,48 @@
         <x:v>46253</x:v>
       </x:c>
       <x:c r="B43" s="23" t="str">
-        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
+        <x:v>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</x:v>
       </x:c>
       <x:c r="C43" s="23" t="str">
-        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D43" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E43" s="23" t="str">
-        <x:v>Revista Super Negócios / ASSERJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
+        <x:v>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</x:v>
       </x:c>
       <x:c r="G43" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H43" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I43" s="23" t="str">
-        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
+        <x:v>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32" t="n">
-        <x:v>46252</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="B44" s="23" t="str">
-        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
+        <x:v>Supermercados entram no planejamento comercial para a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
-        <x:v>Elas em Ação / legado / EVT-0081</x:v>
+        <x:v>Varejo / consumo / oportunidades comerciais</x:v>
       </x:c>
       <x:c r="D44" s="23" t="str">
-        <x:v>Brasília/DF</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E44" s="23" t="str">
-        <x:v>FSports</x:v>
+        <x:v>Revista Super Negócios / ASSERJ</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
+        <x:v>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</x:v>
       </x:c>
       <x:c r="G44" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29074,27 +29074,27 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I44" s="23" t="str">
-        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
+        <x:v>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32" t="n">
-        <x:v>46251</x:v>
+        <x:v>46252</x:v>
       </x:c>
       <x:c r="B45" s="23" t="str">
-        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
+        <x:v>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C45" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
+        <x:v>Elas em Ação / legado / EVT-0081</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Assunção/PRY</x:v>
+        <x:v>Brasília/DF</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>FSports</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
+        <x:v>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</x:v>
       </x:c>
       <x:c r="G45" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29103,7 +29103,7 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I45" s="23" t="str">
-        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
+        <x:v>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -29111,28 +29111,28 @@
         <x:v>46251</x:v>
       </x:c>
       <x:c r="B46" s="23" t="str">
-        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
+        <x:v>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</x:v>
       </x:c>
       <x:c r="C46" s="23" t="str">
-        <x:v>Operação / cidade-sede</x:v>
+        <x:v>Seleções de Base / Sub-15 Feminina</x:v>
       </x:c>
       <x:c r="D46" s="23" t="str">
-        <x:v>Recife/PE</x:v>
+        <x:v>Assunção/PRY</x:v>
       </x:c>
       <x:c r="E46" s="23" t="str">
-        <x:v>Tribuna Online</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F46" s="23" t="str">
-        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</x:v>
       </x:c>
       <x:c r="G46" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H46" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I46" s="23" t="str">
-        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
+        <x:v>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -29140,57 +29140,57 @@
         <x:v>46251</x:v>
       </x:c>
       <x:c r="B47" s="23" t="str">
-        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
+        <x:v>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</x:v>
       </x:c>
       <x:c r="C47" s="23" t="str">
-        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
+        <x:v>Operação / cidade-sede</x:v>
       </x:c>
       <x:c r="D47" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Recife/PE</x:v>
       </x:c>
       <x:c r="E47" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>Tribuna Online</x:v>
       </x:c>
       <x:c r="F47" s="23" t="str">
-        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
+        <x:v>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</x:v>
       </x:c>
       <x:c r="G47" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H47" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I47" s="23" t="str">
-        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
+        <x:v>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="B48" s="23" t="str">
-        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
+        <x:v>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C48" s="23" t="str">
-        <x:v>Calendário / sorteio</x:v>
+        <x:v>Elas Jogam Summit / público / legado / EVT-0021</x:v>
       </x:c>
       <x:c r="D48" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E48" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F48" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
+        <x:v>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</x:v>
       </x:c>
       <x:c r="G48" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H48" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I48" s="23" t="str">
-        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
+        <x:v>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -29198,28 +29198,28 @@
         <x:v>46248</x:v>
       </x:c>
       <x:c r="B49" s="23" t="str">
-        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
+        <x:v>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</x:v>
       </x:c>
       <x:c r="C49" s="23" t="str">
-        <x:v>Patrocínio / ativações</x:v>
+        <x:v>Calendário / sorteio</x:v>
       </x:c>
       <x:c r="D49" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E49" s="23" t="str">
-        <x:v>UOL</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
+        <x:v>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</x:v>
       </x:c>
       <x:c r="G49" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H49" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="I49" s="23" t="str">
-        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
+        <x:v>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -29227,48 +29227,48 @@
         <x:v>46248</x:v>
       </x:c>
       <x:c r="B50" s="23" t="str">
-        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
+        <x:v>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</x:v>
       </x:c>
       <x:c r="C50" s="23" t="str">
-        <x:v>Legado / formação de base / inclusão esportiva</x:v>
+        <x:v>Patrocínio / ativações</x:v>
       </x:c>
       <x:c r="D50" s="23" t="str">
-        <x:v>Diversas cidades/RJ</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E50" s="23" t="str">
-        <x:v>Sesc RJ</x:v>
+        <x:v>UOL</x:v>
       </x:c>
       <x:c r="F50" s="23" t="str">
-        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
+        <x:v>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</x:v>
       </x:c>
       <x:c r="G50" s="23" t="str">
         <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H50" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I50" s="23" t="str">
-        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
+        <x:v>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="32" t="n">
-        <x:v>46247</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="B51" s="23" t="str">
-        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
+        <x:v>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</x:v>
       </x:c>
       <x:c r="C51" s="23" t="str">
-        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
+        <x:v>Legado / formação de base / inclusão esportiva</x:v>
       </x:c>
       <x:c r="D51" s="23" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Diversas cidades/RJ</x:v>
       </x:c>
       <x:c r="E51" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Sesc RJ</x:v>
       </x:c>
       <x:c r="F51" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
+        <x:v>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</x:v>
       </x:c>
       <x:c r="G51" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29277,65 +29277,65 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I51" s="23" t="str">
-        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
+        <x:v>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="32" t="n">
-        <x:v>46246</x:v>
+        <x:v>46247</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
+        <x:v>Base feminina soma 206 atletas convocadas e três desafios internacionais</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>Políticas públicas / educação</x:v>
+        <x:v>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>Folha de S.Paulo</x:v>
+        <x:v>CBF</x:v>
       </x:c>
       <x:c r="F52" s="23" t="str">
-        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</x:v>
       </x:c>
       <x:c r="G52" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H52" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I52" s="23" t="str">
-        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
+        <x:v>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="32" t="n">
-        <x:v>46239</x:v>
+        <x:v>46246</x:v>
       </x:c>
       <x:c r="B53" s="23" t="str">
-        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
+        <x:v>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</x:v>
       </x:c>
       <x:c r="C53" s="23" t="str">
-        <x:v>Calendário / competições nacionais</x:v>
+        <x:v>Políticas públicas / educação</x:v>
       </x:c>
       <x:c r="D53" s="23" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E53" s="23" t="str">
-        <x:v>ge</x:v>
+        <x:v>Folha de S.Paulo</x:v>
       </x:c>
       <x:c r="F53" s="23" t="str">
-        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
+        <x:v>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</x:v>
       </x:c>
       <x:c r="G53" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H53" s="23" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Médio</x:v>
       </x:c>
       <x:c r="I53" s="23" t="str">
-        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
+        <x:v>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -29343,28 +29343,28 @@
         <x:v>46239</x:v>
       </x:c>
       <x:c r="B54" s="23" t="str">
-        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
+        <x:v>CBF determina pausa nacional durante toda a Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C54" s="23" t="str">
-        <x:v>Elas Jogam Summit / legado</x:v>
+        <x:v>Calendário / competições nacionais</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
-        <x:v>São Paulo/SP</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>Donas FC</x:v>
+        <x:v>ge</x:v>
       </x:c>
       <x:c r="F54" s="23" t="str">
-        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
+        <x:v>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</x:v>
       </x:c>
       <x:c r="G54" s="23" t="str">
-        <x:v>Positivo</x:v>
+        <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H54" s="23" t="str">
-        <x:v>Médio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="I54" s="23" t="str">
-        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
+        <x:v>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -29372,19 +29372,19 @@
         <x:v>46239</x:v>
       </x:c>
       <x:c r="B55" s="23" t="str">
-        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
+        <x:v>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C55" s="23" t="str">
-        <x:v>Legado / futebol feminino</x:v>
+        <x:v>Elas Jogam Summit / legado</x:v>
       </x:c>
       <x:c r="D55" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E55" s="23" t="str">
-        <x:v>O Liberal</x:v>
+        <x:v>Donas FC</x:v>
       </x:c>
       <x:c r="F55" s="23" t="str">
-        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
+        <x:v>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</x:v>
       </x:c>
       <x:c r="G55" s="23" t="str">
         <x:v>Positivo</x:v>
@@ -29393,77 +29393,95 @@
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I55" s="23" t="str">
-        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
+        <x:v>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="32" t="n">
-        <x:v>46238</x:v>
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="B56" s="23" t="str">
-        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
+        <x:v>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</x:v>
       </x:c>
       <x:c r="C56" s="23" t="str">
-        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
+        <x:v>Legado / futebol feminino</x:v>
       </x:c>
       <x:c r="D56" s="23" t="str">
         <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E56" s="23" t="str">
-        <x:v>Máquina do Esporte</x:v>
+        <x:v>O Liberal</x:v>
       </x:c>
       <x:c r="F56" s="23" t="str">
-        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
+        <x:v>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</x:v>
       </x:c>
       <x:c r="G56" s="23" t="str">
-        <x:v>Neutro</x:v>
+        <x:v>Positivo</x:v>
       </x:c>
       <x:c r="H56" s="23" t="str">
         <x:v>Médio</x:v>
       </x:c>
       <x:c r="I56" s="23" t="str">
-        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+        <x:v>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="32" t="n">
-        <x:v>46199</x:v>
+        <x:v>46238</x:v>
       </x:c>
       <x:c r="B57" s="23" t="str">
-        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+        <x:v>Especialistas defendem descentralização do legado da Copa Feminina 2027</x:v>
       </x:c>
       <x:c r="C57" s="23" t="str">
-        <x:v>Seleções de Base / calendário 2026</x:v>
+        <x:v>Fórum Sustentabilidade em Campo / legado / EVT-0063</x:v>
       </x:c>
       <x:c r="D57" s="23" t="str">
-        <x:v>Brasil e exterior</x:v>
+        <x:v>São Paulo/SP</x:v>
       </x:c>
       <x:c r="E57" s="23" t="str">
-        <x:v>CBF</x:v>
+        <x:v>Máquina do Esporte</x:v>
       </x:c>
       <x:c r="F57" s="23" t="str">
-        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+        <x:v>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</x:v>
       </x:c>
       <x:c r="G57" s="23" t="str">
         <x:v>Neutro</x:v>
       </x:c>
       <x:c r="H57" s="23" t="str">
+        <x:v>Médio</x:v>
+      </x:c>
+      <x:c r="I57" s="23" t="str">
+        <x:v>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="32" t="n">
+        <x:v>46199</x:v>
+      </x:c>
+      <x:c r="B58" s="23" t="str">
+        <x:v>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</x:v>
+      </x:c>
+      <x:c r="C58" s="23" t="str">
+        <x:v>Seleções de Base / calendário 2026</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="str">
+        <x:v>Brasil e exterior</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="str">
+        <x:v>CBF</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="str">
+        <x:v>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</x:v>
+      </x:c>
+      <x:c r="G58" s="23" t="str">
+        <x:v>Neutro</x:v>
+      </x:c>
+      <x:c r="H58" s="23" t="str">
         <x:v>Alto</x:v>
       </x:c>
-      <x:c r="I57" s="23" t="str">
+      <x:c r="I58" s="23" t="str">
         <x:v>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="6"/>
-      <x:c r="B58" s="23"/>
-      <x:c r="C58" s="23"/>
-      <x:c r="D58" s="23"/>
-      <x:c r="E58" s="23"/>
-      <x:c r="F58" s="23"/>
-      <x:c r="G58" s="23"/>
-      <x:c r="H58" s="23"/>
-      <x:c r="I58" s="23"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="6"/>
@@ -34338,7 +34356,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe989ea0c5434ed5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123ce2cf58094a21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35241,7 +35259,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8c78b12350426a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra539009094e8417e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36120,7 +36138,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef7a1f164264e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb946b802444547"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36543,7 +36561,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb85a636b46be499a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53f814b5ca254e7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Incorpora pesquisa editorial ao Radar e sincroniza planilha
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -1351,7 +1351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:I58"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Data"/>
@@ -30016,31 +30016,31 @@
     </row>
     <row r="2" ht="150.75" customHeight="1" s="1">
       <c r="A2" s="31" t="n">
-        <v>46254</v>
+        <v>46273</v>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
+          <t>Lorena é indicada ao prêmio de melhor goleira da Bola de Ouro 2026</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
+          <t>Seleção Brasileira / Lorena / Bola de Ouro 2026 / ciclo da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Prefeitura de São Paulo</t>
+          <t>CNN Brasil</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
+          <t>https://www.cnnbrasil.com.br/esportes/futebol/futebol-internacional/bola-de-ouro-lorena-e-indicada-a-melhor-goleira-do-futebol-feminino/</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -30050,42 +30050,42 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
+          <t>Lorena, goleira titular da Seleção Brasileira principal e atleta do Kansas City, foi indicada em 08/09/2026 ao prêmio de melhor goleira do futebol feminino da Bola de Ouro 2026. O reconhecimento internacional integra o acompanhamento das principais atletas brasileiras no ciclo de preparação para a Copa do Mundo Feminina FIFA 2027 no Brasil.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" s="1">
       <c r="A3" s="31" t="n">
-        <v>46268</v>
+        <v>46254</v>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
+          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
+          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
+          <t>Prefeitura de São Paulo</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
+          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -30095,42 +30095,42 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
+          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="99.75" customHeight="1" s="1">
       <c r="A4" s="31" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
+          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
+          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -30140,42 +30140,42 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
+          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="128.25" customHeight="1" s="1">
       <c r="A5" s="31" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
+          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
+          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>BRA1 / Agência VIVA</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
+          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -30185,42 +30185,42 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
+          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="32" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
+          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
+          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>BRA1 / Agência VIVA</t>
         </is>
       </c>
       <c r="F6" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
+          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -30230,42 +30230,42 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
+          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="32" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
+          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
+          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>Jornal de Piracicaba / Sampi</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
+          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -30275,42 +30275,42 @@
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
+          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="32" t="n">
-        <v>46251</v>
+        <v>46269</v>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
+          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
+          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Piracicaba/SP</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Diário Oficial do Distrito Federal</t>
+          <t>Jornal de Piracicaba / Sampi</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
+          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
@@ -30325,42 +30325,42 @@
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
+          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="32" t="n">
-        <v>46267</v>
+        <v>46251</v>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
+          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado / Câmara dos Deputados</t>
+          <t>Diário Oficial do Distrito Federal</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
+          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H9" s="23" t="inlineStr">
@@ -30370,87 +30370,87 @@
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
+          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="32" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
+          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
+          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Agência Senado / Câmara dos Deputados</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
+          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
+          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="32" t="n">
-        <v>46265</v>
+        <v>46268</v>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
+          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
+          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
@@ -30460,52 +30460,52 @@
       </c>
       <c r="I11" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
+          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="32" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
+          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
+          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Jornal Grande Bahia / GovBA</t>
+          <t>Prefeitura de Porto Alegre</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H12" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I12" s="23" t="inlineStr">
         <is>
-          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
+          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
         </is>
       </c>
     </row>
@@ -30515,27 +30515,27 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
+          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
+          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>AFP/BOL</t>
+          <t>Jornal Grande Bahia / GovBA</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
+          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
@@ -30550,37 +30550,37 @@
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
+          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="32" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
+          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Mercado / crescimento / futebol feminino</t>
+          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>AFP/BOL</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
+          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -30590,12 +30590,12 @@
       </c>
       <c r="H14" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I14" s="23" t="inlineStr">
         <is>
-          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
+          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
         </is>
       </c>
     </row>
@@ -30605,27 +30605,27 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
+          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
+          <t>Mercado / crescimento / futebol feminino</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>Let's Go Bahia</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
+          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -30635,12 +30635,12 @@
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
+          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
         </is>
       </c>
     </row>
@@ -30650,27 +30650,27 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
+          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento local / cidade-sede</t>
+          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>Let's Go Bahia</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
+          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
@@ -30685,7 +30685,7 @@
       </c>
       <c r="I16" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
+          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
         </is>
       </c>
     </row>
@@ -30695,27 +30695,27 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
+          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento / operação do torneio</t>
+          <t>Voluntariado / engajamento local / cidade-sede</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
+          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -30725,27 +30725,27 @@
       </c>
       <c r="H17" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I17" s="23" t="inlineStr">
         <is>
-          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
+          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="32" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
+          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
+          <t>Voluntariado / engajamento / operação do torneio</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
@@ -30755,12 +30755,12 @@
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
+          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -30775,7 +30775,7 @@
       </c>
       <c r="I18" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
+          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
         </is>
       </c>
     </row>
@@ -30785,12 +30785,12 @@
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
+          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Mídia / futebol feminino / cobertura esportiva</t>
+          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
@@ -30800,12 +30800,12 @@
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>O Globo</t>
+          <t>Agência Senado</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
+          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -30815,12 +30815,12 @@
       </c>
       <c r="H19" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I19" s="23" t="inlineStr">
         <is>
-          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
+          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
         </is>
       </c>
     </row>
@@ -30830,12 +30830,12 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
+          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / operação do torneio / engajamento</t>
+          <t>Mídia / futebol feminino / cobertura esportiva</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
@@ -30845,12 +30845,12 @@
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>O Globo</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
+          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -30860,27 +30860,27 @@
       </c>
       <c r="H20" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I20" s="23" t="inlineStr">
         <is>
-          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
+          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="32" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
+          <t>Voluntariado / operação do torneio / engajamento</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
@@ -30890,17 +30890,17 @@
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>Agência Câmara</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
@@ -30910,52 +30910,52 @@
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
+          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="32" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
+          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Agência Câmara</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
+          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
+          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
         </is>
       </c>
     </row>
@@ -30965,17 +30965,17 @@
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
+          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Polônia</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
@@ -30985,7 +30985,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -31000,22 +31000,22 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="32" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
+          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
@@ -31030,7 +31030,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
@@ -31045,37 +31045,37 @@
       </c>
       <c r="I24" s="23" t="inlineStr">
         <is>
-          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
+          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="32" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
+          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Polônia</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Diário do Nordeste</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
@@ -31085,12 +31085,12 @@
       </c>
       <c r="H25" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I25" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
+          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
         </is>
       </c>
     </row>
@@ -31100,27 +31100,27 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
+          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
+          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Diário do Nordeste</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
+          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
@@ -31130,12 +31130,12 @@
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
         <is>
-          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
         </is>
       </c>
     </row>
@@ -31145,27 +31145,27 @@
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
+          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
+          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Empetur</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -31180,7 +31180,7 @@
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
+          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
         </is>
       </c>
     </row>
@@ -31190,27 +31190,27 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
+          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Tributação / legislação federal / organização</t>
+          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Presidência da República</t>
+          <t>Empetur</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
+          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -31220,12 +31220,12 @@
       </c>
       <c r="H28" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
+          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
         </is>
       </c>
     </row>
@@ -31235,27 +31235,27 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
+          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
+          <t>Tributação / legislação federal / organização</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>Presidência da República</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
+          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -31265,12 +31265,12 @@
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
+          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
         </is>
       </c>
     </row>
@@ -31280,77 +31280,77 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
+          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / infraestrutura / cidade-sede</t>
+          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Diário de Pernambuco</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
         <is>
-          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
+          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
         </is>
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="32" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
+          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
+          <t>Repescagem / infraestrutura / cidade-sede</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>Diário de Pernambuco</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
+          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H31" s="23" t="inlineStr">
@@ -31360,7 +31360,7 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
+          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
         </is>
       </c>
     </row>
@@ -31370,27 +31370,27 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
+          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
+          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
+          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
@@ -31400,12 +31400,12 @@
       </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I32" s="23" t="inlineStr">
         <is>
-          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
+          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
         </is>
       </c>
     </row>
@@ -31415,27 +31415,27 @@
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
+          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
+          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
@@ -31450,7 +31450,7 @@
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
+          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
         </is>
       </c>
     </row>
@@ -31460,27 +31460,27 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
+          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Alerj</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -31490,12 +31490,12 @@
       </c>
       <c r="H34" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I34" s="23" t="inlineStr">
         <is>
-          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
+          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
         </is>
       </c>
     </row>
@@ -31505,27 +31505,27 @@
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
+          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Alerj</t>
         </is>
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
+          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -31535,42 +31535,42 @@
       </c>
       <c r="H35" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I35" s="23" t="inlineStr">
         <is>
-          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
+          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="32" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
+          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Tour da Taça / ativações / EVT-0090</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D36" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
@@ -31580,12 +31580,12 @@
       </c>
       <c r="H36" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I36" s="23" t="inlineStr">
         <is>
-          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
+          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
         </is>
       </c>
     </row>
@@ -31595,27 +31595,27 @@
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
+          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
+          <t>Tour da Taça / ativações / EVT-0090</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Federação Gaúcha de Futebol</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
+          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
@@ -31625,12 +31625,12 @@
       </c>
       <c r="H37" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
+          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -31640,27 +31640,27 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
+          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / preparação das cidades-sede / Recife</t>
+          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
-          <t>Folha de Pernambuco</t>
+          <t>Federação Gaúcha de Futebol</t>
         </is>
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
+          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -31675,7 +31675,7 @@
       </c>
       <c r="I38" s="23" t="inlineStr">
         <is>
-          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
+          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -31685,27 +31685,27 @@
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
+          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Voluntariado / preparação das cidades-sede / Recife</t>
         </is>
       </c>
       <c r="D39" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E39" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Folha de Pernambuco</t>
         </is>
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
+          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
         </is>
       </c>
       <c r="G39" s="23" t="inlineStr">
@@ -31720,7 +31720,7 @@
       </c>
       <c r="I39" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
+          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
         </is>
       </c>
     </row>
@@ -31730,12 +31730,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
+          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D40" s="23" t="inlineStr">
@@ -31750,7 +31750,7 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -31765,7 +31765,7 @@
       </c>
       <c r="I40" s="23" t="inlineStr">
         <is>
-          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
         </is>
       </c>
     </row>
@@ -31775,27 +31775,27 @@
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
+          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
         </is>
       </c>
       <c r="D41" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
         </is>
       </c>
       <c r="G41" s="23" t="inlineStr">
@@ -31810,7 +31810,7 @@
       </c>
       <c r="I41" s="23" t="inlineStr">
         <is>
-          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
+          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
         </is>
       </c>
     </row>
@@ -31820,87 +31820,87 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
+          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
+          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D42" s="23" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo / AFP</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
+          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H42" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I42" s="23" t="inlineStr">
         <is>
-          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
+          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="32" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
+          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>Cultura / turismo / alimentação / Salvador</t>
+          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
         </is>
       </c>
       <c r="D43" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E43" s="23" t="inlineStr">
         <is>
-          <t>A TARDE</t>
+          <t>Folha de S.Paulo / AFP</t>
         </is>
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H43" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I43" s="23" t="inlineStr">
         <is>
-          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
+          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
         </is>
       </c>
     </row>
@@ -31910,42 +31910,42 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
+          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / governança / premiação / EVT-0010</t>
+          <t>Cultura / turismo / alimentação / Salvador</t>
         </is>
       </c>
       <c r="D44" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>A TARDE</t>
         </is>
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
+          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H44" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I44" s="23" t="inlineStr">
         <is>
-          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
+          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
         </is>
       </c>
     </row>
@@ -31955,27 +31955,27 @@
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
+          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Calendário continental / clubes / organização</t>
+          <t>Sorteio / governança / premiação / EVT-0010</t>
         </is>
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>América do Sul / Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Máquina do Esporte</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
@@ -31990,7 +31990,7 @@
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
+          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
         </is>
       </c>
     </row>
@@ -32000,32 +32000,32 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
+          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>Negócios / audiência / patrocínios</t>
+          <t>Calendário continental / clubes / organização</t>
         </is>
       </c>
       <c r="D46" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>América do Sul / Brasil</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>MKT Esportivo</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
+          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -32035,7 +32035,7 @@
       </c>
       <c r="I46" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
+          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
         </is>
       </c>
     </row>
@@ -32045,87 +32045,87 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
+          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação / Porto Alegre</t>
+          <t>Negócios / audiência / patrocínios</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>GZH</t>
+          <t>MKT Esportivo</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
+          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
-          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
+          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="32" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
+          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>Calendário / estádios / EVT-0077</t>
+          <t>Seleção Brasileira / preparação / Porto Alegre</t>
         </is>
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>GZH</t>
         </is>
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
+          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H48" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I48" s="23" t="inlineStr">
         <is>
-          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
+          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
         </is>
       </c>
     </row>
@@ -32135,27 +32135,27 @@
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
+          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
+          <t>Calendário / estádios / EVT-0077</t>
         </is>
       </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
@@ -32165,12 +32165,12 @@
       </c>
       <c r="H49" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I49" s="23" t="inlineStr">
         <is>
-          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
+          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
         </is>
       </c>
     </row>
@@ -32180,27 +32180,27 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
+          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado / EVT-0021</t>
+          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
         </is>
       </c>
       <c r="D50" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>TV Brasil</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
+          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -32215,7 +32215,7 @@
       </c>
       <c r="I50" s="23" t="inlineStr">
         <is>
-          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
+          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
         </is>
       </c>
     </row>
@@ -32225,27 +32225,27 @@
       </c>
       <c r="B51" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
+          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>Turismo / hotelaria / economia local</t>
+          <t>Elas Jogam Summit / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D51" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>TurisNews</t>
+          <t>TV Brasil</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
+          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
@@ -32260,7 +32260,7 @@
       </c>
       <c r="I51" s="23" t="inlineStr">
         <is>
-          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
+          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
         </is>
       </c>
     </row>
@@ -32270,12 +32270,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
+          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>Sustentabilidade / Fortaleza</t>
+          <t>Turismo / hotelaria / economia local</t>
         </is>
       </c>
       <c r="D52" s="23" t="inlineStr">
@@ -32285,12 +32285,12 @@
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>Agência Sebrae de Notícias</t>
+          <t>TurisNews</t>
         </is>
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
+          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
@@ -32305,7 +32305,7 @@
       </c>
       <c r="I52" s="23" t="inlineStr">
         <is>
-          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
+          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
         </is>
       </c>
     </row>
@@ -32315,27 +32315,27 @@
       </c>
       <c r="B53" s="23" t="inlineStr">
         <is>
-          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
+          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
         </is>
       </c>
       <c r="C53" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / calendário / EVT-0010</t>
+          <t>Sustentabilidade / Fortaleza</t>
         </is>
       </c>
       <c r="D53" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E53" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Agência Sebrae de Notícias</t>
         </is>
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
+          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
@@ -32345,42 +32345,42 @@
       </c>
       <c r="H53" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I53" s="23" t="inlineStr">
         <is>
-          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
+          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="32" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
+          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / negócios</t>
+          <t>Sorteio / calendário / EVT-0010</t>
         </is>
       </c>
       <c r="D54" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E54" s="23" t="inlineStr">
         <is>
-          <t>Exame</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
         </is>
       </c>
       <c r="G54" s="23" t="inlineStr">
@@ -32395,7 +32395,7 @@
       </c>
       <c r="I54" s="23" t="inlineStr">
         <is>
-          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
+          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
         </is>
       </c>
     </row>
@@ -32405,27 +32405,27 @@
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
+          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>Tributação / organização / políticas públicas</t>
+          <t>Patrocínio / negócios</t>
         </is>
       </c>
       <c r="D55" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E55" s="23" t="inlineStr">
         <is>
-          <t>Governo do Estado do Rio de Janeiro</t>
+          <t>Exame</t>
         </is>
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
+          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
@@ -32440,37 +32440,37 @@
       </c>
       <c r="I55" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
+          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="32" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
+          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
+          <t>Tributação / organização / políticas públicas</t>
         </is>
       </c>
       <c r="D56" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>Correio</t>
+          <t>Governo do Estado do Rio de Janeiro</t>
         </is>
       </c>
       <c r="F56" s="23" t="inlineStr">
         <is>
-          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
+          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
         </is>
       </c>
       <c r="G56" s="23" t="inlineStr">
@@ -32480,42 +32480,42 @@
       </c>
       <c r="H56" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I56" s="23" t="inlineStr">
         <is>
-          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
+          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="32" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="B57" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
+          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
         </is>
       </c>
       <c r="C57" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
         </is>
       </c>
       <c r="D57" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E57" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>Correio</t>
         </is>
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
+          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
@@ -32530,37 +32530,37 @@
       </c>
       <c r="I57" s="23" t="inlineStr">
         <is>
-          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
+          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="32" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
+          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
         </is>
       </c>
       <c r="C58" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D58" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F58" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
+          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
         </is>
       </c>
       <c r="G58" s="23" t="inlineStr">
@@ -32575,7 +32575,7 @@
       </c>
       <c r="I58" s="23" t="inlineStr">
         <is>
-          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
+          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
         </is>
       </c>
     </row>
@@ -32585,12 +32585,12 @@
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
+          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / relacionamento</t>
+          <t>Seleção Brasileira / preparação</t>
         </is>
       </c>
       <c r="D59" s="23" t="inlineStr">
@@ -32600,17 +32600,17 @@
       </c>
       <c r="E59" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
@@ -32620,7 +32620,7 @@
       </c>
       <c r="I59" s="23" t="inlineStr">
         <is>
-          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
+          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
         </is>
       </c>
     </row>
@@ -32630,12 +32630,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
+          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sedes</t>
+          <t>Ingressos / relacionamento</t>
         </is>
       </c>
       <c r="D60" s="23" t="inlineStr">
@@ -32645,27 +32645,27 @@
       </c>
       <c r="E60" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F60" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
         </is>
       </c>
       <c r="G60" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H60" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I60" s="23" t="inlineStr">
         <is>
-          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
+          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
         </is>
       </c>
     </row>
@@ -32675,12 +32675,12 @@
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
+          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
         <is>
-          <t>Investimentos públicos / segurança / infraestrutura</t>
+          <t>Calendário / sedes</t>
         </is>
       </c>
       <c r="D61" s="23" t="inlineStr">
@@ -32690,17 +32690,17 @@
       </c>
       <c r="E61" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F61" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
+          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
         </is>
       </c>
       <c r="G61" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H61" s="23" t="inlineStr">
@@ -32710,7 +32710,7 @@
       </c>
       <c r="I61" s="23" t="inlineStr">
         <is>
-          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
+          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
         </is>
       </c>
     </row>
@@ -32720,12 +32720,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
+          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / sorteio</t>
+          <t>Investimentos públicos / segurança / infraestrutura</t>
         </is>
       </c>
       <c r="D62" s="23" t="inlineStr">
@@ -32735,12 +32735,12 @@
       </c>
       <c r="E62" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F62" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
         </is>
       </c>
       <c r="G62" s="23" t="inlineStr">
@@ -32755,27 +32755,27 @@
       </c>
       <c r="I62" s="23" t="inlineStr">
         <is>
-          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
+          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="33" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
+          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Repescagem / sorteio</t>
         </is>
       </c>
       <c r="D63" s="23" t="inlineStr">
         <is>
-          <t>Brasil / Polônia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E63" s="23" t="inlineStr">
@@ -32785,22 +32785,22 @@
       </c>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
         </is>
       </c>
       <c r="G63" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H63" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I63" s="23" t="inlineStr">
         <is>
-          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
+          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
         </is>
       </c>
     </row>
@@ -32810,42 +32810,42 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
+          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D64" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasil / Polônia</t>
         </is>
       </c>
       <c r="E64" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F64" s="23" t="inlineStr">
         <is>
-          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
+          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
         </is>
       </c>
       <c r="G64" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H64" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I64" s="23" t="inlineStr">
         <is>
-          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
+          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
         </is>
       </c>
     </row>
@@ -32855,12 +32855,12 @@
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
+          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
         <is>
-          <t>Varejo / consumo / oportunidades comerciais</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D65" s="23" t="inlineStr">
@@ -32870,57 +32870,57 @@
       </c>
       <c r="E65" s="23" t="inlineStr">
         <is>
-          <t>Revista Super Negócios / ASSERJ</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F65" s="23" t="inlineStr">
         <is>
-          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
+          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
         </is>
       </c>
       <c r="G65" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H65" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I65" s="23" t="inlineStr">
         <is>
-          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
+          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="33" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
+          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
         <is>
-          <t>Elas em Ação / legado / EVT-0081</t>
+          <t>Varejo / consumo / oportunidades comerciais</t>
         </is>
       </c>
       <c r="D66" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E66" s="23" t="inlineStr">
         <is>
-          <t>FSports</t>
+          <t>Revista Super Negócios / ASSERJ</t>
         </is>
       </c>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
+          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
         </is>
       </c>
       <c r="G66" s="23" t="inlineStr">
@@ -32935,37 +32935,37 @@
       </c>
       <c r="I66" s="23" t="inlineStr">
         <is>
-          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
+          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="33" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
+          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15 Feminina</t>
+          <t>Elas em Ação / legado / EVT-0081</t>
         </is>
       </c>
       <c r="D67" s="23" t="inlineStr">
         <is>
-          <t>Assunção/PRY</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E67" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>FSports</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
+          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
         </is>
       </c>
       <c r="G67" s="23" t="inlineStr">
@@ -32980,7 +32980,7 @@
       </c>
       <c r="I67" s="23" t="inlineStr">
         <is>
-          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
+          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
         </is>
       </c>
     </row>
@@ -32990,27 +32990,27 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>FIFA e FPF alinham prepa